<commit_message>
Now the units is handled much better in log_curve_new.py. Units are converted automatically based on the style/template
</commit_message>
<xml_diff>
--- a/excels/project_table_new.xlsx
+++ b/excels/project_table_new.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\emb\Documents\PycharmProjects\blixt_rp\excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33F4F91E-B701-4092-B456-8345C338237D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B4B8311-7757-458A-A8CF-DD0D20B6BF02}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30624" yWindow="0" windowWidth="30912" windowHeight="16656" tabRatio="685" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1200" yWindow="4380" windowWidth="28800" windowHeight="16335" tabRatio="685" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Well settings" sheetId="1" r:id="rId1"/>
@@ -62,7 +62,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="919" uniqueCount="389">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="919" uniqueCount="391">
   <si>
     <t>Select Yes or No</t>
   </si>
@@ -1238,6 +1238,12 @@
   </si>
   <si>
     <t>Well F copies the well path and checkshots from well A</t>
+  </si>
+  <si>
+    <t>fract</t>
+  </si>
+  <si>
+    <t>dimensionless</t>
   </si>
 </sst>
 </file>
@@ -1936,13 +1942,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:I13"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="5.6640625" customWidth="1"/>
-    <col min="2" max="2" width="12.44140625" customWidth="1"/>
+    <col min="1" max="1" width="5.7109375" customWidth="1"/>
+    <col min="2" max="2" width="12.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1953,7 +1959,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:9" s="1" customFormat="1" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:9" s="1" customFormat="1" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
@@ -1982,7 +1988,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>21</v>
       </c>
@@ -2002,7 +2008,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>21</v>
       </c>
@@ -2016,7 +2022,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>21</v>
       </c>
@@ -2030,7 +2036,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>21</v>
       </c>
@@ -2044,7 +2050,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>21</v>
       </c>
@@ -2058,7 +2064,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>11</v>
       </c>
@@ -2078,7 +2084,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>21</v>
       </c>
@@ -2095,7 +2101,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B10" s="13"/>
       <c r="C10" s="20" t="s">
         <v>23</v>
@@ -2104,7 +2110,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="C11" s="21" t="s">
         <v>35</v>
       </c>
@@ -2112,7 +2118,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="C12" s="22" t="s">
         <v>37</v>
       </c>
@@ -2120,7 +2126,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="C13" s="23" t="s">
         <v>39</v>
       </c>
@@ -2144,19 +2150,19 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
   <dimension ref="A1:D4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="2" width="10.33203125" customWidth="1"/>
-    <col min="3" max="3" width="17.44140625" customWidth="1"/>
+    <col min="1" max="2" width="10.28515625" customWidth="1"/>
+    <col min="3" max="3" width="17.42578125" customWidth="1"/>
     <col min="4" max="4" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="26.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D1" s="5" t="s">
         <v>324</v>
       </c>
     </row>
-    <row r="2" spans="1:4" s="8" customFormat="1" ht="30.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:4" s="8" customFormat="1" ht="30.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="9" t="s">
         <v>279</v>
       </c>
@@ -2170,7 +2176,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>28</v>
       </c>
@@ -2184,7 +2190,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>28</v>
       </c>
@@ -2229,9 +2235,9 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CCD9C215-DCD2-40A2-A7D5-172DC530BE0E}">
   <dimension ref="A1:Q2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
       <c r="D1" s="2"/>
@@ -2252,7 +2258,7 @@
       </c>
       <c r="O1" s="2"/>
     </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>374</v>
       </c>
@@ -2305,9 +2311,9 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3CCC2506-3BD3-4476-A9AA-1673C259914E}">
   <dimension ref="A1:M2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" s="2"/>
       <c r="B1" s="2" t="s">
         <v>379</v>
@@ -2320,7 +2326,7 @@
       <c r="I1" s="2"/>
       <c r="K1" s="2"/>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>375</v>
       </c>
@@ -2366,19 +2372,19 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
   <dimension ref="A1:Q18"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="16.33203125" customWidth="1"/>
-    <col min="3" max="3" width="12.33203125" customWidth="1"/>
-    <col min="4" max="4" width="9.88671875" customWidth="1"/>
+    <col min="2" max="2" width="16.28515625" customWidth="1"/>
+    <col min="3" max="3" width="12.28515625" customWidth="1"/>
+    <col min="4" max="4" width="9.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="H1" s="2" t="s">
         <v>362</v>
       </c>
     </row>
-    <row r="2" spans="1:17" s="6" customFormat="1" ht="42.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:17" s="6" customFormat="1" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2" s="6" t="s">
         <v>326</v>
       </c>
@@ -2428,7 +2434,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>11</v>
       </c>
@@ -2482,7 +2488,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>21</v>
       </c>
@@ -2533,7 +2539,7 @@
         <v>355</v>
       </c>
     </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
       <c r="E5" t="s">
         <v>340</v>
       </c>
@@ -2560,7 +2566,7 @@
         <v>357</v>
       </c>
     </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
       <c r="F6" t="s">
         <v>27</v>
       </c>
@@ -2581,7 +2587,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
       <c r="F7" t="s">
         <v>30</v>
       </c>
@@ -2599,7 +2605,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
       <c r="F8" t="s">
         <v>33</v>
       </c>
@@ -2611,7 +2617,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
       <c r="F9" t="s">
         <v>24</v>
       </c>
@@ -2623,7 +2629,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="10" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:17" x14ac:dyDescent="0.25">
       <c r="F10" t="s">
         <v>36</v>
       </c>
@@ -2635,7 +2641,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:17" x14ac:dyDescent="0.25">
       <c r="F11" t="s">
         <v>38</v>
       </c>
@@ -2647,7 +2653,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:17" x14ac:dyDescent="0.25">
       <c r="F12" t="s">
         <v>40</v>
       </c>
@@ -2659,7 +2665,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:17" x14ac:dyDescent="0.25">
       <c r="F13" t="s">
         <v>343</v>
       </c>
@@ -2671,7 +2677,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:17" x14ac:dyDescent="0.25">
       <c r="F14" t="s">
         <v>344</v>
       </c>
@@ -2683,7 +2689,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:17" x14ac:dyDescent="0.25">
       <c r="F15" t="s">
         <v>121</v>
       </c>
@@ -2695,7 +2701,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:17" x14ac:dyDescent="0.25">
       <c r="F16" t="s">
         <v>345</v>
       </c>
@@ -2707,7 +2713,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="8:9" x14ac:dyDescent="0.3">
+    <row r="17" spans="8:9" x14ac:dyDescent="0.25">
       <c r="H17" s="30" t="s">
         <v>173</v>
       </c>
@@ -2716,7 +2722,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="8:9" x14ac:dyDescent="0.3">
+    <row r="18" spans="8:9" x14ac:dyDescent="0.25">
       <c r="H18" s="30" t="s">
         <v>174</v>
       </c>
@@ -2734,19 +2740,19 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:R11"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="2" width="9.6640625" style="13" customWidth="1"/>
-    <col min="3" max="3" width="15.88671875" customWidth="1"/>
-    <col min="4" max="5" width="11.5546875" customWidth="1"/>
+    <col min="1" max="2" width="9.7109375" style="13" customWidth="1"/>
+    <col min="3" max="3" width="15.85546875" customWidth="1"/>
+    <col min="4" max="5" width="11.5703125" customWidth="1"/>
     <col min="6" max="7" width="10" customWidth="1"/>
-    <col min="11" max="11" width="16.109375" customWidth="1"/>
+    <col min="11" max="11" width="16.140625" customWidth="1"/>
     <col min="13" max="13" width="7" customWidth="1"/>
-    <col min="16" max="16" width="6.5546875" customWidth="1"/>
-    <col min="17" max="17" width="4.6640625" customWidth="1"/>
+    <col min="16" max="16" width="6.5703125" customWidth="1"/>
+    <col min="17" max="17" width="4.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A1" s="11" t="s">
         <v>41</v>
       </c>
@@ -2754,7 +2760,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="2" spans="1:18" s="1" customFormat="1" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:18" s="1" customFormat="1" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="12" t="s">
         <v>3</v>
       </c>
@@ -2810,7 +2816,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A3" s="13" t="s">
         <v>12</v>
       </c>
@@ -2839,7 +2845,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A4" s="13" t="s">
         <v>12</v>
       </c>
@@ -2856,7 +2862,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A5" s="13" t="s">
         <v>15</v>
       </c>
@@ -2882,7 +2888,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A6" s="13" t="s">
         <v>18</v>
       </c>
@@ -2908,7 +2914,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A7" s="13" t="s">
         <v>22</v>
       </c>
@@ -2937,7 +2943,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A8" s="13" t="s">
         <v>25</v>
       </c>
@@ -2954,7 +2960,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A9" s="13" t="s">
         <v>25</v>
       </c>
@@ -2977,7 +2983,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A10" s="13" t="s">
         <v>28</v>
       </c>
@@ -3009,7 +3015,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A11" s="13" t="s">
         <v>31</v>
       </c>
@@ -3066,13 +3072,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{725EDE5F-2F74-4F10-B375-EE1EEF8AD52D}">
   <dimension ref="A1:M20"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="3" max="3" width="15.33203125" customWidth="1"/>
-    <col min="4" max="4" width="14.5546875" customWidth="1"/>
+    <col min="3" max="3" width="15.28515625" customWidth="1"/>
+    <col min="4" max="4" width="14.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" s="11" t="s">
         <v>41</v>
       </c>
@@ -3086,7 +3092,7 @@
         <v>382</v>
       </c>
     </row>
-    <row r="2" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="12" t="s">
         <v>3</v>
       </c>
@@ -3123,7 +3129,7 @@
       <c r="L2" s="1"/>
       <c r="M2" s="1"/>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" s="13" t="s">
         <v>12</v>
       </c>
@@ -3149,7 +3155,7 @@
         <v>385</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" s="13" t="s">
         <v>12</v>
       </c>
@@ -3172,11 +3178,11 @@
         <v>387</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" s="13"/>
       <c r="C5" s="4"/>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" s="13" t="s">
         <v>15</v>
       </c>
@@ -3202,7 +3208,7 @@
         <v>385</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" s="13" t="s">
         <v>15</v>
       </c>
@@ -3225,11 +3231,11 @@
         <v>387</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" s="13"/>
       <c r="C8" s="4"/>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" s="13" t="s">
         <v>18</v>
       </c>
@@ -3255,7 +3261,7 @@
         <v>385</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" s="13" t="s">
         <v>18</v>
       </c>
@@ -3278,11 +3284,11 @@
         <v>387</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" s="13"/>
       <c r="C11" s="4"/>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A12" s="13" t="s">
         <v>22</v>
       </c>
@@ -3291,11 +3297,11 @@
       </c>
       <c r="C12" s="4"/>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A13" s="13"/>
       <c r="C13" s="4"/>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A14" s="13" t="s">
         <v>25</v>
       </c>
@@ -3304,7 +3310,7 @@
       </c>
       <c r="C14" s="4"/>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A15" s="13" t="s">
         <v>25</v>
       </c>
@@ -3313,11 +3319,11 @@
       </c>
       <c r="C15" s="4"/>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A16" s="13"/>
       <c r="C16" s="4"/>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" s="13" t="s">
         <v>28</v>
       </c>
@@ -3346,7 +3352,7 @@
         <v>388</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" s="13" t="s">
         <v>28</v>
       </c>
@@ -3369,11 +3375,11 @@
         <v>387</v>
       </c>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" s="13"/>
       <c r="C19" s="4"/>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" s="13" t="s">
         <v>31</v>
       </c>
@@ -3411,19 +3417,19 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:O31"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.44140625" customWidth="1"/>
-    <col min="2" max="2" width="14.109375" customWidth="1"/>
-    <col min="3" max="3" width="14.5546875" customWidth="1"/>
+    <col min="1" max="1" width="11.42578125" customWidth="1"/>
+    <col min="2" max="2" width="14.140625" customWidth="1"/>
+    <col min="3" max="3" width="14.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>175</v>
       </c>
     </row>
-    <row r="2" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>176</v>
       </c>
@@ -3470,7 +3476,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>190</v>
       </c>
@@ -3505,7 +3511,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
         <v>45</v>
       </c>
@@ -3537,7 +3543,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
         <v>47</v>
       </c>
@@ -3569,7 +3575,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>198</v>
       </c>
@@ -3604,7 +3610,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>201</v>
       </c>
@@ -3612,7 +3618,7 @@
         <v>202</v>
       </c>
       <c r="C7" t="s">
-        <v>195</v>
+        <v>389</v>
       </c>
       <c r="D7" t="s">
         <v>197</v>
@@ -3639,7 +3645,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>203</v>
       </c>
@@ -3674,7 +3680,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
         <v>207</v>
       </c>
@@ -3699,7 +3705,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
         <v>209</v>
       </c>
@@ -3724,7 +3730,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>210</v>
       </c>
@@ -3732,7 +3738,7 @@
         <v>52</v>
       </c>
       <c r="C11" t="s">
-        <v>195</v>
+        <v>389</v>
       </c>
       <c r="D11" t="s">
         <v>197</v>
@@ -3759,7 +3765,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>211</v>
       </c>
@@ -3767,7 +3773,7 @@
         <v>53</v>
       </c>
       <c r="C12" t="s">
-        <v>195</v>
+        <v>389</v>
       </c>
       <c r="D12" t="s">
         <v>197</v>
@@ -3794,7 +3800,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>214</v>
       </c>
@@ -3802,7 +3808,7 @@
         <v>54</v>
       </c>
       <c r="C13" t="s">
-        <v>195</v>
+        <v>389</v>
       </c>
       <c r="D13" t="s">
         <v>197</v>
@@ -3829,7 +3835,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>77</v>
       </c>
@@ -3864,7 +3870,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>216</v>
       </c>
@@ -3899,7 +3905,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>219</v>
       </c>
@@ -3934,7 +3940,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>222</v>
       </c>
@@ -3969,7 +3975,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>225</v>
       </c>
@@ -4004,7 +4010,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>227</v>
       </c>
@@ -4039,7 +4045,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>229</v>
       </c>
@@ -4074,7 +4080,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>231</v>
       </c>
@@ -4112,7 +4118,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>236</v>
       </c>
@@ -4120,7 +4126,7 @@
         <v>237</v>
       </c>
       <c r="C22" t="s">
-        <v>195</v>
+        <v>389</v>
       </c>
       <c r="D22" t="s">
         <v>197</v>
@@ -4141,7 +4147,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>238</v>
       </c>
@@ -4149,7 +4155,7 @@
         <v>239</v>
       </c>
       <c r="C23" t="s">
-        <v>195</v>
+        <v>389</v>
       </c>
       <c r="D23" t="s">
         <v>233</v>
@@ -4176,7 +4182,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>242</v>
       </c>
@@ -4207,7 +4213,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>245</v>
       </c>
@@ -4242,7 +4248,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B26" t="s">
         <v>57</v>
       </c>
@@ -4262,7 +4268,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B27" t="s">
         <v>381</v>
       </c>
@@ -4288,7 +4294,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B28" t="s">
         <v>247</v>
       </c>
@@ -4314,7 +4320,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>248</v>
       </c>
@@ -4343,7 +4349,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>250</v>
       </c>
@@ -4372,12 +4378,12 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B31" t="s">
         <v>252</v>
       </c>
       <c r="C31" t="s">
-        <v>195</v>
+        <v>390</v>
       </c>
       <c r="D31" t="s">
         <v>197</v>
@@ -4412,13 +4418,13 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:M17"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
-    <col min="6" max="6" width="15.5546875" customWidth="1"/>
+    <col min="6" max="6" width="15.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" s="2"/>
       <c r="B1" s="2" t="s">
         <v>112</v>
@@ -4435,7 +4441,7 @@
       <c r="I1" s="2"/>
       <c r="K1" s="2"/>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>115</v>
       </c>
@@ -4476,7 +4482,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>125</v>
       </c>
@@ -4502,7 +4508,7 @@
         <v>-18877.708702820371</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>131</v>
       </c>
@@ -4528,7 +4534,7 @@
         <v>-19045.139985898601</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>133</v>
       </c>
@@ -4554,7 +4560,7 @@
         <v>-5.4445188599886638</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>135</v>
       </c>
@@ -4580,7 +4586,7 @@
         <v>2.671411511624413</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>137</v>
       </c>
@@ -4606,7 +4612,7 @@
         <v>9.5532474786010475</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>125</v>
       </c>
@@ -4632,7 +4638,7 @@
         <v>2866.0938229725748</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>131</v>
       </c>
@@ -4658,7 +4664,7 @@
         <v>1490.761502865475</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>133</v>
       </c>
@@ -4684,7 +4690,7 @@
         <v>2.217459469264154</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>135</v>
       </c>
@@ -4710,7 +4716,7 @@
         <v>0.2337935274525294</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>137</v>
       </c>
@@ -4736,7 +4742,7 @@
         <v>2.0873115011979051E-2</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>125</v>
       </c>
@@ -4762,7 +4768,7 @@
         <v>1351.711647219304</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>131</v>
       </c>
@@ -4788,7 +4794,7 @@
         <v>150.9391394665019</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>133</v>
       </c>
@@ -4814,7 +4820,7 @@
         <v>1.940117188288828</v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>135</v>
       </c>
@@ -4840,7 +4846,7 @@
         <v>-2.0146865510893688E-2</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>137</v>
       </c>
@@ -4874,22 +4880,22 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:G42"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="3" max="3" width="16.6640625" customWidth="1"/>
+    <col min="3" max="3" width="16.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>153</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="5" spans="1:7" s="1" customFormat="1" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" s="1" customFormat="1" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>2</v>
       </c>
@@ -4912,7 +4918,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
         <v>12</v>
       </c>
@@ -4932,7 +4938,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="7" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
         <v>12</v>
       </c>
@@ -4949,7 +4955,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="8" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
         <v>12</v>
       </c>
@@ -4966,7 +4972,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="9" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
         <v>12</v>
       </c>
@@ -4983,7 +4989,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="10" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
         <v>12</v>
       </c>
@@ -5000,7 +5006,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="11" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
         <v>12</v>
       </c>
@@ -5017,7 +5023,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
         <v>12</v>
       </c>
@@ -5034,7 +5040,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B13" t="s">
         <v>15</v>
       </c>
@@ -5051,7 +5057,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="14" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="B14" t="s">
         <v>15</v>
       </c>
@@ -5068,7 +5074,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="15" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="B15" t="s">
         <v>15</v>
       </c>
@@ -5085,7 +5091,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="16" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="B16" t="s">
         <v>15</v>
       </c>
@@ -5102,7 +5108,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="17" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B17" t="s">
         <v>15</v>
       </c>
@@ -5119,7 +5125,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="18" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B18" t="s">
         <v>15</v>
       </c>
@@ -5136,7 +5142,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="19" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B19" t="s">
         <v>15</v>
       </c>
@@ -5153,7 +5159,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="20" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B20" t="s">
         <v>18</v>
       </c>
@@ -5170,7 +5176,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="21" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B21" t="s">
         <v>18</v>
       </c>
@@ -5187,7 +5193,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="22" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B22" t="s">
         <v>18</v>
       </c>
@@ -5204,7 +5210,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="23" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B23" t="s">
         <v>18</v>
       </c>
@@ -5221,7 +5227,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="24" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B24" t="s">
         <v>18</v>
       </c>
@@ -5238,7 +5244,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="25" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B25" t="s">
         <v>18</v>
       </c>
@@ -5255,7 +5261,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="26" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B26" t="s">
         <v>18</v>
       </c>
@@ -5272,7 +5278,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="27" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B27" t="s">
         <v>28</v>
       </c>
@@ -5289,7 +5295,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="28" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B28" t="s">
         <v>28</v>
       </c>
@@ -5306,7 +5312,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="29" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B29" t="s">
         <v>28</v>
       </c>
@@ -5323,7 +5329,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="30" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B30" t="s">
         <v>28</v>
       </c>
@@ -5340,7 +5346,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="31" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B31" t="s">
         <v>28</v>
       </c>
@@ -5357,7 +5363,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="32" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B32" t="s">
         <v>28</v>
       </c>
@@ -5374,7 +5380,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="33" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B33" t="s">
         <v>28</v>
       </c>
@@ -5391,7 +5397,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="34" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="34" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B34" t="s">
         <v>31</v>
       </c>
@@ -5408,7 +5414,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="35" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="35" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B35" t="s">
         <v>31</v>
       </c>
@@ -5425,7 +5431,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="36" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="36" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B36" t="s">
         <v>31</v>
       </c>
@@ -5442,7 +5448,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="37" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="37" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B37" t="s">
         <v>31</v>
       </c>
@@ -5459,7 +5465,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="38" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="38" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B38" t="s">
         <v>31</v>
       </c>
@@ -5476,7 +5482,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="39" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="39" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B39" t="s">
         <v>31</v>
       </c>
@@ -5493,7 +5499,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="40" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="40" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B40" t="s">
         <v>31</v>
       </c>
@@ -5510,7 +5516,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="41" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="41" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B41" t="s">
         <v>31</v>
       </c>
@@ -5527,7 +5533,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="42" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="42" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B42" t="s">
         <v>31</v>
       </c>
@@ -5561,25 +5567,25 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:O8"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8.5546875" customWidth="1"/>
+    <col min="1" max="1" width="8.5703125" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
-    <col min="3" max="3" width="12.88671875" customWidth="1"/>
+    <col min="3" max="3" width="12.85546875" customWidth="1"/>
     <col min="4" max="4" width="10" customWidth="1"/>
-    <col min="6" max="6" width="6.6640625" customWidth="1"/>
-    <col min="7" max="7" width="6.5546875" customWidth="1"/>
-    <col min="8" max="8" width="8.33203125" customWidth="1"/>
-    <col min="9" max="9" width="5.5546875" customWidth="1"/>
-    <col min="10" max="10" width="6.5546875" customWidth="1"/>
-    <col min="11" max="11" width="6.109375" customWidth="1"/>
-    <col min="12" max="12" width="5.109375" customWidth="1"/>
-    <col min="13" max="13" width="5.5546875" customWidth="1"/>
-    <col min="14" max="14" width="5.109375" customWidth="1"/>
-    <col min="15" max="15" width="4.44140625" customWidth="1"/>
+    <col min="6" max="6" width="6.7109375" customWidth="1"/>
+    <col min="7" max="7" width="6.5703125" customWidth="1"/>
+    <col min="8" max="8" width="8.28515625" customWidth="1"/>
+    <col min="9" max="9" width="5.5703125" customWidth="1"/>
+    <col min="10" max="10" width="6.5703125" customWidth="1"/>
+    <col min="11" max="11" width="6.140625" customWidth="1"/>
+    <col min="12" max="12" width="5.140625" customWidth="1"/>
+    <col min="13" max="13" width="5.5703125" customWidth="1"/>
+    <col min="14" max="14" width="5.140625" customWidth="1"/>
+    <col min="15" max="15" width="4.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>255</v>
       </c>
@@ -5587,7 +5593,7 @@
         <v>256</v>
       </c>
     </row>
-    <row r="2" spans="1:15" s="8" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:15" s="8" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="8" t="s">
         <v>257</v>
       </c>
@@ -5634,7 +5640,7 @@
         <v>271</v>
       </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>272</v>
       </c>
@@ -5674,7 +5680,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>275</v>
       </c>
@@ -5689,19 +5695,19 @@
         <v>276</v>
       </c>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B5" s="3"/>
       <c r="C5" s="3"/>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B7" s="3"/>
       <c r="C7" s="3"/>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B8" s="3"/>
       <c r="C8" s="3"/>
     </row>
@@ -5720,13 +5726,13 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
   <dimension ref="A1:H21"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="4" width="10.33203125" customWidth="1"/>
-    <col min="5" max="6" width="8.5546875" customWidth="1"/>
+    <col min="2" max="4" width="10.28515625" customWidth="1"/>
+    <col min="5" max="6" width="8.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -5734,7 +5740,7 @@
         <v>277</v>
       </c>
     </row>
-    <row r="2" spans="1:8" s="8" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:8" s="8" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
@@ -5760,7 +5766,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:8" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="31" t="s">
         <v>21</v>
       </c>
@@ -5775,7 +5781,7 @@
       </c>
       <c r="G3" s="32"/>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>21</v>
       </c>
@@ -5801,7 +5807,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>21</v>
       </c>
@@ -5827,7 +5833,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:8" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="31" t="s">
         <v>21</v>
       </c>
@@ -5851,7 +5857,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>11</v>
       </c>
@@ -5877,7 +5883,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>11</v>
       </c>
@@ -5903,7 +5909,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="31" t="s">
         <v>11</v>
       </c>
@@ -5927,7 +5933,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="21" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="21" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H21" t="s">
         <v>287</v>
       </c>
@@ -5971,18 +5977,18 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
   <dimension ref="A1:G33"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.44140625" customWidth="1"/>
+    <col min="1" max="1" width="17.42578125" customWidth="1"/>
     <col min="6" max="6" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="26.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F1" s="7" t="s">
         <v>288</v>
       </c>
     </row>
-    <row r="2" spans="1:7" s="8" customFormat="1" ht="30.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:7" s="8" customFormat="1" ht="30.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="33" t="s">
         <v>257</v>
       </c>
@@ -6005,7 +6011,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>291</v>
       </c>
@@ -6022,7 +6028,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>292</v>
       </c>
@@ -6045,7 +6051,7 @@
         <v>294</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>295</v>
       </c>
@@ -6062,7 +6068,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>296</v>
       </c>
@@ -6079,7 +6085,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>297</v>
       </c>
@@ -6096,7 +6102,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>298</v>
       </c>
@@ -6113,7 +6119,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>299</v>
       </c>
@@ -6130,7 +6136,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>300</v>
       </c>
@@ -6147,7 +6153,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>301</v>
       </c>
@@ -6164,7 +6170,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>302</v>
       </c>
@@ -6181,7 +6187,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>303</v>
       </c>
@@ -6198,7 +6204,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>304</v>
       </c>
@@ -6215,7 +6221,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>305</v>
       </c>
@@ -6232,7 +6238,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>306</v>
       </c>
@@ -6249,7 +6255,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>307</v>
       </c>
@@ -6266,7 +6272,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>308</v>
       </c>
@@ -6283,7 +6289,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>309</v>
       </c>
@@ -6300,7 +6306,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>310</v>
       </c>
@@ -6317,7 +6323,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>311</v>
       </c>
@@ -6334,7 +6340,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>312</v>
       </c>
@@ -6351,7 +6357,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>313</v>
       </c>
@@ -6368,7 +6374,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>314</v>
       </c>
@@ -6385,7 +6391,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>315</v>
       </c>
@@ -6402,7 +6408,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>316</v>
       </c>
@@ -6419,7 +6425,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>317</v>
       </c>
@@ -6436,7 +6442,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>318</v>
       </c>
@@ -6453,7 +6459,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>319</v>
       </c>
@@ -6470,7 +6476,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>320</v>
       </c>
@@ -6487,7 +6493,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>321</v>
       </c>
@@ -6504,7 +6510,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>322</v>
       </c>
@@ -6521,7 +6527,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>323</v>
       </c>

</xml_diff>

<commit_message>
Many changes, moving many tools and tests in to core.py and test_core.py
</commit_message>
<xml_diff>
--- a/excels/project_table_new.xlsx
+++ b/excels/project_table_new.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\emb\Documents\PycharmProjects\blixt_rp\excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E99CE9E1-843E-4F77-875C-73CA1F1F2C2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35FB3776-D67A-48FE-BCDC-572D7E260DE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3948" yWindow="2400" windowWidth="46080" windowHeight="12168" tabRatio="685" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4104" yWindow="2184" windowWidth="38016" windowHeight="12168" tabRatio="685" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Well settings" sheetId="1" r:id="rId1"/>
@@ -19,13 +19,14 @@
     <sheet name="Templates" sheetId="7" r:id="rId4"/>
     <sheet name="Regressions" sheetId="5" r:id="rId5"/>
     <sheet name="Working intervals" sheetId="6" r:id="rId6"/>
-    <sheet name="Fluids" sheetId="8" r:id="rId7"/>
-    <sheet name="Fluid mixtures" sheetId="9" r:id="rId8"/>
-    <sheet name="Minerals" sheetId="10" r:id="rId9"/>
-    <sheet name="Mineral mixtures" sheetId="11" r:id="rId10"/>
-    <sheet name="Prospects overview" sheetId="13" r:id="rId11"/>
-    <sheet name="QSI decision table" sheetId="14" r:id="rId12"/>
-    <sheet name="Utils" sheetId="12" r:id="rId13"/>
+    <sheet name="Stratigraphic units" sheetId="16" r:id="rId7"/>
+    <sheet name="Fluids" sheetId="8" r:id="rId8"/>
+    <sheet name="Fluid mixtures" sheetId="9" r:id="rId9"/>
+    <sheet name="Minerals" sheetId="10" r:id="rId10"/>
+    <sheet name="Mineral mixtures" sheetId="11" r:id="rId11"/>
+    <sheet name="Prospects overview" sheetId="13" r:id="rId12"/>
+    <sheet name="QSI decision table" sheetId="14" r:id="rId13"/>
+    <sheet name="Utils" sheetId="12" r:id="rId14"/>
   </sheets>
   <definedNames>
     <definedName name="AvoClasses">Utils!$Q$3:$Q$7</definedName>
@@ -62,7 +63,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="919" uniqueCount="391">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="976" uniqueCount="394">
   <si>
     <t>Select Yes or No</t>
   </si>
@@ -1244,6 +1245,15 @@
   </si>
   <si>
     <t>dimensionless</t>
+  </si>
+  <si>
+    <t>Level</t>
+  </si>
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t xml:space="preserve">high value means subunit </t>
   </si>
 </sst>
 </file>
@@ -1511,7 +1521,58 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="15">
+  <dxfs count="17">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C5700"/>
@@ -1560,36 +1621,6 @@
       <fill>
         <patternFill>
           <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2136,10 +2167,10 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A3:A20">
-    <cfRule type="cellIs" dxfId="14" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="16" priority="1" operator="equal">
       <formula>"Yes"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="13" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="15" priority="2" operator="equal">
       <formula>"No"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -2148,6 +2179,582 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
+  <dimension ref="A1:G33"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="17.44140625" customWidth="1"/>
+    <col min="6" max="6" width="18" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" ht="26.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="F1" s="7" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" s="8" customFormat="1" ht="30.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="33" t="s">
+        <v>257</v>
+      </c>
+      <c r="B2" s="34" t="s">
+        <v>258</v>
+      </c>
+      <c r="C2" s="34" t="s">
+        <v>259</v>
+      </c>
+      <c r="D2" s="34" t="s">
+        <v>260</v>
+      </c>
+      <c r="E2" s="33" t="s">
+        <v>289</v>
+      </c>
+      <c r="F2" s="33" t="s">
+        <v>261</v>
+      </c>
+      <c r="G2" s="33" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>291</v>
+      </c>
+      <c r="B3">
+        <v>36.6</v>
+      </c>
+      <c r="C3">
+        <v>45</v>
+      </c>
+      <c r="D3">
+        <v>2.65</v>
+      </c>
+      <c r="E3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>292</v>
+      </c>
+      <c r="B4">
+        <v>11.4</v>
+      </c>
+      <c r="C4">
+        <v>3</v>
+      </c>
+      <c r="D4">
+        <v>2.35</v>
+      </c>
+      <c r="E4">
+        <v>0</v>
+      </c>
+      <c r="F4" t="s">
+        <v>293</v>
+      </c>
+      <c r="G4" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>295</v>
+      </c>
+      <c r="B5">
+        <v>76.8</v>
+      </c>
+      <c r="C5">
+        <v>32</v>
+      </c>
+      <c r="D5">
+        <v>2.71</v>
+      </c>
+      <c r="E5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>296</v>
+      </c>
+      <c r="B6">
+        <v>94.9</v>
+      </c>
+      <c r="C6">
+        <v>45</v>
+      </c>
+      <c r="D6">
+        <v>2.87</v>
+      </c>
+      <c r="E6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>297</v>
+      </c>
+      <c r="B7">
+        <v>26</v>
+      </c>
+      <c r="C7">
+        <v>32</v>
+      </c>
+      <c r="D7">
+        <v>2.35</v>
+      </c>
+      <c r="E7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>298</v>
+      </c>
+      <c r="B8">
+        <v>47</v>
+      </c>
+      <c r="C8">
+        <v>39</v>
+      </c>
+      <c r="D8">
+        <v>2.94</v>
+      </c>
+      <c r="E8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>299</v>
+      </c>
+      <c r="B9">
+        <v>114</v>
+      </c>
+      <c r="C9">
+        <v>68</v>
+      </c>
+      <c r="D9">
+        <v>3.01</v>
+      </c>
+      <c r="E9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>300</v>
+      </c>
+      <c r="B10">
+        <v>55</v>
+      </c>
+      <c r="C10">
+        <v>28</v>
+      </c>
+      <c r="D10">
+        <v>2.62</v>
+      </c>
+      <c r="E10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>301</v>
+      </c>
+      <c r="B11">
+        <v>48</v>
+      </c>
+      <c r="C11">
+        <v>24</v>
+      </c>
+      <c r="D11">
+        <v>2.56</v>
+      </c>
+      <c r="E11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>302</v>
+      </c>
+      <c r="B12">
+        <v>85</v>
+      </c>
+      <c r="C12">
+        <v>38</v>
+      </c>
+      <c r="D12">
+        <v>2.73</v>
+      </c>
+      <c r="E12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>303</v>
+      </c>
+      <c r="B13">
+        <v>52</v>
+      </c>
+      <c r="C13">
+        <v>31.5</v>
+      </c>
+      <c r="D13">
+        <v>2.82</v>
+      </c>
+      <c r="E13">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>304</v>
+      </c>
+      <c r="B14">
+        <v>50</v>
+      </c>
+      <c r="C14">
+        <v>27.5</v>
+      </c>
+      <c r="D14">
+        <v>3</v>
+      </c>
+      <c r="E14">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>305</v>
+      </c>
+      <c r="B15">
+        <v>25.2</v>
+      </c>
+      <c r="C15">
+        <v>15.3</v>
+      </c>
+      <c r="D15">
+        <v>2.16</v>
+      </c>
+      <c r="E15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>306</v>
+      </c>
+      <c r="B16">
+        <v>66.5</v>
+      </c>
+      <c r="C16">
+        <v>34</v>
+      </c>
+      <c r="D16">
+        <v>3</v>
+      </c>
+      <c r="E16">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>307</v>
+      </c>
+      <c r="B17">
+        <v>58</v>
+      </c>
+      <c r="C17">
+        <v>30</v>
+      </c>
+      <c r="D17">
+        <v>2.31</v>
+      </c>
+      <c r="E17">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>308</v>
+      </c>
+      <c r="B18">
+        <v>158</v>
+      </c>
+      <c r="C18">
+        <v>149</v>
+      </c>
+      <c r="D18">
+        <v>5.0199999999999996</v>
+      </c>
+      <c r="E18">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>309</v>
+      </c>
+      <c r="B19">
+        <v>27</v>
+      </c>
+      <c r="C19">
+        <v>17</v>
+      </c>
+      <c r="D19">
+        <v>2.68</v>
+      </c>
+      <c r="E19">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>310</v>
+      </c>
+      <c r="B20">
+        <v>123.7</v>
+      </c>
+      <c r="C20">
+        <v>51</v>
+      </c>
+      <c r="D20">
+        <v>3.96</v>
+      </c>
+      <c r="E20">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>311</v>
+      </c>
+      <c r="B21">
+        <v>15</v>
+      </c>
+      <c r="C21">
+        <v>10</v>
+      </c>
+      <c r="D21">
+        <v>2.67</v>
+      </c>
+      <c r="E21">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>312</v>
+      </c>
+      <c r="B22">
+        <v>17.96</v>
+      </c>
+      <c r="C22">
+        <v>32.409999999999997</v>
+      </c>
+      <c r="D22">
+        <v>2.52</v>
+      </c>
+      <c r="E22">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>313</v>
+      </c>
+      <c r="B23">
+        <v>55.8</v>
+      </c>
+      <c r="C23">
+        <v>33.299999999999997</v>
+      </c>
+      <c r="D23">
+        <v>2.59</v>
+      </c>
+      <c r="E23">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>314</v>
+      </c>
+      <c r="B24">
+        <v>87</v>
+      </c>
+      <c r="C24">
+        <v>43</v>
+      </c>
+      <c r="D24">
+        <v>3.12</v>
+      </c>
+      <c r="E24">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>315</v>
+      </c>
+      <c r="B25">
+        <v>103.67</v>
+      </c>
+      <c r="C25">
+        <v>60.82</v>
+      </c>
+      <c r="D25">
+        <v>3.32</v>
+      </c>
+      <c r="E25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>316</v>
+      </c>
+      <c r="B26">
+        <v>129.13999999999999</v>
+      </c>
+      <c r="C26">
+        <v>79.150000000000006</v>
+      </c>
+      <c r="D26">
+        <v>3.31</v>
+      </c>
+      <c r="E26">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
+        <v>317</v>
+      </c>
+      <c r="B27">
+        <v>4.5199999999999996</v>
+      </c>
+      <c r="C27">
+        <v>2.61</v>
+      </c>
+      <c r="D27">
+        <v>1.24</v>
+      </c>
+      <c r="E27">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
+        <v>318</v>
+      </c>
+      <c r="B28">
+        <v>160.29</v>
+      </c>
+      <c r="C28">
+        <v>91.38</v>
+      </c>
+      <c r="D28">
+        <v>5.18</v>
+      </c>
+      <c r="E28">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
+        <v>319</v>
+      </c>
+      <c r="B29">
+        <v>62.2</v>
+      </c>
+      <c r="C29">
+        <v>25.7</v>
+      </c>
+      <c r="D29">
+        <v>2.71</v>
+      </c>
+      <c r="E29">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A30" t="s">
+        <v>320</v>
+      </c>
+      <c r="B30">
+        <v>146.25</v>
+      </c>
+      <c r="C30">
+        <v>68.150000000000006</v>
+      </c>
+      <c r="D30">
+        <v>2.76</v>
+      </c>
+      <c r="E30">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
+        <v>321</v>
+      </c>
+      <c r="B31">
+        <v>48.35</v>
+      </c>
+      <c r="C31">
+        <v>21.9</v>
+      </c>
+      <c r="D31">
+        <v>2.44</v>
+      </c>
+      <c r="E31">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A32" t="s">
+        <v>322</v>
+      </c>
+      <c r="B32">
+        <v>2.9</v>
+      </c>
+      <c r="C32">
+        <v>2.7</v>
+      </c>
+      <c r="D32">
+        <v>1.3</v>
+      </c>
+      <c r="E32">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A33" t="s">
+        <v>323</v>
+      </c>
+      <c r="B33">
+        <v>12.3</v>
+      </c>
+      <c r="C33">
+        <v>15.6</v>
+      </c>
+      <c r="D33">
+        <v>2.6259999999999999</v>
+      </c>
+      <c r="E33">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
   <dimension ref="A1:D4"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -2206,15 +2813,15 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A3:C15 D5:D6">
-    <cfRule type="cellIs" dxfId="7" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="4" priority="1" operator="equal">
       <formula>"Initial"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A3:C17 D5:D6">
-    <cfRule type="cellIs" dxfId="6" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="3" priority="2" operator="equal">
       <formula>"Inital"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="5" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="2" priority="3" operator="equal">
       <formula>"Final"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -2232,7 +2839,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CCD9C215-DCD2-40A2-A7D5-172DC530BE0E}">
   <dimension ref="A1:Q2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -2308,7 +2915,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3CCC2506-3BD3-4476-A9AA-1673C259914E}">
   <dimension ref="A1:M2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -2369,7 +2976,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
   <dimension ref="A1:Q18"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -3049,10 +3656,10 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="B3:B16">
-    <cfRule type="cellIs" dxfId="12" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="14" priority="1" operator="equal">
       <formula>"Yes"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="11" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="13" priority="2" operator="equal">
       <formula>"No"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3391,10 +3998,10 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="B3:B20">
-    <cfRule type="cellIs" dxfId="10" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="12" priority="1" operator="equal">
       <formula>"Yes"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="9" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="11" priority="2" operator="equal">
       <formula>"No"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5565,6 +6172,281 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9DE0C751-ACC1-462A-82AF-4CE9BB91C06B}">
+  <dimension ref="A2:G21"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="C4" t="s">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A5" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>257</v>
+      </c>
+      <c r="C5" s="12" t="s">
+        <v>391</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>392</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>11</v>
+      </c>
+      <c r="B6" t="s">
+        <v>127</v>
+      </c>
+      <c r="C6">
+        <v>1</v>
+      </c>
+      <c r="F6" s="20" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>11</v>
+      </c>
+      <c r="B7" t="s">
+        <v>146</v>
+      </c>
+      <c r="C7">
+        <v>1</v>
+      </c>
+      <c r="F7" s="26" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>11</v>
+      </c>
+      <c r="B8" t="s">
+        <v>161</v>
+      </c>
+      <c r="C8">
+        <v>1</v>
+      </c>
+      <c r="F8" s="22" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>11</v>
+      </c>
+      <c r="B9" t="s">
+        <v>162</v>
+      </c>
+      <c r="C9">
+        <v>1</v>
+      </c>
+      <c r="F9" s="23" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>11</v>
+      </c>
+      <c r="B10" t="s">
+        <v>163</v>
+      </c>
+      <c r="C10">
+        <v>1</v>
+      </c>
+      <c r="F10" s="27" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>11</v>
+      </c>
+      <c r="B11" t="s">
+        <v>164</v>
+      </c>
+      <c r="C11">
+        <v>1</v>
+      </c>
+      <c r="F11" s="24" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>21</v>
+      </c>
+      <c r="B12" t="s">
+        <v>139</v>
+      </c>
+      <c r="C12">
+        <v>1</v>
+      </c>
+      <c r="F12" s="25" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>21</v>
+      </c>
+      <c r="B13" s="30" t="s">
+        <v>165</v>
+      </c>
+      <c r="C13">
+        <v>1</v>
+      </c>
+      <c r="F13" s="16" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>21</v>
+      </c>
+      <c r="B14" s="30" t="s">
+        <v>167</v>
+      </c>
+      <c r="C14">
+        <v>1</v>
+      </c>
+      <c r="F14" s="20" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>21</v>
+      </c>
+      <c r="B15" s="30" t="s">
+        <v>168</v>
+      </c>
+      <c r="C15">
+        <v>1</v>
+      </c>
+      <c r="F15" s="26" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>21</v>
+      </c>
+      <c r="B16" s="30" t="s">
+        <v>169</v>
+      </c>
+      <c r="C16">
+        <v>1</v>
+      </c>
+      <c r="F16" s="22" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>21</v>
+      </c>
+      <c r="B17" s="30" t="s">
+        <v>170</v>
+      </c>
+      <c r="C17">
+        <v>1</v>
+      </c>
+      <c r="F17" s="23" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>21</v>
+      </c>
+      <c r="B18" s="30" t="s">
+        <v>171</v>
+      </c>
+      <c r="C18">
+        <v>1</v>
+      </c>
+      <c r="F18" s="27" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>21</v>
+      </c>
+      <c r="B19" s="30" t="s">
+        <v>172</v>
+      </c>
+      <c r="C19">
+        <v>1</v>
+      </c>
+      <c r="F19" s="24" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>21</v>
+      </c>
+      <c r="B20" s="30" t="s">
+        <v>173</v>
+      </c>
+      <c r="C20">
+        <v>1</v>
+      </c>
+      <c r="F20" s="25" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>21</v>
+      </c>
+      <c r="B21" s="30" t="s">
+        <v>174</v>
+      </c>
+      <c r="C21">
+        <v>1</v>
+      </c>
+      <c r="F21" s="16" t="s">
+        <v>19</v>
+      </c>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="A6:A22">
+    <cfRule type="cellIs" dxfId="1" priority="1" operator="equal">
+      <formula>"Yes"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="0" priority="2" operator="equal">
+      <formula>"No"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:O8"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -5713,7 +6595,7 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A3:A28">
-    <cfRule type="duplicateValues" dxfId="8" priority="6"/>
+    <cfRule type="duplicateValues" dxfId="10" priority="6"/>
   </conditionalFormatting>
   <dataValidations count="1">
     <dataValidation showInputMessage="1" showErrorMessage="1" prompt="No duplicate names please" sqref="A3:A38" xr:uid="{00000000-0002-0000-0700-000000000000}"/>
@@ -5723,7 +6605,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
   <dimension ref="A1:H21"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -5940,23 +6822,23 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A3:A32">
-    <cfRule type="cellIs" dxfId="4" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="9" priority="1" operator="equal">
       <formula>"Yes"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="3" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="8" priority="2" operator="equal">
       <formula>"No"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B3:D15">
-    <cfRule type="cellIs" dxfId="2" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="7" priority="3" operator="equal">
       <formula>"Initial"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B3:D17">
-    <cfRule type="cellIs" dxfId="1" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="6" priority="4" operator="equal">
       <formula>"Inital"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="5" operator="equal">
+    <cfRule type="cellIs" dxfId="5" priority="5" operator="equal">
       <formula>"Final"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5972,580 +6854,4 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
-  <dimension ref="A1:G33"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="17.44140625" customWidth="1"/>
-    <col min="6" max="6" width="18" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:7" ht="26.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="F1" s="7" t="s">
-        <v>288</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" s="8" customFormat="1" ht="30.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="33" t="s">
-        <v>257</v>
-      </c>
-      <c r="B2" s="34" t="s">
-        <v>258</v>
-      </c>
-      <c r="C2" s="34" t="s">
-        <v>259</v>
-      </c>
-      <c r="D2" s="34" t="s">
-        <v>260</v>
-      </c>
-      <c r="E2" s="33" t="s">
-        <v>289</v>
-      </c>
-      <c r="F2" s="33" t="s">
-        <v>261</v>
-      </c>
-      <c r="G2" s="33" t="s">
-        <v>290</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>291</v>
-      </c>
-      <c r="B3">
-        <v>36.6</v>
-      </c>
-      <c r="C3">
-        <v>45</v>
-      </c>
-      <c r="D3">
-        <v>2.65</v>
-      </c>
-      <c r="E3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>292</v>
-      </c>
-      <c r="B4">
-        <v>11.4</v>
-      </c>
-      <c r="C4">
-        <v>3</v>
-      </c>
-      <c r="D4">
-        <v>2.35</v>
-      </c>
-      <c r="E4">
-        <v>0</v>
-      </c>
-      <c r="F4" t="s">
-        <v>293</v>
-      </c>
-      <c r="G4" t="s">
-        <v>294</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>295</v>
-      </c>
-      <c r="B5">
-        <v>76.8</v>
-      </c>
-      <c r="C5">
-        <v>32</v>
-      </c>
-      <c r="D5">
-        <v>2.71</v>
-      </c>
-      <c r="E5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>296</v>
-      </c>
-      <c r="B6">
-        <v>94.9</v>
-      </c>
-      <c r="C6">
-        <v>45</v>
-      </c>
-      <c r="D6">
-        <v>2.87</v>
-      </c>
-      <c r="E6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>297</v>
-      </c>
-      <c r="B7">
-        <v>26</v>
-      </c>
-      <c r="C7">
-        <v>32</v>
-      </c>
-      <c r="D7">
-        <v>2.35</v>
-      </c>
-      <c r="E7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>298</v>
-      </c>
-      <c r="B8">
-        <v>47</v>
-      </c>
-      <c r="C8">
-        <v>39</v>
-      </c>
-      <c r="D8">
-        <v>2.94</v>
-      </c>
-      <c r="E8">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>299</v>
-      </c>
-      <c r="B9">
-        <v>114</v>
-      </c>
-      <c r="C9">
-        <v>68</v>
-      </c>
-      <c r="D9">
-        <v>3.01</v>
-      </c>
-      <c r="E9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>300</v>
-      </c>
-      <c r="B10">
-        <v>55</v>
-      </c>
-      <c r="C10">
-        <v>28</v>
-      </c>
-      <c r="D10">
-        <v>2.62</v>
-      </c>
-      <c r="E10">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
-        <v>301</v>
-      </c>
-      <c r="B11">
-        <v>48</v>
-      </c>
-      <c r="C11">
-        <v>24</v>
-      </c>
-      <c r="D11">
-        <v>2.56</v>
-      </c>
-      <c r="E11">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
-        <v>302</v>
-      </c>
-      <c r="B12">
-        <v>85</v>
-      </c>
-      <c r="C12">
-        <v>38</v>
-      </c>
-      <c r="D12">
-        <v>2.73</v>
-      </c>
-      <c r="E12">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A13" t="s">
-        <v>303</v>
-      </c>
-      <c r="B13">
-        <v>52</v>
-      </c>
-      <c r="C13">
-        <v>31.5</v>
-      </c>
-      <c r="D13">
-        <v>2.82</v>
-      </c>
-      <c r="E13">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A14" t="s">
-        <v>304</v>
-      </c>
-      <c r="B14">
-        <v>50</v>
-      </c>
-      <c r="C14">
-        <v>27.5</v>
-      </c>
-      <c r="D14">
-        <v>3</v>
-      </c>
-      <c r="E14">
-        <v>275</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A15" t="s">
-        <v>305</v>
-      </c>
-      <c r="B15">
-        <v>25.2</v>
-      </c>
-      <c r="C15">
-        <v>15.3</v>
-      </c>
-      <c r="D15">
-        <v>2.16</v>
-      </c>
-      <c r="E15">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A16" t="s">
-        <v>306</v>
-      </c>
-      <c r="B16">
-        <v>66.5</v>
-      </c>
-      <c r="C16">
-        <v>34</v>
-      </c>
-      <c r="D16">
-        <v>3</v>
-      </c>
-      <c r="E16">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A17" t="s">
-        <v>307</v>
-      </c>
-      <c r="B17">
-        <v>58</v>
-      </c>
-      <c r="C17">
-        <v>30</v>
-      </c>
-      <c r="D17">
-        <v>2.31</v>
-      </c>
-      <c r="E17">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A18" t="s">
-        <v>308</v>
-      </c>
-      <c r="B18">
-        <v>158</v>
-      </c>
-      <c r="C18">
-        <v>149</v>
-      </c>
-      <c r="D18">
-        <v>5.0199999999999996</v>
-      </c>
-      <c r="E18">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A19" t="s">
-        <v>309</v>
-      </c>
-      <c r="B19">
-        <v>27</v>
-      </c>
-      <c r="C19">
-        <v>17</v>
-      </c>
-      <c r="D19">
-        <v>2.68</v>
-      </c>
-      <c r="E19">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A20" t="s">
-        <v>310</v>
-      </c>
-      <c r="B20">
-        <v>123.7</v>
-      </c>
-      <c r="C20">
-        <v>51</v>
-      </c>
-      <c r="D20">
-        <v>3.96</v>
-      </c>
-      <c r="E20">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A21" t="s">
-        <v>311</v>
-      </c>
-      <c r="B21">
-        <v>15</v>
-      </c>
-      <c r="C21">
-        <v>10</v>
-      </c>
-      <c r="D21">
-        <v>2.67</v>
-      </c>
-      <c r="E21">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A22" t="s">
-        <v>312</v>
-      </c>
-      <c r="B22">
-        <v>17.96</v>
-      </c>
-      <c r="C22">
-        <v>32.409999999999997</v>
-      </c>
-      <c r="D22">
-        <v>2.52</v>
-      </c>
-      <c r="E22">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A23" t="s">
-        <v>313</v>
-      </c>
-      <c r="B23">
-        <v>55.8</v>
-      </c>
-      <c r="C23">
-        <v>33.299999999999997</v>
-      </c>
-      <c r="D23">
-        <v>2.59</v>
-      </c>
-      <c r="E23">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A24" t="s">
-        <v>314</v>
-      </c>
-      <c r="B24">
-        <v>87</v>
-      </c>
-      <c r="C24">
-        <v>43</v>
-      </c>
-      <c r="D24">
-        <v>3.12</v>
-      </c>
-      <c r="E24">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A25" t="s">
-        <v>315</v>
-      </c>
-      <c r="B25">
-        <v>103.67</v>
-      </c>
-      <c r="C25">
-        <v>60.82</v>
-      </c>
-      <c r="D25">
-        <v>3.32</v>
-      </c>
-      <c r="E25">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A26" t="s">
-        <v>316</v>
-      </c>
-      <c r="B26">
-        <v>129.13999999999999</v>
-      </c>
-      <c r="C26">
-        <v>79.150000000000006</v>
-      </c>
-      <c r="D26">
-        <v>3.31</v>
-      </c>
-      <c r="E26">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A27" t="s">
-        <v>317</v>
-      </c>
-      <c r="B27">
-        <v>4.5199999999999996</v>
-      </c>
-      <c r="C27">
-        <v>2.61</v>
-      </c>
-      <c r="D27">
-        <v>1.24</v>
-      </c>
-      <c r="E27">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A28" t="s">
-        <v>318</v>
-      </c>
-      <c r="B28">
-        <v>160.29</v>
-      </c>
-      <c r="C28">
-        <v>91.38</v>
-      </c>
-      <c r="D28">
-        <v>5.18</v>
-      </c>
-      <c r="E28">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A29" t="s">
-        <v>319</v>
-      </c>
-      <c r="B29">
-        <v>62.2</v>
-      </c>
-      <c r="C29">
-        <v>25.7</v>
-      </c>
-      <c r="D29">
-        <v>2.71</v>
-      </c>
-      <c r="E29">
-        <v>275</v>
-      </c>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A30" t="s">
-        <v>320</v>
-      </c>
-      <c r="B30">
-        <v>146.25</v>
-      </c>
-      <c r="C30">
-        <v>68.150000000000006</v>
-      </c>
-      <c r="D30">
-        <v>2.76</v>
-      </c>
-      <c r="E30">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A31" t="s">
-        <v>321</v>
-      </c>
-      <c r="B31">
-        <v>48.35</v>
-      </c>
-      <c r="C31">
-        <v>21.9</v>
-      </c>
-      <c r="D31">
-        <v>2.44</v>
-      </c>
-      <c r="E31">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A32" t="s">
-        <v>322</v>
-      </c>
-      <c r="B32">
-        <v>2.9</v>
-      </c>
-      <c r="C32">
-        <v>2.7</v>
-      </c>
-      <c r="D32">
-        <v>1.3</v>
-      </c>
-      <c r="E32">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A33" t="s">
-        <v>323</v>
-      </c>
-      <c r="B33">
-        <v>12.3</v>
-      </c>
-      <c r="C33">
-        <v>15.6</v>
-      </c>
-      <c r="D33">
-        <v>2.6259999999999999</v>
-      </c>
-      <c r="E33">
-        <v>0</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
A lot of work on plotting synthetic seismic using the log_plotter.py. Still in progress
</commit_message>
<xml_diff>
--- a/excels/project_table_new.xlsx
+++ b/excels/project_table_new.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\emb\Documents\PycharmProjects\blixt_rp\excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35FB3776-D67A-48FE-BCDC-572D7E260DE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F369DA65-5AF8-4DDF-BAD2-7DE56728FBCC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4104" yWindow="2184" windowWidth="38016" windowHeight="12168" tabRatio="685" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="33204" yWindow="2664" windowWidth="27168" windowHeight="12168" tabRatio="685" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Well settings" sheetId="1" r:id="rId1"/>
@@ -1524,27 +1524,6 @@
   <dxfs count="17">
     <dxf>
       <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
         <color rgb="FF9C5700"/>
       </font>
       <fill>
@@ -1632,6 +1611,27 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFC00000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2813,15 +2813,15 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A3:C15 D5:D6">
-    <cfRule type="cellIs" dxfId="4" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="2" priority="1" operator="equal">
       <formula>"Initial"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A3:C17 D5:D6">
-    <cfRule type="cellIs" dxfId="3" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
       <formula>"Inital"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="0" priority="3" operator="equal">
       <formula>"Final"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -4132,10 +4132,10 @@
         <v>193</v>
       </c>
       <c r="F4" s="3">
-        <v>3500</v>
+        <v>2000</v>
       </c>
       <c r="G4" s="3">
-        <v>4800</v>
+        <v>5000</v>
       </c>
       <c r="I4" t="s">
         <v>194</v>
@@ -4164,10 +4164,10 @@
         <v>193</v>
       </c>
       <c r="F5" s="3">
-        <v>1800</v>
+        <v>800</v>
       </c>
       <c r="G5" s="3">
-        <v>3000</v>
+        <v>3500</v>
       </c>
       <c r="I5" t="s">
         <v>194</v>
@@ -4459,10 +4459,10 @@
         <v>193</v>
       </c>
       <c r="F14" s="3">
-        <v>2</v>
+        <v>1.8</v>
       </c>
       <c r="G14" s="3">
-        <v>3</v>
+        <v>3.2</v>
       </c>
       <c r="I14" t="s">
         <v>194</v>
@@ -6211,7 +6211,7 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>11</v>
+        <v>21</v>
       </c>
       <c r="B6" t="s">
         <v>127</v>
@@ -6435,10 +6435,10 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A6:A22">
-    <cfRule type="cellIs" dxfId="1" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="10" priority="1" operator="equal">
       <formula>"Yes"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="9" priority="2" operator="equal">
       <formula>"No"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -6595,7 +6595,7 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A3:A28">
-    <cfRule type="duplicateValues" dxfId="10" priority="6"/>
+    <cfRule type="duplicateValues" dxfId="8" priority="6"/>
   </conditionalFormatting>
   <dataValidations count="1">
     <dataValidation showInputMessage="1" showErrorMessage="1" prompt="No duplicate names please" sqref="A3:A38" xr:uid="{00000000-0002-0000-0700-000000000000}"/>
@@ -6822,23 +6822,23 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A3:A32">
-    <cfRule type="cellIs" dxfId="9" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="7" priority="1" operator="equal">
       <formula>"Yes"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="8" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="6" priority="2" operator="equal">
       <formula>"No"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B3:D15">
-    <cfRule type="cellIs" dxfId="7" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="5" priority="3" operator="equal">
       <formula>"Initial"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B3:D17">
-    <cfRule type="cellIs" dxfId="6" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="4" priority="4" operator="equal">
       <formula>"Inital"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="5" priority="5" operator="equal">
+    <cfRule type="cellIs" dxfId="3" priority="5" operator="equal">
       <formula>"Final"</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
Added a function interactive_edits() to plot_logs_new.py which allows interactive fixes of logs, and saving the result to las
</commit_message>
<xml_diff>
--- a/excels/project_table_new.xlsx
+++ b/excels/project_table_new.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\emb\Documents\PycharmProjects\blixt_rp\excels\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marte\PycharmProjects\blixt_rp\excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F369DA65-5AF8-4DDF-BAD2-7DE56728FBCC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B569FA14-30A6-4A63-8194-BCD6B539ECE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="33204" yWindow="2664" windowWidth="27168" windowHeight="12168" tabRatio="685" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4950" yWindow="1455" windowWidth="21600" windowHeight="13440" tabRatio="685" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Well settings" sheetId="1" r:id="rId1"/>
@@ -63,7 +63,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="976" uniqueCount="394">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="976" uniqueCount="395">
   <si>
     <t>Select Yes or No</t>
   </si>
@@ -1254,6 +1254,9 @@
   </si>
   <si>
     <t xml:space="preserve">high value means subunit </t>
+  </si>
+  <si>
+    <t>us / F</t>
   </si>
 </sst>
 </file>
@@ -1973,13 +1976,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:I13"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="5.6640625" customWidth="1"/>
-    <col min="2" max="2" width="12.44140625" customWidth="1"/>
+    <col min="1" max="1" width="5.7109375" customWidth="1"/>
+    <col min="2" max="2" width="12.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1990,7 +1993,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:9" s="1" customFormat="1" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:9" s="1" customFormat="1" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
@@ -2019,7 +2022,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>21</v>
       </c>
@@ -2039,7 +2042,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>21</v>
       </c>
@@ -2053,7 +2056,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>21</v>
       </c>
@@ -2067,7 +2070,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>21</v>
       </c>
@@ -2081,7 +2084,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>21</v>
       </c>
@@ -2095,7 +2098,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>11</v>
       </c>
@@ -2115,7 +2118,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>21</v>
       </c>
@@ -2132,7 +2135,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B10" s="13"/>
       <c r="C10" s="20" t="s">
         <v>23</v>
@@ -2141,7 +2144,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="C11" s="21" t="s">
         <v>35</v>
       </c>
@@ -2149,7 +2152,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="C12" s="22" t="s">
         <v>37</v>
       </c>
@@ -2157,7 +2160,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="C13" s="23" t="s">
         <v>39</v>
       </c>
@@ -2181,18 +2184,18 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
   <dimension ref="A1:G33"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.44140625" customWidth="1"/>
+    <col min="1" max="1" width="17.42578125" customWidth="1"/>
     <col min="6" max="6" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="26.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F1" s="7" t="s">
         <v>288</v>
       </c>
     </row>
-    <row r="2" spans="1:7" s="8" customFormat="1" ht="30.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:7" s="8" customFormat="1" ht="30.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="33" t="s">
         <v>257</v>
       </c>
@@ -2215,7 +2218,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>291</v>
       </c>
@@ -2232,7 +2235,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>292</v>
       </c>
@@ -2255,7 +2258,7 @@
         <v>294</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>295</v>
       </c>
@@ -2272,7 +2275,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>296</v>
       </c>
@@ -2289,7 +2292,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>297</v>
       </c>
@@ -2306,7 +2309,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>298</v>
       </c>
@@ -2323,7 +2326,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>299</v>
       </c>
@@ -2340,7 +2343,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>300</v>
       </c>
@@ -2357,7 +2360,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>301</v>
       </c>
@@ -2374,7 +2377,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>302</v>
       </c>
@@ -2391,7 +2394,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>303</v>
       </c>
@@ -2408,7 +2411,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>304</v>
       </c>
@@ -2425,7 +2428,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>305</v>
       </c>
@@ -2442,7 +2445,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>306</v>
       </c>
@@ -2459,7 +2462,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>307</v>
       </c>
@@ -2476,7 +2479,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>308</v>
       </c>
@@ -2493,7 +2496,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>309</v>
       </c>
@@ -2510,7 +2513,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>310</v>
       </c>
@@ -2527,7 +2530,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>311</v>
       </c>
@@ -2544,7 +2547,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>312</v>
       </c>
@@ -2561,7 +2564,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>313</v>
       </c>
@@ -2578,7 +2581,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>314</v>
       </c>
@@ -2595,7 +2598,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>315</v>
       </c>
@@ -2612,7 +2615,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>316</v>
       </c>
@@ -2629,7 +2632,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>317</v>
       </c>
@@ -2646,7 +2649,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>318</v>
       </c>
@@ -2663,7 +2666,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>319</v>
       </c>
@@ -2680,7 +2683,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>320</v>
       </c>
@@ -2697,7 +2700,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>321</v>
       </c>
@@ -2714,7 +2717,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>322</v>
       </c>
@@ -2731,7 +2734,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>323</v>
       </c>
@@ -2757,19 +2760,19 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
   <dimension ref="A1:D4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="2" width="10.33203125" customWidth="1"/>
-    <col min="3" max="3" width="17.44140625" customWidth="1"/>
+    <col min="1" max="2" width="10.28515625" customWidth="1"/>
+    <col min="3" max="3" width="17.42578125" customWidth="1"/>
     <col min="4" max="4" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="26.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D1" s="5" t="s">
         <v>324</v>
       </c>
     </row>
-    <row r="2" spans="1:4" s="8" customFormat="1" ht="30.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:4" s="8" customFormat="1" ht="30.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="9" t="s">
         <v>279</v>
       </c>
@@ -2783,7 +2786,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>28</v>
       </c>
@@ -2797,7 +2800,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>28</v>
       </c>
@@ -2842,9 +2845,9 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CCD9C215-DCD2-40A2-A7D5-172DC530BE0E}">
   <dimension ref="A1:Q2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
       <c r="D1" s="2"/>
@@ -2865,7 +2868,7 @@
       </c>
       <c r="O1" s="2"/>
     </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>374</v>
       </c>
@@ -2918,9 +2921,9 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3CCC2506-3BD3-4476-A9AA-1673C259914E}">
   <dimension ref="A1:M2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" s="2"/>
       <c r="B1" s="2" t="s">
         <v>379</v>
@@ -2933,7 +2936,7 @@
       <c r="I1" s="2"/>
       <c r="K1" s="2"/>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>375</v>
       </c>
@@ -2979,19 +2982,19 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
   <dimension ref="A1:Q18"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="16.33203125" customWidth="1"/>
-    <col min="3" max="3" width="12.33203125" customWidth="1"/>
-    <col min="4" max="4" width="9.88671875" customWidth="1"/>
+    <col min="2" max="2" width="16.28515625" customWidth="1"/>
+    <col min="3" max="3" width="12.28515625" customWidth="1"/>
+    <col min="4" max="4" width="9.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="H1" s="2" t="s">
         <v>362</v>
       </c>
     </row>
-    <row r="2" spans="1:17" s="6" customFormat="1" ht="42.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:17" s="6" customFormat="1" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2" s="6" t="s">
         <v>326</v>
       </c>
@@ -3041,7 +3044,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>11</v>
       </c>
@@ -3095,7 +3098,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>21</v>
       </c>
@@ -3146,7 +3149,7 @@
         <v>355</v>
       </c>
     </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
       <c r="E5" t="s">
         <v>340</v>
       </c>
@@ -3173,7 +3176,7 @@
         <v>357</v>
       </c>
     </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
       <c r="F6" t="s">
         <v>27</v>
       </c>
@@ -3194,7 +3197,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
       <c r="F7" t="s">
         <v>30</v>
       </c>
@@ -3212,7 +3215,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
       <c r="F8" t="s">
         <v>33</v>
       </c>
@@ -3224,7 +3227,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
       <c r="F9" t="s">
         <v>24</v>
       </c>
@@ -3236,7 +3239,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="10" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:17" x14ac:dyDescent="0.25">
       <c r="F10" t="s">
         <v>36</v>
       </c>
@@ -3248,7 +3251,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:17" x14ac:dyDescent="0.25">
       <c r="F11" t="s">
         <v>38</v>
       </c>
@@ -3260,7 +3263,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:17" x14ac:dyDescent="0.25">
       <c r="F12" t="s">
         <v>40</v>
       </c>
@@ -3272,7 +3275,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:17" x14ac:dyDescent="0.25">
       <c r="F13" t="s">
         <v>343</v>
       </c>
@@ -3284,7 +3287,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:17" x14ac:dyDescent="0.25">
       <c r="F14" t="s">
         <v>344</v>
       </c>
@@ -3296,7 +3299,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:17" x14ac:dyDescent="0.25">
       <c r="F15" t="s">
         <v>121</v>
       </c>
@@ -3308,7 +3311,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:17" x14ac:dyDescent="0.25">
       <c r="F16" t="s">
         <v>345</v>
       </c>
@@ -3320,7 +3323,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="8:9" x14ac:dyDescent="0.3">
+    <row r="17" spans="8:9" x14ac:dyDescent="0.25">
       <c r="H17" s="30" t="s">
         <v>173</v>
       </c>
@@ -3329,7 +3332,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="8:9" x14ac:dyDescent="0.3">
+    <row r="18" spans="8:9" x14ac:dyDescent="0.25">
       <c r="H18" s="30" t="s">
         <v>174</v>
       </c>
@@ -3347,19 +3350,19 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:R11"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="2" width="9.6640625" style="13" customWidth="1"/>
-    <col min="3" max="3" width="15.88671875" customWidth="1"/>
-    <col min="4" max="5" width="11.5546875" customWidth="1"/>
+    <col min="1" max="2" width="9.7109375" style="13" customWidth="1"/>
+    <col min="3" max="3" width="15.85546875" customWidth="1"/>
+    <col min="4" max="5" width="11.5703125" customWidth="1"/>
     <col min="6" max="7" width="10" customWidth="1"/>
-    <col min="11" max="11" width="16.109375" customWidth="1"/>
+    <col min="11" max="11" width="16.140625" customWidth="1"/>
     <col min="13" max="13" width="7" customWidth="1"/>
-    <col min="16" max="16" width="6.5546875" customWidth="1"/>
-    <col min="17" max="17" width="4.6640625" customWidth="1"/>
+    <col min="16" max="16" width="6.5703125" customWidth="1"/>
+    <col min="17" max="17" width="4.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A1" s="11" t="s">
         <v>41</v>
       </c>
@@ -3367,7 +3370,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="2" spans="1:18" s="1" customFormat="1" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:18" s="1" customFormat="1" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="12" t="s">
         <v>3</v>
       </c>
@@ -3423,7 +3426,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A3" s="13" t="s">
         <v>12</v>
       </c>
@@ -3452,7 +3455,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A4" s="13" t="s">
         <v>12</v>
       </c>
@@ -3469,7 +3472,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A5" s="13" t="s">
         <v>15</v>
       </c>
@@ -3495,7 +3498,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A6" s="13" t="s">
         <v>18</v>
       </c>
@@ -3521,7 +3524,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A7" s="13" t="s">
         <v>22</v>
       </c>
@@ -3550,7 +3553,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A8" s="13" t="s">
         <v>25</v>
       </c>
@@ -3567,7 +3570,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A9" s="13" t="s">
         <v>25</v>
       </c>
@@ -3590,7 +3593,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A10" s="13" t="s">
         <v>28</v>
       </c>
@@ -3622,7 +3625,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A11" s="13" t="s">
         <v>31</v>
       </c>
@@ -3679,13 +3682,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{725EDE5F-2F74-4F10-B375-EE1EEF8AD52D}">
   <dimension ref="A1:M20"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="3" max="3" width="15.33203125" customWidth="1"/>
-    <col min="4" max="4" width="14.5546875" customWidth="1"/>
+    <col min="3" max="3" width="15.28515625" customWidth="1"/>
+    <col min="4" max="4" width="14.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" s="11" t="s">
         <v>41</v>
       </c>
@@ -3699,7 +3702,7 @@
         <v>382</v>
       </c>
     </row>
-    <row r="2" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="12" t="s">
         <v>3</v>
       </c>
@@ -3736,7 +3739,7 @@
       <c r="L2" s="1"/>
       <c r="M2" s="1"/>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" s="13" t="s">
         <v>12</v>
       </c>
@@ -3762,7 +3765,7 @@
         <v>385</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" s="13" t="s">
         <v>12</v>
       </c>
@@ -3785,11 +3788,11 @@
         <v>387</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" s="13"/>
       <c r="C5" s="4"/>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" s="13" t="s">
         <v>15</v>
       </c>
@@ -3815,7 +3818,7 @@
         <v>385</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" s="13" t="s">
         <v>15</v>
       </c>
@@ -3838,11 +3841,11 @@
         <v>387</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" s="13"/>
       <c r="C8" s="4"/>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" s="13" t="s">
         <v>18</v>
       </c>
@@ -3868,7 +3871,7 @@
         <v>385</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" s="13" t="s">
         <v>18</v>
       </c>
@@ -3891,11 +3894,11 @@
         <v>387</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" s="13"/>
       <c r="C11" s="4"/>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A12" s="13" t="s">
         <v>22</v>
       </c>
@@ -3904,11 +3907,11 @@
       </c>
       <c r="C12" s="4"/>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A13" s="13"/>
       <c r="C13" s="4"/>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A14" s="13" t="s">
         <v>25</v>
       </c>
@@ -3917,7 +3920,7 @@
       </c>
       <c r="C14" s="4"/>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A15" s="13" t="s">
         <v>25</v>
       </c>
@@ -3926,11 +3929,11 @@
       </c>
       <c r="C15" s="4"/>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A16" s="13"/>
       <c r="C16" s="4"/>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" s="13" t="s">
         <v>28</v>
       </c>
@@ -3959,7 +3962,7 @@
         <v>388</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" s="13" t="s">
         <v>28</v>
       </c>
@@ -3982,11 +3985,11 @@
         <v>387</v>
       </c>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" s="13"/>
       <c r="C19" s="4"/>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" s="13" t="s">
         <v>31</v>
       </c>
@@ -4024,19 +4027,19 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:O31"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.44140625" customWidth="1"/>
-    <col min="2" max="2" width="14.109375" customWidth="1"/>
-    <col min="3" max="3" width="14.5546875" customWidth="1"/>
+    <col min="1" max="1" width="11.42578125" customWidth="1"/>
+    <col min="2" max="2" width="14.140625" customWidth="1"/>
+    <col min="3" max="3" width="14.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>175</v>
       </c>
     </row>
-    <row r="2" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>176</v>
       </c>
@@ -4083,7 +4086,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>190</v>
       </c>
@@ -4118,7 +4121,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
         <v>45</v>
       </c>
@@ -4150,7 +4153,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
         <v>47</v>
       </c>
@@ -4182,7 +4185,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>198</v>
       </c>
@@ -4217,7 +4220,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>201</v>
       </c>
@@ -4252,7 +4255,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>203</v>
       </c>
@@ -4287,7 +4290,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
         <v>207</v>
       </c>
@@ -4312,7 +4315,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
         <v>209</v>
       </c>
@@ -4337,7 +4340,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>210</v>
       </c>
@@ -4372,7 +4375,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>211</v>
       </c>
@@ -4407,7 +4410,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>214</v>
       </c>
@@ -4442,7 +4445,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>77</v>
       </c>
@@ -4477,7 +4480,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>216</v>
       </c>
@@ -4512,7 +4515,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>219</v>
       </c>
@@ -4547,7 +4550,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>222</v>
       </c>
@@ -4572,17 +4575,17 @@
       <c r="I17" t="s">
         <v>194</v>
       </c>
-      <c r="K17" s="25" t="s">
-        <v>224</v>
+      <c r="K17" s="36" t="s">
+        <v>254</v>
       </c>
       <c r="L17" t="s">
         <v>195</v>
       </c>
       <c r="M17">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>225</v>
       </c>
@@ -4590,7 +4593,7 @@
         <v>46</v>
       </c>
       <c r="C18" t="s">
-        <v>226</v>
+        <v>394</v>
       </c>
       <c r="D18" t="s">
         <v>197</v>
@@ -4617,7 +4620,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>227</v>
       </c>
@@ -4652,7 +4655,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>229</v>
       </c>
@@ -4687,7 +4690,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>231</v>
       </c>
@@ -4725,7 +4728,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>236</v>
       </c>
@@ -4754,7 +4757,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>238</v>
       </c>
@@ -4789,7 +4792,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>242</v>
       </c>
@@ -4820,7 +4823,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>245</v>
       </c>
@@ -4855,7 +4858,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B26" t="s">
         <v>57</v>
       </c>
@@ -4875,7 +4878,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B27" t="s">
         <v>381</v>
       </c>
@@ -4901,7 +4904,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B28" t="s">
         <v>247</v>
       </c>
@@ -4927,7 +4930,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>248</v>
       </c>
@@ -4956,7 +4959,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>250</v>
       </c>
@@ -4985,7 +4988,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B31" t="s">
         <v>252</v>
       </c>
@@ -5025,13 +5028,13 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:M17"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
-    <col min="6" max="6" width="15.5546875" customWidth="1"/>
+    <col min="6" max="6" width="15.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" s="2"/>
       <c r="B1" s="2" t="s">
         <v>112</v>
@@ -5048,7 +5051,7 @@
       <c r="I1" s="2"/>
       <c r="K1" s="2"/>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>115</v>
       </c>
@@ -5089,7 +5092,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>125</v>
       </c>
@@ -5115,7 +5118,7 @@
         <v>-18877.708702820371</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>131</v>
       </c>
@@ -5141,7 +5144,7 @@
         <v>-19045.139985898601</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>133</v>
       </c>
@@ -5167,7 +5170,7 @@
         <v>-5.4445188599886638</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>135</v>
       </c>
@@ -5193,7 +5196,7 @@
         <v>2.671411511624413</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>137</v>
       </c>
@@ -5219,7 +5222,7 @@
         <v>9.5532474786010475</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>125</v>
       </c>
@@ -5245,7 +5248,7 @@
         <v>2866.0938229725748</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>131</v>
       </c>
@@ -5271,7 +5274,7 @@
         <v>1490.761502865475</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>133</v>
       </c>
@@ -5297,7 +5300,7 @@
         <v>2.217459469264154</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>135</v>
       </c>
@@ -5323,7 +5326,7 @@
         <v>0.2337935274525294</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>137</v>
       </c>
@@ -5349,7 +5352,7 @@
         <v>2.0873115011979051E-2</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>125</v>
       </c>
@@ -5375,7 +5378,7 @@
         <v>1351.711647219304</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>131</v>
       </c>
@@ -5401,7 +5404,7 @@
         <v>150.9391394665019</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>133</v>
       </c>
@@ -5427,7 +5430,7 @@
         <v>1.940117188288828</v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>135</v>
       </c>
@@ -5453,7 +5456,7 @@
         <v>-2.0146865510893688E-2</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>137</v>
       </c>
@@ -5487,22 +5490,22 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:G42"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="3" max="3" width="16.6640625" customWidth="1"/>
+    <col min="3" max="3" width="16.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>153</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="5" spans="1:7" s="1" customFormat="1" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" s="1" customFormat="1" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>2</v>
       </c>
@@ -5525,7 +5528,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
         <v>12</v>
       </c>
@@ -5545,7 +5548,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="7" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
         <v>12</v>
       </c>
@@ -5562,7 +5565,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="8" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
         <v>12</v>
       </c>
@@ -5579,7 +5582,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="9" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
         <v>12</v>
       </c>
@@ -5596,7 +5599,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="10" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
         <v>12</v>
       </c>
@@ -5613,7 +5616,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="11" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
         <v>12</v>
       </c>
@@ -5630,7 +5633,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
         <v>12</v>
       </c>
@@ -5647,7 +5650,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B13" t="s">
         <v>15</v>
       </c>
@@ -5664,7 +5667,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="14" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="B14" t="s">
         <v>15</v>
       </c>
@@ -5681,7 +5684,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="15" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="B15" t="s">
         <v>15</v>
       </c>
@@ -5698,7 +5701,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="16" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="B16" t="s">
         <v>15</v>
       </c>
@@ -5715,7 +5718,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="17" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B17" t="s">
         <v>15</v>
       </c>
@@ -5732,7 +5735,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="18" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B18" t="s">
         <v>15</v>
       </c>
@@ -5749,7 +5752,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="19" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B19" t="s">
         <v>15</v>
       </c>
@@ -5766,7 +5769,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="20" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B20" t="s">
         <v>18</v>
       </c>
@@ -5783,7 +5786,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="21" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B21" t="s">
         <v>18</v>
       </c>
@@ -5800,7 +5803,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="22" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B22" t="s">
         <v>18</v>
       </c>
@@ -5817,7 +5820,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="23" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B23" t="s">
         <v>18</v>
       </c>
@@ -5834,7 +5837,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="24" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B24" t="s">
         <v>18</v>
       </c>
@@ -5851,7 +5854,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="25" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B25" t="s">
         <v>18</v>
       </c>
@@ -5868,7 +5871,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="26" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B26" t="s">
         <v>18</v>
       </c>
@@ -5885,7 +5888,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="27" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B27" t="s">
         <v>28</v>
       </c>
@@ -5902,7 +5905,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="28" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B28" t="s">
         <v>28</v>
       </c>
@@ -5919,7 +5922,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="29" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B29" t="s">
         <v>28</v>
       </c>
@@ -5936,7 +5939,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="30" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B30" t="s">
         <v>28</v>
       </c>
@@ -5953,7 +5956,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="31" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B31" t="s">
         <v>28</v>
       </c>
@@ -5970,7 +5973,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="32" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B32" t="s">
         <v>28</v>
       </c>
@@ -5987,7 +5990,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="33" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B33" t="s">
         <v>28</v>
       </c>
@@ -6004,7 +6007,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="34" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="34" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B34" t="s">
         <v>31</v>
       </c>
@@ -6021,7 +6024,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="35" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="35" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B35" t="s">
         <v>31</v>
       </c>
@@ -6038,7 +6041,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="36" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="36" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B36" t="s">
         <v>31</v>
       </c>
@@ -6055,7 +6058,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="37" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="37" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B37" t="s">
         <v>31</v>
       </c>
@@ -6072,7 +6075,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="38" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="38" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B38" t="s">
         <v>31</v>
       </c>
@@ -6089,7 +6092,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="39" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="39" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B39" t="s">
         <v>31</v>
       </c>
@@ -6106,7 +6109,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="40" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="40" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B40" t="s">
         <v>31</v>
       </c>
@@ -6123,7 +6126,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="41" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="41" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B41" t="s">
         <v>31</v>
       </c>
@@ -6140,7 +6143,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="42" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="42" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B42" t="s">
         <v>31</v>
       </c>
@@ -6174,19 +6177,19 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9DE0C751-ACC1-462A-82AF-4CE9BB91C06B}">
   <dimension ref="A2:G21"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C4" t="s">
         <v>393</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>2</v>
       </c>
@@ -6209,7 +6212,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>21</v>
       </c>
@@ -6223,7 +6226,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>11</v>
       </c>
@@ -6237,7 +6240,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>11</v>
       </c>
@@ -6251,7 +6254,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>11</v>
       </c>
@@ -6265,7 +6268,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>11</v>
       </c>
@@ -6279,7 +6282,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>11</v>
       </c>
@@ -6293,7 +6296,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>21</v>
       </c>
@@ -6307,9 +6310,9 @@
         <v>224</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="B13" s="30" t="s">
         <v>165</v>
@@ -6321,9 +6324,9 @@
         <v>19</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="B14" s="30" t="s">
         <v>167</v>
@@ -6335,9 +6338,9 @@
         <v>23</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="B15" s="30" t="s">
         <v>168</v>
@@ -6349,9 +6352,9 @@
         <v>212</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="B16" s="30" t="s">
         <v>169</v>
@@ -6363,9 +6366,9 @@
         <v>37</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="B17" s="30" t="s">
         <v>170</v>
@@ -6377,9 +6380,9 @@
         <v>39</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="B18" s="30" t="s">
         <v>171</v>
@@ -6391,9 +6394,9 @@
         <v>218</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="B19" s="30" t="s">
         <v>172</v>
@@ -6405,9 +6408,9 @@
         <v>221</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="B20" s="30" t="s">
         <v>173</v>
@@ -6419,9 +6422,9 @@
         <v>224</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="B21" s="30" t="s">
         <v>174</v>
@@ -6449,25 +6452,25 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:O8"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8.5546875" customWidth="1"/>
+    <col min="1" max="1" width="8.5703125" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
-    <col min="3" max="3" width="12.88671875" customWidth="1"/>
+    <col min="3" max="3" width="12.85546875" customWidth="1"/>
     <col min="4" max="4" width="10" customWidth="1"/>
-    <col min="6" max="6" width="6.6640625" customWidth="1"/>
-    <col min="7" max="7" width="6.5546875" customWidth="1"/>
-    <col min="8" max="8" width="8.33203125" customWidth="1"/>
-    <col min="9" max="9" width="5.5546875" customWidth="1"/>
-    <col min="10" max="10" width="6.5546875" customWidth="1"/>
-    <col min="11" max="11" width="6.109375" customWidth="1"/>
-    <col min="12" max="12" width="5.109375" customWidth="1"/>
-    <col min="13" max="13" width="5.5546875" customWidth="1"/>
-    <col min="14" max="14" width="5.109375" customWidth="1"/>
-    <col min="15" max="15" width="4.44140625" customWidth="1"/>
+    <col min="6" max="6" width="6.7109375" customWidth="1"/>
+    <col min="7" max="7" width="6.5703125" customWidth="1"/>
+    <col min="8" max="8" width="8.28515625" customWidth="1"/>
+    <col min="9" max="9" width="5.5703125" customWidth="1"/>
+    <col min="10" max="10" width="6.5703125" customWidth="1"/>
+    <col min="11" max="11" width="6.140625" customWidth="1"/>
+    <col min="12" max="12" width="5.140625" customWidth="1"/>
+    <col min="13" max="13" width="5.5703125" customWidth="1"/>
+    <col min="14" max="14" width="5.140625" customWidth="1"/>
+    <col min="15" max="15" width="4.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>255</v>
       </c>
@@ -6475,7 +6478,7 @@
         <v>256</v>
       </c>
     </row>
-    <row r="2" spans="1:15" s="8" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:15" s="8" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="8" t="s">
         <v>257</v>
       </c>
@@ -6522,7 +6525,7 @@
         <v>271</v>
       </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>272</v>
       </c>
@@ -6562,7 +6565,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>275</v>
       </c>
@@ -6577,19 +6580,19 @@
         <v>276</v>
       </c>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B5" s="3"/>
       <c r="C5" s="3"/>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B7" s="3"/>
       <c r="C7" s="3"/>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B8" s="3"/>
       <c r="C8" s="3"/>
     </row>
@@ -6608,13 +6611,13 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
   <dimension ref="A1:H21"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="4" width="10.33203125" customWidth="1"/>
-    <col min="5" max="6" width="8.5546875" customWidth="1"/>
+    <col min="2" max="4" width="10.28515625" customWidth="1"/>
+    <col min="5" max="6" width="8.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -6622,7 +6625,7 @@
         <v>277</v>
       </c>
     </row>
-    <row r="2" spans="1:8" s="8" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:8" s="8" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
@@ -6648,7 +6651,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:8" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="31" t="s">
         <v>21</v>
       </c>
@@ -6663,7 +6666,7 @@
       </c>
       <c r="G3" s="32"/>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>21</v>
       </c>
@@ -6689,7 +6692,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>21</v>
       </c>
@@ -6715,7 +6718,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:8" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="31" t="s">
         <v>21</v>
       </c>
@@ -6739,7 +6742,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>11</v>
       </c>
@@ -6765,7 +6768,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>11</v>
       </c>
@@ -6791,7 +6794,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="31" t="s">
         <v>11</v>
       </c>
@@ -6815,7 +6818,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="21" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="21" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H21" t="s">
         <v>287</v>
       </c>

</xml_diff>

<commit_message>
Ongoing work on building an interactive cross_plotter.py
</commit_message>
<xml_diff>
--- a/excels/project_table_new.xlsx
+++ b/excels/project_table_new.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marte\PycharmProjects\blixt_rp\excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B569FA14-30A6-4A63-8194-BCD6B539ECE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43F48BFA-352F-47DA-A5F7-C50A78A1105D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4950" yWindow="1455" windowWidth="21600" windowHeight="13440" tabRatio="685" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="780" yWindow="780" windowWidth="21600" windowHeight="11295" tabRatio="685" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Well settings" sheetId="1" r:id="rId1"/>
@@ -2044,7 +2044,7 @@
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="B4" s="13" t="s">
         <v>15</v>
@@ -2058,7 +2058,7 @@
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="B5" s="13" t="s">
         <v>18</v>

</xml_diff>

<commit_message>
Moved log_plotter.py to blixt_rp Ongoing work to create a cross_plotter.py
</commit_message>
<xml_diff>
--- a/excels/project_table_new.xlsx
+++ b/excels/project_table_new.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marte\PycharmProjects\blixt_rp\excels\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\emb\Documents\PycharmProjects\blixt_rp\excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43F48BFA-352F-47DA-A5F7-C50A78A1105D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D0D9EB2-1CD8-4A9B-B628-D4C9ACB0E881}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="780" yWindow="780" windowWidth="21600" windowHeight="11295" tabRatio="685" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="6840" yWindow="1410" windowWidth="28800" windowHeight="17145" tabRatio="685" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Well settings" sheetId="1" r:id="rId1"/>
@@ -63,7 +63,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="976" uniqueCount="395">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="978" uniqueCount="395">
   <si>
     <t>Select Yes or No</t>
   </si>
@@ -744,9 +744,6 @@
   </si>
   <si>
     <t>AC,DT</t>
-  </si>
-  <si>
-    <t>$\mu s/F$</t>
   </si>
   <si>
     <t>ACS,DTS</t>
@@ -1257,6 +1254,9 @@
   </si>
   <si>
     <t>us / F</t>
+  </si>
+  <si>
+    <t>PENOBSCOTL_30</t>
   </si>
 </sst>
 </file>
@@ -2136,7 +2136,12 @@
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B10" s="13"/>
+      <c r="A10" t="s">
+        <v>21</v>
+      </c>
+      <c r="B10" s="13" t="s">
+        <v>394</v>
+      </c>
       <c r="C10" s="20" t="s">
         <v>23</v>
       </c>
@@ -2192,35 +2197,35 @@
   <sheetData>
     <row r="1" spans="1:7" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F1" s="7" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="2" spans="1:7" s="8" customFormat="1" ht="30.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="33" t="s">
+        <v>256</v>
+      </c>
+      <c r="B2" s="34" t="s">
         <v>257</v>
       </c>
-      <c r="B2" s="34" t="s">
+      <c r="C2" s="34" t="s">
         <v>258</v>
       </c>
-      <c r="C2" s="34" t="s">
+      <c r="D2" s="34" t="s">
         <v>259</v>
       </c>
-      <c r="D2" s="34" t="s">
+      <c r="E2" s="33" t="s">
+        <v>288</v>
+      </c>
+      <c r="F2" s="33" t="s">
         <v>260</v>
       </c>
-      <c r="E2" s="33" t="s">
+      <c r="G2" s="33" t="s">
         <v>289</v>
-      </c>
-      <c r="F2" s="33" t="s">
-        <v>261</v>
-      </c>
-      <c r="G2" s="33" t="s">
-        <v>290</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="B3">
         <v>36.6</v>
@@ -2237,7 +2242,7 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B4">
         <v>11.4</v>
@@ -2252,15 +2257,15 @@
         <v>0</v>
       </c>
       <c r="F4" t="s">
+        <v>292</v>
+      </c>
+      <c r="G4" t="s">
         <v>293</v>
-      </c>
-      <c r="G4" t="s">
-        <v>294</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="B5">
         <v>76.8</v>
@@ -2277,7 +2282,7 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="B6">
         <v>94.9</v>
@@ -2294,7 +2299,7 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="B7">
         <v>26</v>
@@ -2311,7 +2316,7 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="B8">
         <v>47</v>
@@ -2328,7 +2333,7 @@
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="B9">
         <v>114</v>
@@ -2345,7 +2350,7 @@
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="B10">
         <v>55</v>
@@ -2362,7 +2367,7 @@
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="B11">
         <v>48</v>
@@ -2379,7 +2384,7 @@
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="B12">
         <v>85</v>
@@ -2396,7 +2401,7 @@
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="B13">
         <v>52</v>
@@ -2413,7 +2418,7 @@
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="B14">
         <v>50</v>
@@ -2430,7 +2435,7 @@
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="B15">
         <v>25.2</v>
@@ -2447,7 +2452,7 @@
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="B16">
         <v>66.5</v>
@@ -2464,7 +2469,7 @@
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="B17">
         <v>58</v>
@@ -2481,7 +2486,7 @@
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="B18">
         <v>158</v>
@@ -2498,7 +2503,7 @@
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="B19">
         <v>27</v>
@@ -2515,7 +2520,7 @@
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="B20">
         <v>123.7</v>
@@ -2532,7 +2537,7 @@
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="B21">
         <v>15</v>
@@ -2549,7 +2554,7 @@
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="B22">
         <v>17.96</v>
@@ -2566,7 +2571,7 @@
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="B23">
         <v>55.8</v>
@@ -2583,7 +2588,7 @@
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="B24">
         <v>87</v>
@@ -2600,7 +2605,7 @@
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="B25">
         <v>103.67</v>
@@ -2617,7 +2622,7 @@
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="B26">
         <v>129.13999999999999</v>
@@ -2634,7 +2639,7 @@
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="B27">
         <v>4.5199999999999996</v>
@@ -2651,7 +2656,7 @@
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="B28">
         <v>160.29</v>
@@ -2668,7 +2673,7 @@
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="B29">
         <v>62.2</v>
@@ -2685,7 +2690,7 @@
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="B30">
         <v>146.25</v>
@@ -2702,7 +2707,7 @@
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="B31">
         <v>48.35</v>
@@ -2719,7 +2724,7 @@
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="B32">
         <v>2.9</v>
@@ -2736,7 +2741,7 @@
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="B33">
         <v>12.3</v>
@@ -2769,21 +2774,21 @@
   <sheetData>
     <row r="1" spans="1:4" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D1" s="5" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
     </row>
     <row r="2" spans="1:4" s="8" customFormat="1" ht="30.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="9" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="B2" s="9" t="s">
         <v>116</v>
       </c>
       <c r="C2" s="8" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="D2" s="10" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -2794,10 +2799,10 @@
         <v>162</v>
       </c>
       <c r="C3" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -2808,7 +2813,7 @@
         <v>162</v>
       </c>
       <c r="C4" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="D4" t="s">
         <v>64</v>
@@ -2861,49 +2866,49 @@
       <c r="J1" s="2"/>
       <c r="K1" s="2"/>
       <c r="L1" s="2" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="M1" s="2" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="O1" s="2"/>
     </row>
     <row r="2" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>362</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>369</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>370</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>371</v>
+      </c>
+      <c r="F2" s="1" t="s">
         <v>363</v>
       </c>
-      <c r="C2" s="1" t="s">
-        <v>370</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>371</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>372</v>
-      </c>
-      <c r="F2" s="1" t="s">
+      <c r="G2" s="1" t="s">
         <v>364</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="H2" s="1" t="s">
         <v>365</v>
-      </c>
-      <c r="H2" s="1" t="s">
-        <v>366</v>
       </c>
       <c r="I2" s="1" t="s">
         <v>157</v>
       </c>
       <c r="J2" s="1" t="s">
+        <v>366</v>
+      </c>
+      <c r="K2" s="1" t="s">
         <v>367</v>
       </c>
-      <c r="K2" s="1" t="s">
+      <c r="L2" s="1" t="s">
         <v>368</v>
-      </c>
-      <c r="L2" s="1" t="s">
-        <v>369</v>
       </c>
       <c r="M2" s="1" t="s">
         <v>8</v>
@@ -2926,7 +2931,7 @@
     <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" s="2"/>
       <c r="B1" s="2" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="C1" s="2"/>
       <c r="D1" s="2"/>
@@ -2938,22 +2943,22 @@
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>99</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="D2" s="1" t="s">
+        <v>375</v>
+      </c>
+      <c r="E2" s="1" t="s">
         <v>376</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="F2" s="1" t="s">
         <v>377</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>378</v>
       </c>
       <c r="G2" s="1"/>
       <c r="H2" s="1"/>
@@ -2991,57 +2996,57 @@
   <sheetData>
     <row r="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="H1" s="2" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
     </row>
     <row r="2" spans="1:17" s="6" customFormat="1" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2" s="6" t="s">
+        <v>325</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>269</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>277</v>
+      </c>
+      <c r="E2" t="s">
         <v>326</v>
       </c>
-      <c r="C2" s="6" t="s">
-        <v>270</v>
-      </c>
-      <c r="D2" s="6" t="s">
-        <v>278</v>
-      </c>
-      <c r="E2" t="s">
+      <c r="F2" s="6" t="s">
         <v>327</v>
       </c>
-      <c r="F2" s="6" t="s">
+      <c r="G2" s="6" t="s">
         <v>328</v>
-      </c>
-      <c r="G2" s="6" t="s">
-        <v>329</v>
       </c>
       <c r="H2" s="1" t="s">
         <v>116</v>
       </c>
       <c r="I2" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="J2" s="6" t="s">
+        <v>329</v>
+      </c>
+      <c r="K2" t="s">
         <v>330</v>
       </c>
-      <c r="K2" t="s">
+      <c r="L2" t="s">
         <v>331</v>
       </c>
-      <c r="L2" t="s">
+      <c r="M2" t="s">
         <v>332</v>
       </c>
-      <c r="M2" t="s">
+      <c r="N2" t="s">
         <v>333</v>
-      </c>
-      <c r="N2" t="s">
-        <v>334</v>
       </c>
       <c r="O2" t="s">
         <v>102</v>
       </c>
       <c r="P2" t="s">
+        <v>348</v>
+      </c>
+      <c r="Q2" t="s">
         <v>349</v>
-      </c>
-      <c r="Q2" t="s">
-        <v>350</v>
       </c>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.25">
@@ -3049,16 +3054,16 @@
         <v>11</v>
       </c>
       <c r="B3" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="C3" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="D3" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="E3" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="F3" t="s">
         <v>14</v>
@@ -3074,16 +3079,16 @@
         <v>4</v>
       </c>
       <c r="J3" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="K3" t="s">
+        <v>335</v>
+      </c>
+      <c r="L3" t="s">
         <v>336</v>
       </c>
-      <c r="L3" t="s">
+      <c r="M3" t="s">
         <v>337</v>
-      </c>
-      <c r="M3" t="s">
-        <v>338</v>
       </c>
       <c r="N3" t="s">
         <v>128</v>
@@ -3092,10 +3097,10 @@
         <v>106</v>
       </c>
       <c r="P3" t="s">
+        <v>350</v>
+      </c>
+      <c r="Q3" t="s">
         <v>351</v>
-      </c>
-      <c r="Q3" t="s">
-        <v>352</v>
       </c>
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.25">
@@ -3103,16 +3108,16 @@
         <v>21</v>
       </c>
       <c r="B4" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="C4" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="D4" t="s">
+        <v>282</v>
+      </c>
+      <c r="E4" t="s">
         <v>283</v>
-      </c>
-      <c r="E4" t="s">
-        <v>284</v>
       </c>
       <c r="F4" t="s">
         <v>17</v>
@@ -3128,36 +3133,36 @@
         <v>4</v>
       </c>
       <c r="J4" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="K4" t="s">
         <v>103</v>
       </c>
       <c r="L4" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="M4" t="s">
         <v>105</v>
       </c>
       <c r="O4" t="s">
+        <v>352</v>
+      </c>
+      <c r="P4" t="s">
         <v>353</v>
       </c>
-      <c r="P4" t="s">
+      <c r="Q4" t="s">
         <v>354</v>
-      </c>
-      <c r="Q4" t="s">
-        <v>355</v>
       </c>
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.25">
       <c r="E5" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="F5" t="s">
         <v>20</v>
       </c>
       <c r="G5" s="13" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="H5" t="s">
         <v>161</v>
@@ -3170,10 +3175,10 @@
         <v>105</v>
       </c>
       <c r="O5" t="s">
+        <v>355</v>
+      </c>
+      <c r="Q5" t="s">
         <v>356</v>
-      </c>
-      <c r="Q5" t="s">
-        <v>357</v>
       </c>
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.25">
@@ -3181,7 +3186,7 @@
         <v>27</v>
       </c>
       <c r="G6" s="13" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="H6" t="s">
         <v>162</v>
@@ -3191,10 +3196,10 @@
         <v>4</v>
       </c>
       <c r="O6" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="Q6" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
     </row>
     <row r="7" spans="1:17" x14ac:dyDescent="0.25">
@@ -3209,10 +3214,10 @@
         <v>4</v>
       </c>
       <c r="O7" t="s">
+        <v>358</v>
+      </c>
+      <c r="Q7" t="s">
         <v>359</v>
-      </c>
-      <c r="Q7" t="s">
-        <v>360</v>
       </c>
     </row>
     <row r="8" spans="1:17" x14ac:dyDescent="0.25">
@@ -3277,7 +3282,7 @@
     </row>
     <row r="13" spans="1:17" x14ac:dyDescent="0.25">
       <c r="F13" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="H13" s="30" t="s">
         <v>169</v>
@@ -3289,7 +3294,7 @@
     </row>
     <row r="14" spans="1:17" x14ac:dyDescent="0.25">
       <c r="F14" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="H14" s="30" t="s">
         <v>170</v>
@@ -3313,7 +3318,7 @@
     </row>
     <row r="16" spans="1:17" x14ac:dyDescent="0.25">
       <c r="F16" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="H16" s="30" t="s">
         <v>172</v>
@@ -3699,7 +3704,7 @@
         <v>98</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
     </row>
     <row r="2" spans="1:13" ht="30" x14ac:dyDescent="0.25">
@@ -3719,19 +3724,19 @@
         <v>102</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="K2" s="1" t="s">
         <v>10</v>
@@ -3756,13 +3761,13 @@
         <v>106</v>
       </c>
       <c r="F3" t="s">
+        <v>382</v>
+      </c>
+      <c r="G3" t="s">
         <v>383</v>
       </c>
-      <c r="G3" t="s">
+      <c r="H3" t="s">
         <v>384</v>
-      </c>
-      <c r="H3" t="s">
-        <v>385</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
@@ -3782,10 +3787,10 @@
         <v>106</v>
       </c>
       <c r="G4" t="s">
+        <v>385</v>
+      </c>
+      <c r="I4" t="s">
         <v>386</v>
-      </c>
-      <c r="I4" t="s">
-        <v>387</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
@@ -3809,13 +3814,13 @@
         <v>106</v>
       </c>
       <c r="F6" t="s">
+        <v>382</v>
+      </c>
+      <c r="G6" t="s">
         <v>383</v>
       </c>
-      <c r="G6" t="s">
+      <c r="H6" t="s">
         <v>384</v>
-      </c>
-      <c r="H6" t="s">
-        <v>385</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
@@ -3835,10 +3840,10 @@
         <v>106</v>
       </c>
       <c r="G7" t="s">
+        <v>385</v>
+      </c>
+      <c r="I7" t="s">
         <v>386</v>
-      </c>
-      <c r="I7" t="s">
-        <v>387</v>
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.25">
@@ -3862,13 +3867,13 @@
         <v>106</v>
       </c>
       <c r="F9" t="s">
+        <v>382</v>
+      </c>
+      <c r="G9" t="s">
         <v>383</v>
       </c>
-      <c r="G9" t="s">
+      <c r="H9" t="s">
         <v>384</v>
-      </c>
-      <c r="H9" t="s">
-        <v>385</v>
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.25">
@@ -3888,10 +3893,10 @@
         <v>106</v>
       </c>
       <c r="G10" t="s">
+        <v>385</v>
+      </c>
+      <c r="I10" t="s">
         <v>386</v>
-      </c>
-      <c r="I10" t="s">
-        <v>387</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.25">
@@ -3950,16 +3955,16 @@
         <v>106</v>
       </c>
       <c r="F17" t="s">
+        <v>382</v>
+      </c>
+      <c r="G17" t="s">
         <v>383</v>
       </c>
-      <c r="G17" t="s">
+      <c r="H17" t="s">
         <v>384</v>
       </c>
-      <c r="H17" t="s">
-        <v>385</v>
-      </c>
       <c r="K17" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.25">
@@ -3979,10 +3984,10 @@
         <v>106</v>
       </c>
       <c r="G18" t="s">
+        <v>385</v>
+      </c>
+      <c r="I18" t="s">
         <v>386</v>
-      </c>
-      <c r="I18" t="s">
-        <v>387</v>
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.25">
@@ -4080,7 +4085,7 @@
         <v>188</v>
       </c>
       <c r="N2" s="1" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="O2" s="1" t="s">
         <v>189</v>
@@ -4228,7 +4233,7 @@
         <v>202</v>
       </c>
       <c r="C7" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="D7" t="s">
         <v>197</v>
@@ -4348,7 +4353,7 @@
         <v>52</v>
       </c>
       <c r="C11" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="D11" t="s">
         <v>197</v>
@@ -4383,7 +4388,7 @@
         <v>53</v>
       </c>
       <c r="C12" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="D12" t="s">
         <v>197</v>
@@ -4418,7 +4423,7 @@
         <v>54</v>
       </c>
       <c r="C13" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="D13" t="s">
         <v>197</v>
@@ -4576,7 +4581,7 @@
         <v>194</v>
       </c>
       <c r="K17" s="36" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="L17" t="s">
         <v>195</v>
@@ -4593,7 +4598,7 @@
         <v>46</v>
       </c>
       <c r="C18" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="D18" t="s">
         <v>197</v>
@@ -4622,13 +4627,13 @@
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
+        <v>226</v>
+      </c>
+      <c r="B19" t="s">
         <v>227</v>
       </c>
-      <c r="B19" t="s">
-        <v>228</v>
-      </c>
       <c r="C19" t="s">
-        <v>226</v>
+        <v>393</v>
       </c>
       <c r="D19" t="s">
         <v>197</v>
@@ -4657,13 +4662,13 @@
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
+        <v>228</v>
+      </c>
+      <c r="B20" t="s">
+        <v>228</v>
+      </c>
+      <c r="C20" t="s">
         <v>229</v>
-      </c>
-      <c r="B20" t="s">
-        <v>229</v>
-      </c>
-      <c r="C20" t="s">
-        <v>230</v>
       </c>
       <c r="D20" t="s">
         <v>197</v>
@@ -4692,16 +4697,16 @@
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
+        <v>230</v>
+      </c>
+      <c r="B21" t="s">
         <v>231</v>
       </c>
-      <c r="B21" t="s">
+      <c r="C21" t="s">
+        <v>229</v>
+      </c>
+      <c r="D21" t="s">
         <v>232</v>
-      </c>
-      <c r="C21" t="s">
-        <v>230</v>
-      </c>
-      <c r="D21" t="s">
-        <v>233</v>
       </c>
       <c r="E21" t="s">
         <v>193</v>
@@ -4713,10 +4718,10 @@
         <v>5</v>
       </c>
       <c r="I21" t="s">
+        <v>233</v>
+      </c>
+      <c r="J21" t="s">
         <v>234</v>
-      </c>
-      <c r="J21" t="s">
-        <v>235</v>
       </c>
       <c r="K21" s="19" t="s">
         <v>206</v>
@@ -4730,13 +4735,13 @@
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
+        <v>235</v>
+      </c>
+      <c r="B22" t="s">
         <v>236</v>
       </c>
-      <c r="B22" t="s">
-        <v>237</v>
-      </c>
       <c r="C22" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="D22" t="s">
         <v>197</v>
@@ -4759,16 +4764,16 @@
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
+        <v>237</v>
+      </c>
+      <c r="B23" t="s">
         <v>238</v>
       </c>
-      <c r="B23" t="s">
-        <v>239</v>
-      </c>
       <c r="C23" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="D23" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="F23" s="3">
         <v>0</v>
@@ -4777,10 +4782,10 @@
         <v>0.5</v>
       </c>
       <c r="I23" t="s">
+        <v>239</v>
+      </c>
+      <c r="J23" t="s">
         <v>240</v>
-      </c>
-      <c r="J23" t="s">
-        <v>241</v>
       </c>
       <c r="K23" s="21" t="s">
         <v>35</v>
@@ -4794,13 +4799,13 @@
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
+        <v>241</v>
+      </c>
+      <c r="B24" t="s">
         <v>242</v>
       </c>
-      <c r="B24" t="s">
+      <c r="C24" t="s">
         <v>243</v>
-      </c>
-      <c r="C24" t="s">
-        <v>244</v>
       </c>
       <c r="D24" t="s">
         <v>197</v>
@@ -4825,10 +4830,10 @@
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
+        <v>244</v>
+      </c>
+      <c r="B25" t="s">
         <v>245</v>
-      </c>
-      <c r="B25" t="s">
-        <v>246</v>
       </c>
       <c r="C25" t="s">
         <v>220</v>
@@ -4880,7 +4885,7 @@
     </row>
     <row r="27" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B27" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="C27" t="s">
         <v>1</v>
@@ -4895,7 +4900,7 @@
         <v>194</v>
       </c>
       <c r="K27" s="36" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="L27" t="s">
         <v>213</v>
@@ -4906,7 +4911,7 @@
     </row>
     <row r="28" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B28" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="C28" t="s">
         <v>1</v>
@@ -4932,10 +4937,10 @@
     </row>
     <row r="29" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
+        <v>247</v>
+      </c>
+      <c r="B29" t="s">
         <v>248</v>
-      </c>
-      <c r="B29" t="s">
-        <v>249</v>
       </c>
       <c r="C29" t="s">
         <v>17</v>
@@ -4961,10 +4966,10 @@
     </row>
     <row r="30" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
+        <v>249</v>
+      </c>
+      <c r="B30" t="s">
         <v>250</v>
-      </c>
-      <c r="B30" t="s">
-        <v>251</v>
       </c>
       <c r="C30" t="s">
         <v>17</v>
@@ -4990,10 +4995,10 @@
     </row>
     <row r="31" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B31" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="C31" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="D31" t="s">
         <v>197</v>
@@ -5002,10 +5007,10 @@
         <v>193</v>
       </c>
       <c r="I31" t="s">
+        <v>252</v>
+      </c>
+      <c r="K31" s="36" t="s">
         <v>253</v>
-      </c>
-      <c r="K31" s="36" t="s">
-        <v>254</v>
       </c>
       <c r="L31" t="s">
         <v>195</v>
@@ -6186,7 +6191,7 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C4" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
@@ -6194,13 +6199,13 @@
         <v>2</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="C5" s="12" t="s">
+        <v>390</v>
+      </c>
+      <c r="D5" s="1" t="s">
         <v>391</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>392</v>
       </c>
       <c r="E5" s="1" t="s">
         <v>157</v>
@@ -6472,67 +6477,67 @@
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="E1" s="7" t="s">
         <v>255</v>
-      </c>
-      <c r="E1" s="7" t="s">
-        <v>256</v>
       </c>
     </row>
     <row r="2" spans="1:15" s="8" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="8" t="s">
+        <v>256</v>
+      </c>
+      <c r="B2" s="9" t="s">
         <v>257</v>
       </c>
-      <c r="B2" s="9" t="s">
+      <c r="C2" s="9" t="s">
         <v>258</v>
       </c>
-      <c r="C2" s="9" t="s">
+      <c r="D2" s="9" t="s">
         <v>259</v>
       </c>
-      <c r="D2" s="9" t="s">
+      <c r="E2" s="8" t="s">
         <v>260</v>
       </c>
-      <c r="E2" s="8" t="s">
+      <c r="F2" s="8" t="s">
         <v>261</v>
       </c>
-      <c r="F2" s="8" t="s">
+      <c r="G2" s="8" t="s">
         <v>262</v>
       </c>
-      <c r="G2" s="8" t="s">
+      <c r="H2" s="8" t="s">
         <v>263</v>
       </c>
-      <c r="H2" s="8" t="s">
+      <c r="I2" s="8" t="s">
         <v>264</v>
       </c>
-      <c r="I2" s="8" t="s">
+      <c r="J2" s="8" t="s">
         <v>265</v>
       </c>
-      <c r="J2" s="8" t="s">
+      <c r="K2" s="8" t="s">
         <v>266</v>
       </c>
-      <c r="K2" s="8" t="s">
+      <c r="L2" s="8" t="s">
         <v>267</v>
       </c>
-      <c r="L2" s="8" t="s">
+      <c r="M2" s="8" t="s">
         <v>268</v>
       </c>
-      <c r="M2" s="8" t="s">
+      <c r="N2" s="8" t="s">
         <v>269</v>
       </c>
-      <c r="N2" s="8" t="s">
+      <c r="O2" s="8" t="s">
         <v>270</v>
-      </c>
-      <c r="O2" s="8" t="s">
-        <v>271</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="B3" s="3"/>
       <c r="C3" s="3"/>
       <c r="E3" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="F3">
         <v>0.03</v>
@@ -6559,7 +6564,7 @@
         <v>0.6</v>
       </c>
       <c r="N3" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="O3">
         <v>2</v>
@@ -6567,7 +6572,7 @@
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="B4" s="3">
         <v>2.68</v>
@@ -6577,7 +6582,7 @@
         <v>1.0229999999999999</v>
       </c>
       <c r="E4" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
@@ -6622,7 +6627,7 @@
         <v>0</v>
       </c>
       <c r="G1" s="7" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="2" spans="1:8" s="8" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -6630,25 +6635,25 @@
         <v>2</v>
       </c>
       <c r="B2" s="9" t="s">
+        <v>277</v>
+      </c>
+      <c r="C2" s="9" t="s">
         <v>278</v>
-      </c>
-      <c r="C2" s="9" t="s">
-        <v>279</v>
       </c>
       <c r="D2" s="9" t="s">
         <v>116</v>
       </c>
       <c r="E2" s="9" t="s">
+        <v>279</v>
+      </c>
+      <c r="F2" s="8" t="s">
         <v>280</v>
       </c>
-      <c r="F2" s="8" t="s">
+      <c r="G2" s="9" t="s">
         <v>281</v>
       </c>
-      <c r="G2" s="9" t="s">
-        <v>282</v>
-      </c>
       <c r="H2" s="8" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -6659,10 +6664,10 @@
       <c r="C3" s="31"/>
       <c r="D3" s="31"/>
       <c r="E3" s="31" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="F3" s="31" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="G3" s="32"/>
     </row>
@@ -6671,7 +6676,7 @@
         <v>21</v>
       </c>
       <c r="B4" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="C4" t="s">
         <v>28</v>
@@ -6680,16 +6685,16 @@
         <v>162</v>
       </c>
       <c r="E4" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="F4" t="s">
+        <v>283</v>
+      </c>
+      <c r="G4" t="s">
         <v>284</v>
       </c>
-      <c r="G4" t="s">
-        <v>285</v>
-      </c>
       <c r="H4" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -6697,7 +6702,7 @@
         <v>21</v>
       </c>
       <c r="B5" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="C5" t="s">
         <v>28</v>
@@ -6706,16 +6711,16 @@
         <v>162</v>
       </c>
       <c r="E5" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="F5" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="G5" t="s">
         <v>87</v>
       </c>
       <c r="H5" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -6723,7 +6728,7 @@
         <v>21</v>
       </c>
       <c r="B6" s="31" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="C6" s="31" t="s">
         <v>28</v>
@@ -6732,14 +6737,14 @@
         <v>162</v>
       </c>
       <c r="E6" s="31" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="F6" s="31"/>
       <c r="G6" s="31">
         <v>1</v>
       </c>
       <c r="H6" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
@@ -6747,7 +6752,7 @@
         <v>11</v>
       </c>
       <c r="B7" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="C7" t="s">
         <v>28</v>
@@ -6756,16 +6761,16 @@
         <v>162</v>
       </c>
       <c r="E7" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="F7" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="G7" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="H7" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
@@ -6773,7 +6778,7 @@
         <v>11</v>
       </c>
       <c r="B8" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="C8" t="s">
         <v>28</v>
@@ -6782,16 +6787,16 @@
         <v>162</v>
       </c>
       <c r="E8" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="F8" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="G8">
         <v>0.2</v>
       </c>
       <c r="H8" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -6799,7 +6804,7 @@
         <v>11</v>
       </c>
       <c r="B9" s="31" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="C9" s="31" t="s">
         <v>28</v>
@@ -6808,19 +6813,19 @@
         <v>162</v>
       </c>
       <c r="E9" s="31" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="F9" s="31"/>
       <c r="G9" s="31">
         <v>1</v>
       </c>
       <c r="H9" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
     </row>
     <row r="21" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H21" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Ongoing work on a new fluids_new.py
</commit_message>
<xml_diff>
--- a/excels/project_table_new.xlsx
+++ b/excels/project_table_new.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\emb\Documents\PycharmProjects\blixt_rp\excels\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marte\PycharmProjects\blixt_rp\excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D0D9EB2-1CD8-4A9B-B628-D4C9ACB0E881}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{738B2E76-12C4-40EF-9A6D-681BD1D2C820}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6840" yWindow="1410" windowWidth="28800" windowHeight="17145" tabRatio="685" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="780" yWindow="780" windowWidth="21600" windowHeight="11295" tabRatio="685" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Well settings" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
Found a bug in un_translate method of LogTable. The fix can have consequences for other places. Hope it is limited.
</commit_message>
<xml_diff>
--- a/excels/project_table_new.xlsx
+++ b/excels/project_table_new.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marte\PycharmProjects\blixt_rp\excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{738B2E76-12C4-40EF-9A6D-681BD1D2C820}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{E980F469-474F-4B73-B796-7F6A4284919D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="780" yWindow="780" windowWidth="21600" windowHeight="11295" tabRatio="685" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="750" yWindow="2985" windowWidth="21495" windowHeight="12720" tabRatio="685" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Well settings" sheetId="1" r:id="rId1"/>
@@ -641,9 +641,6 @@
     <t>RDEP,RES_D_RSI</t>
   </si>
   <si>
-    <t>$\Omega m$</t>
-  </si>
-  <si>
     <t>log</t>
   </si>
   <si>
@@ -1257,6 +1254,9 @@
   </si>
   <si>
     <t>PENOBSCOTL_30</t>
+  </si>
+  <si>
+    <t>Ohm m</t>
   </si>
 </sst>
 </file>
@@ -2024,7 +2024,7 @@
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="B3" s="13" t="s">
         <v>12</v>
@@ -2044,7 +2044,7 @@
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>11</v>
+        <v>21</v>
       </c>
       <c r="B4" s="13" t="s">
         <v>15</v>
@@ -2058,7 +2058,7 @@
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>11</v>
+        <v>21</v>
       </c>
       <c r="B5" s="13" t="s">
         <v>18</v>
@@ -2100,7 +2100,7 @@
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>11</v>
+        <v>21</v>
       </c>
       <c r="B8" s="13" t="s">
         <v>28</v>
@@ -2140,7 +2140,7 @@
         <v>21</v>
       </c>
       <c r="B10" s="13" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="C10" s="20" t="s">
         <v>23</v>
@@ -2197,35 +2197,35 @@
   <sheetData>
     <row r="1" spans="1:7" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F1" s="7" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="2" spans="1:7" s="8" customFormat="1" ht="30.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="33" t="s">
+        <v>255</v>
+      </c>
+      <c r="B2" s="34" t="s">
         <v>256</v>
       </c>
-      <c r="B2" s="34" t="s">
+      <c r="C2" s="34" t="s">
         <v>257</v>
       </c>
-      <c r="C2" s="34" t="s">
+      <c r="D2" s="34" t="s">
         <v>258</v>
       </c>
-      <c r="D2" s="34" t="s">
+      <c r="E2" s="33" t="s">
+        <v>287</v>
+      </c>
+      <c r="F2" s="33" t="s">
         <v>259</v>
       </c>
-      <c r="E2" s="33" t="s">
+      <c r="G2" s="33" t="s">
         <v>288</v>
-      </c>
-      <c r="F2" s="33" t="s">
-        <v>260</v>
-      </c>
-      <c r="G2" s="33" t="s">
-        <v>289</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="B3">
         <v>36.6</v>
@@ -2242,7 +2242,7 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="B4">
         <v>11.4</v>
@@ -2257,15 +2257,15 @@
         <v>0</v>
       </c>
       <c r="F4" t="s">
+        <v>291</v>
+      </c>
+      <c r="G4" t="s">
         <v>292</v>
-      </c>
-      <c r="G4" t="s">
-        <v>293</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="B5">
         <v>76.8</v>
@@ -2282,7 +2282,7 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="B6">
         <v>94.9</v>
@@ -2299,7 +2299,7 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="B7">
         <v>26</v>
@@ -2316,7 +2316,7 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="B8">
         <v>47</v>
@@ -2333,7 +2333,7 @@
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="B9">
         <v>114</v>
@@ -2350,7 +2350,7 @@
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="B10">
         <v>55</v>
@@ -2367,7 +2367,7 @@
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="B11">
         <v>48</v>
@@ -2384,7 +2384,7 @@
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="B12">
         <v>85</v>
@@ -2401,7 +2401,7 @@
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="B13">
         <v>52</v>
@@ -2418,7 +2418,7 @@
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="B14">
         <v>50</v>
@@ -2435,7 +2435,7 @@
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="B15">
         <v>25.2</v>
@@ -2452,7 +2452,7 @@
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="B16">
         <v>66.5</v>
@@ -2469,7 +2469,7 @@
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="B17">
         <v>58</v>
@@ -2486,7 +2486,7 @@
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="B18">
         <v>158</v>
@@ -2503,7 +2503,7 @@
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="B19">
         <v>27</v>
@@ -2520,7 +2520,7 @@
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="B20">
         <v>123.7</v>
@@ -2537,7 +2537,7 @@
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="B21">
         <v>15</v>
@@ -2554,7 +2554,7 @@
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="B22">
         <v>17.96</v>
@@ -2571,7 +2571,7 @@
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="B23">
         <v>55.8</v>
@@ -2588,7 +2588,7 @@
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="B24">
         <v>87</v>
@@ -2605,7 +2605,7 @@
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="B25">
         <v>103.67</v>
@@ -2622,7 +2622,7 @@
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="B26">
         <v>129.13999999999999</v>
@@ -2639,7 +2639,7 @@
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="B27">
         <v>4.5199999999999996</v>
@@ -2656,7 +2656,7 @@
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="B28">
         <v>160.29</v>
@@ -2673,7 +2673,7 @@
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="B29">
         <v>62.2</v>
@@ -2690,7 +2690,7 @@
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="B30">
         <v>146.25</v>
@@ -2707,7 +2707,7 @@
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="B31">
         <v>48.35</v>
@@ -2724,7 +2724,7 @@
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="B32">
         <v>2.9</v>
@@ -2741,7 +2741,7 @@
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="B33">
         <v>12.3</v>
@@ -2774,21 +2774,21 @@
   <sheetData>
     <row r="1" spans="1:4" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D1" s="5" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
     </row>
     <row r="2" spans="1:4" s="8" customFormat="1" ht="30.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="9" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="B2" s="9" t="s">
         <v>116</v>
       </c>
       <c r="C2" s="8" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="D2" s="10" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -2799,10 +2799,10 @@
         <v>162</v>
       </c>
       <c r="C3" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -2813,7 +2813,7 @@
         <v>162</v>
       </c>
       <c r="C4" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="D4" t="s">
         <v>64</v>
@@ -2866,49 +2866,49 @@
       <c r="J1" s="2"/>
       <c r="K1" s="2"/>
       <c r="L1" s="2" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="M1" s="2" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="O1" s="2"/>
     </row>
     <row r="2" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>361</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>368</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>369</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>370</v>
+      </c>
+      <c r="F2" s="1" t="s">
         <v>362</v>
       </c>
-      <c r="C2" s="1" t="s">
-        <v>369</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>370</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>371</v>
-      </c>
-      <c r="F2" s="1" t="s">
+      <c r="G2" s="1" t="s">
         <v>363</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="H2" s="1" t="s">
         <v>364</v>
-      </c>
-      <c r="H2" s="1" t="s">
-        <v>365</v>
       </c>
       <c r="I2" s="1" t="s">
         <v>157</v>
       </c>
       <c r="J2" s="1" t="s">
+        <v>365</v>
+      </c>
+      <c r="K2" s="1" t="s">
         <v>366</v>
       </c>
-      <c r="K2" s="1" t="s">
+      <c r="L2" s="1" t="s">
         <v>367</v>
-      </c>
-      <c r="L2" s="1" t="s">
-        <v>368</v>
       </c>
       <c r="M2" s="1" t="s">
         <v>8</v>
@@ -2931,7 +2931,7 @@
     <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" s="2"/>
       <c r="B1" s="2" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="C1" s="2"/>
       <c r="D1" s="2"/>
@@ -2943,22 +2943,22 @@
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>99</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="D2" s="1" t="s">
+        <v>374</v>
+      </c>
+      <c r="E2" s="1" t="s">
         <v>375</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="F2" s="1" t="s">
         <v>376</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>377</v>
       </c>
       <c r="G2" s="1"/>
       <c r="H2" s="1"/>
@@ -2996,57 +2996,57 @@
   <sheetData>
     <row r="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="H1" s="2" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
     </row>
     <row r="2" spans="1:17" s="6" customFormat="1" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2" s="6" t="s">
+        <v>324</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>268</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>276</v>
+      </c>
+      <c r="E2" t="s">
         <v>325</v>
       </c>
-      <c r="C2" s="6" t="s">
-        <v>269</v>
-      </c>
-      <c r="D2" s="6" t="s">
-        <v>277</v>
-      </c>
-      <c r="E2" t="s">
+      <c r="F2" s="6" t="s">
         <v>326</v>
       </c>
-      <c r="F2" s="6" t="s">
+      <c r="G2" s="6" t="s">
         <v>327</v>
-      </c>
-      <c r="G2" s="6" t="s">
-        <v>328</v>
       </c>
       <c r="H2" s="1" t="s">
         <v>116</v>
       </c>
       <c r="I2" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="J2" s="6" t="s">
+        <v>328</v>
+      </c>
+      <c r="K2" t="s">
         <v>329</v>
       </c>
-      <c r="K2" t="s">
+      <c r="L2" t="s">
         <v>330</v>
       </c>
-      <c r="L2" t="s">
+      <c r="M2" t="s">
         <v>331</v>
       </c>
-      <c r="M2" t="s">
+      <c r="N2" t="s">
         <v>332</v>
-      </c>
-      <c r="N2" t="s">
-        <v>333</v>
       </c>
       <c r="O2" t="s">
         <v>102</v>
       </c>
       <c r="P2" t="s">
+        <v>347</v>
+      </c>
+      <c r="Q2" t="s">
         <v>348</v>
-      </c>
-      <c r="Q2" t="s">
-        <v>349</v>
       </c>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.25">
@@ -3054,22 +3054,22 @@
         <v>11</v>
       </c>
       <c r="B3" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="C3" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="D3" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="E3" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="F3" t="s">
         <v>14</v>
       </c>
       <c r="G3" s="13" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="H3" t="s">
         <v>127</v>
@@ -3079,16 +3079,16 @@
         <v>4</v>
       </c>
       <c r="J3" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="K3" t="s">
+        <v>334</v>
+      </c>
+      <c r="L3" t="s">
         <v>335</v>
       </c>
-      <c r="L3" t="s">
+      <c r="M3" t="s">
         <v>336</v>
-      </c>
-      <c r="M3" t="s">
-        <v>337</v>
       </c>
       <c r="N3" t="s">
         <v>128</v>
@@ -3097,10 +3097,10 @@
         <v>106</v>
       </c>
       <c r="P3" t="s">
+        <v>349</v>
+      </c>
+      <c r="Q3" t="s">
         <v>350</v>
-      </c>
-      <c r="Q3" t="s">
-        <v>351</v>
       </c>
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.25">
@@ -3108,22 +3108,22 @@
         <v>21</v>
       </c>
       <c r="B4" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="C4" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="D4" t="s">
+        <v>281</v>
+      </c>
+      <c r="E4" t="s">
         <v>282</v>
-      </c>
-      <c r="E4" t="s">
-        <v>283</v>
       </c>
       <c r="F4" t="s">
         <v>17</v>
       </c>
       <c r="G4" s="13" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="H4" t="s">
         <v>146</v>
@@ -3133,36 +3133,36 @@
         <v>4</v>
       </c>
       <c r="J4" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="K4" t="s">
         <v>103</v>
       </c>
       <c r="L4" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="M4" t="s">
         <v>105</v>
       </c>
       <c r="O4" t="s">
+        <v>351</v>
+      </c>
+      <c r="P4" t="s">
         <v>352</v>
       </c>
-      <c r="P4" t="s">
+      <c r="Q4" t="s">
         <v>353</v>
-      </c>
-      <c r="Q4" t="s">
-        <v>354</v>
       </c>
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.25">
       <c r="E5" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="F5" t="s">
         <v>20</v>
       </c>
       <c r="G5" s="13" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="H5" t="s">
         <v>161</v>
@@ -3175,10 +3175,10 @@
         <v>105</v>
       </c>
       <c r="O5" t="s">
+        <v>354</v>
+      </c>
+      <c r="Q5" t="s">
         <v>355</v>
-      </c>
-      <c r="Q5" t="s">
-        <v>356</v>
       </c>
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.25">
@@ -3186,7 +3186,7 @@
         <v>27</v>
       </c>
       <c r="G6" s="13" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="H6" t="s">
         <v>162</v>
@@ -3196,10 +3196,10 @@
         <v>4</v>
       </c>
       <c r="O6" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="Q6" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
     </row>
     <row r="7" spans="1:17" x14ac:dyDescent="0.25">
@@ -3214,10 +3214,10 @@
         <v>4</v>
       </c>
       <c r="O7" t="s">
+        <v>357</v>
+      </c>
+      <c r="Q7" t="s">
         <v>358</v>
-      </c>
-      <c r="Q7" t="s">
-        <v>359</v>
       </c>
     </row>
     <row r="8" spans="1:17" x14ac:dyDescent="0.25">
@@ -3282,7 +3282,7 @@
     </row>
     <row r="13" spans="1:17" x14ac:dyDescent="0.25">
       <c r="F13" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="H13" s="30" t="s">
         <v>169</v>
@@ -3294,7 +3294,7 @@
     </row>
     <row r="14" spans="1:17" x14ac:dyDescent="0.25">
       <c r="F14" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="H14" s="30" t="s">
         <v>170</v>
@@ -3318,7 +3318,7 @@
     </row>
     <row r="16" spans="1:17" x14ac:dyDescent="0.25">
       <c r="F16" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="H16" s="30" t="s">
         <v>172</v>
@@ -3436,7 +3436,7 @@
         <v>12</v>
       </c>
       <c r="B3" t="s">
-        <v>11</v>
+        <v>21</v>
       </c>
       <c r="C3" s="4" t="s">
         <v>59</v>
@@ -3704,7 +3704,7 @@
         <v>98</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
     </row>
     <row r="2" spans="1:13" ht="30" x14ac:dyDescent="0.25">
@@ -3724,19 +3724,19 @@
         <v>102</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="K2" s="1" t="s">
         <v>10</v>
@@ -3761,13 +3761,13 @@
         <v>106</v>
       </c>
       <c r="F3" t="s">
+        <v>381</v>
+      </c>
+      <c r="G3" t="s">
         <v>382</v>
       </c>
-      <c r="G3" t="s">
+      <c r="H3" t="s">
         <v>383</v>
-      </c>
-      <c r="H3" t="s">
-        <v>384</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
@@ -3787,10 +3787,10 @@
         <v>106</v>
       </c>
       <c r="G4" t="s">
+        <v>384</v>
+      </c>
+      <c r="I4" t="s">
         <v>385</v>
-      </c>
-      <c r="I4" t="s">
-        <v>386</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
@@ -3814,13 +3814,13 @@
         <v>106</v>
       </c>
       <c r="F6" t="s">
+        <v>381</v>
+      </c>
+      <c r="G6" t="s">
         <v>382</v>
       </c>
-      <c r="G6" t="s">
+      <c r="H6" t="s">
         <v>383</v>
-      </c>
-      <c r="H6" t="s">
-        <v>384</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
@@ -3840,10 +3840,10 @@
         <v>106</v>
       </c>
       <c r="G7" t="s">
+        <v>384</v>
+      </c>
+      <c r="I7" t="s">
         <v>385</v>
-      </c>
-      <c r="I7" t="s">
-        <v>386</v>
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.25">
@@ -3867,13 +3867,13 @@
         <v>106</v>
       </c>
       <c r="F9" t="s">
+        <v>381</v>
+      </c>
+      <c r="G9" t="s">
         <v>382</v>
       </c>
-      <c r="G9" t="s">
+      <c r="H9" t="s">
         <v>383</v>
-      </c>
-      <c r="H9" t="s">
-        <v>384</v>
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.25">
@@ -3893,10 +3893,10 @@
         <v>106</v>
       </c>
       <c r="G10" t="s">
+        <v>384</v>
+      </c>
+      <c r="I10" t="s">
         <v>385</v>
-      </c>
-      <c r="I10" t="s">
-        <v>386</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.25">
@@ -3955,16 +3955,16 @@
         <v>106</v>
       </c>
       <c r="F17" t="s">
+        <v>381</v>
+      </c>
+      <c r="G17" t="s">
         <v>382</v>
       </c>
-      <c r="G17" t="s">
+      <c r="H17" t="s">
         <v>383</v>
       </c>
-      <c r="H17" t="s">
-        <v>384</v>
-      </c>
       <c r="K17" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.25">
@@ -3984,10 +3984,10 @@
         <v>106</v>
       </c>
       <c r="G18" t="s">
+        <v>384</v>
+      </c>
+      <c r="I18" t="s">
         <v>385</v>
-      </c>
-      <c r="I18" t="s">
-        <v>386</v>
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.25">
@@ -4085,7 +4085,7 @@
         <v>188</v>
       </c>
       <c r="N2" s="1" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="O2" s="1" t="s">
         <v>189</v>
@@ -4099,13 +4099,13 @@
         <v>55</v>
       </c>
       <c r="C3" t="s">
+        <v>394</v>
+      </c>
+      <c r="D3" t="s">
         <v>191</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
         <v>192</v>
-      </c>
-      <c r="E3" t="s">
-        <v>193</v>
       </c>
       <c r="F3" s="3">
         <v>0.2</v>
@@ -4114,13 +4114,13 @@
         <v>200</v>
       </c>
       <c r="I3" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="K3" s="14" t="s">
         <v>13</v>
       </c>
       <c r="L3" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="M3">
         <v>1</v>
@@ -4131,13 +4131,13 @@
         <v>45</v>
       </c>
       <c r="C4" t="s">
+        <v>195</v>
+      </c>
+      <c r="D4" t="s">
         <v>196</v>
       </c>
-      <c r="D4" t="s">
-        <v>197</v>
-      </c>
       <c r="E4" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="F4" s="3">
         <v>2000</v>
@@ -4146,13 +4146,13 @@
         <v>5000</v>
       </c>
       <c r="I4" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="K4" s="15" t="s">
         <v>16</v>
       </c>
       <c r="L4" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="M4">
         <v>1</v>
@@ -4163,13 +4163,13 @@
         <v>47</v>
       </c>
       <c r="C5" t="s">
+        <v>195</v>
+      </c>
+      <c r="D5" t="s">
         <v>196</v>
       </c>
-      <c r="D5" t="s">
-        <v>197</v>
-      </c>
       <c r="E5" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="F5" s="3">
         <v>800</v>
@@ -4178,13 +4178,13 @@
         <v>3500</v>
       </c>
       <c r="I5" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="K5" s="16" t="s">
         <v>19</v>
       </c>
       <c r="L5" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="M5">
         <v>1</v>
@@ -4192,19 +4192,19 @@
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>197</v>
+      </c>
+      <c r="B6" t="s">
         <v>198</v>
       </c>
-      <c r="B6" t="s">
+      <c r="C6" t="s">
         <v>199</v>
       </c>
-      <c r="C6" t="s">
-        <v>200</v>
-      </c>
       <c r="D6" t="s">
+        <v>191</v>
+      </c>
+      <c r="E6" t="s">
         <v>192</v>
-      </c>
-      <c r="E6" t="s">
-        <v>193</v>
       </c>
       <c r="F6" s="3">
         <v>0.01</v>
@@ -4213,13 +4213,13 @@
         <v>2000</v>
       </c>
       <c r="I6" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="K6" s="17" t="s">
         <v>26</v>
       </c>
       <c r="L6" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="M6">
         <v>1</v>
@@ -4227,19 +4227,19 @@
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>200</v>
+      </c>
+      <c r="B7" t="s">
         <v>201</v>
       </c>
-      <c r="B7" t="s">
-        <v>202</v>
-      </c>
       <c r="C7" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="D7" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="E7" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="F7" s="3">
         <v>1.4</v>
@@ -4248,13 +4248,13 @@
         <v>4</v>
       </c>
       <c r="I7" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="K7" s="18" t="s">
         <v>29</v>
       </c>
       <c r="L7" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="M7">
         <v>1</v>
@@ -4262,19 +4262,19 @@
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>202</v>
+      </c>
+      <c r="B8" t="s">
         <v>203</v>
       </c>
-      <c r="B8" t="s">
+      <c r="C8" t="s">
         <v>204</v>
       </c>
-      <c r="C8" t="s">
-        <v>205</v>
-      </c>
       <c r="D8" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="E8" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="F8" s="3">
         <v>6500</v>
@@ -4283,13 +4283,13 @@
         <v>11000</v>
       </c>
       <c r="I8" t="s">
+        <v>193</v>
+      </c>
+      <c r="K8" s="19" t="s">
+        <v>205</v>
+      </c>
+      <c r="L8" t="s">
         <v>194</v>
-      </c>
-      <c r="K8" s="19" t="s">
-        <v>206</v>
-      </c>
-      <c r="L8" t="s">
-        <v>195</v>
       </c>
       <c r="M8">
         <v>1</v>
@@ -4297,24 +4297,24 @@
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
+        <v>206</v>
+      </c>
+      <c r="C9" t="s">
         <v>207</v>
       </c>
-      <c r="C9" t="s">
-        <v>208</v>
-      </c>
       <c r="D9" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="E9" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="F9" s="3"/>
       <c r="G9" s="3"/>
       <c r="I9" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="K9" s="19" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="M9">
         <v>1</v>
@@ -4322,24 +4322,24 @@
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="C10" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="D10" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="E10" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="F10" s="3"/>
       <c r="G10" s="3"/>
       <c r="I10" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="K10" s="19" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="M10">
         <v>1</v>
@@ -4347,19 +4347,19 @@
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B11" t="s">
         <v>52</v>
       </c>
       <c r="C11" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="D11" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="E11" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="F11" s="3">
         <v>0</v>
@@ -4368,13 +4368,13 @@
         <v>0.3</v>
       </c>
       <c r="I11" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="K11" s="20" t="s">
         <v>23</v>
       </c>
       <c r="L11" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="M11">
         <v>1</v>
@@ -4382,19 +4382,19 @@
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="B12" t="s">
         <v>53</v>
       </c>
       <c r="C12" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="D12" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="E12" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="F12" s="3">
         <v>0</v>
@@ -4403,13 +4403,13 @@
         <v>1</v>
       </c>
       <c r="I12" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="K12" s="26" t="s">
+        <v>211</v>
+      </c>
+      <c r="L12" t="s">
         <v>212</v>
-      </c>
-      <c r="L12" t="s">
-        <v>213</v>
       </c>
       <c r="M12">
         <v>1</v>
@@ -4417,19 +4417,19 @@
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="B13" t="s">
         <v>54</v>
       </c>
       <c r="C13" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="D13" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="E13" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="F13" s="3">
         <v>0</v>
@@ -4438,13 +4438,13 @@
         <v>1</v>
       </c>
       <c r="I13" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="K13" s="22" t="s">
         <v>37</v>
       </c>
       <c r="L13" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="M13">
         <v>1</v>
@@ -4458,13 +4458,13 @@
         <v>50</v>
       </c>
       <c r="C14" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="D14" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="E14" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="F14" s="3">
         <v>1.8</v>
@@ -4473,13 +4473,13 @@
         <v>3.2</v>
       </c>
       <c r="I14" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="K14" s="23" t="s">
         <v>39</v>
       </c>
       <c r="L14" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="M14">
         <v>1</v>
@@ -4487,19 +4487,19 @@
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="B15" t="s">
         <v>51</v>
       </c>
       <c r="C15" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="D15" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="E15" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="F15" s="3">
         <v>0.45</v>
@@ -4508,13 +4508,13 @@
         <v>-0.15</v>
       </c>
       <c r="I15" t="s">
+        <v>193</v>
+      </c>
+      <c r="K15" s="27" t="s">
+        <v>217</v>
+      </c>
+      <c r="L15" t="s">
         <v>194</v>
-      </c>
-      <c r="K15" s="27" t="s">
-        <v>218</v>
-      </c>
-      <c r="L15" t="s">
-        <v>195</v>
       </c>
       <c r="M15">
         <v>1</v>
@@ -4522,19 +4522,19 @@
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="B16" t="s">
         <v>56</v>
       </c>
       <c r="C16" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="D16" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="E16" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="F16" s="3">
         <v>6</v>
@@ -4543,13 +4543,13 @@
         <v>10</v>
       </c>
       <c r="I16" t="s">
+        <v>193</v>
+      </c>
+      <c r="K16" s="24" t="s">
+        <v>220</v>
+      </c>
+      <c r="L16" t="s">
         <v>194</v>
-      </c>
-      <c r="K16" s="24" t="s">
-        <v>221</v>
-      </c>
-      <c r="L16" t="s">
-        <v>195</v>
       </c>
       <c r="M16">
         <v>1</v>
@@ -4557,19 +4557,19 @@
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="B17" t="s">
         <v>49</v>
       </c>
       <c r="C17" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="D17" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="E17" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="F17" s="3">
         <v>0</v>
@@ -4578,13 +4578,13 @@
         <v>350</v>
       </c>
       <c r="I17" t="s">
+        <v>193</v>
+      </c>
+      <c r="K17" s="36" t="s">
+        <v>252</v>
+      </c>
+      <c r="L17" t="s">
         <v>194</v>
-      </c>
-      <c r="K17" s="36" t="s">
-        <v>253</v>
-      </c>
-      <c r="L17" t="s">
-        <v>195</v>
       </c>
       <c r="M17">
         <v>1</v>
@@ -4592,19 +4592,19 @@
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="B18" t="s">
         <v>46</v>
       </c>
       <c r="C18" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="D18" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="E18" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="F18" s="3">
         <v>40</v>
@@ -4613,13 +4613,13 @@
         <v>150</v>
       </c>
       <c r="I18" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="K18" s="16" t="s">
         <v>19</v>
       </c>
       <c r="L18" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="M18">
         <v>1</v>
@@ -4627,19 +4627,19 @@
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
+        <v>225</v>
+      </c>
+      <c r="B19" t="s">
         <v>226</v>
       </c>
-      <c r="B19" t="s">
-        <v>227</v>
-      </c>
       <c r="C19" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="D19" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="E19" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="F19" s="3">
         <v>80</v>
@@ -4648,13 +4648,13 @@
         <v>300</v>
       </c>
       <c r="I19" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="K19" s="17" t="s">
         <v>26</v>
       </c>
       <c r="L19" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="M19">
         <v>1</v>
@@ -4662,19 +4662,19 @@
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
+        <v>227</v>
+      </c>
+      <c r="B20" t="s">
+        <v>227</v>
+      </c>
+      <c r="C20" t="s">
         <v>228</v>
       </c>
-      <c r="B20" t="s">
-        <v>228</v>
-      </c>
-      <c r="C20" t="s">
-        <v>229</v>
-      </c>
       <c r="D20" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="E20" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="F20" s="3">
         <v>0</v>
@@ -4683,13 +4683,13 @@
         <v>15</v>
       </c>
       <c r="I20" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="K20" s="18" t="s">
         <v>29</v>
       </c>
       <c r="L20" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="M20">
         <v>1</v>
@@ -4697,19 +4697,19 @@
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
+        <v>229</v>
+      </c>
+      <c r="B21" t="s">
         <v>230</v>
       </c>
-      <c r="B21" t="s">
+      <c r="C21" t="s">
+        <v>228</v>
+      </c>
+      <c r="D21" t="s">
         <v>231</v>
       </c>
-      <c r="C21" t="s">
-        <v>229</v>
-      </c>
-      <c r="D21" t="s">
-        <v>232</v>
-      </c>
       <c r="E21" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="F21" s="3">
         <v>0</v>
@@ -4718,16 +4718,16 @@
         <v>5</v>
       </c>
       <c r="I21" t="s">
+        <v>232</v>
+      </c>
+      <c r="J21" t="s">
         <v>233</v>
       </c>
-      <c r="J21" t="s">
-        <v>234</v>
-      </c>
       <c r="K21" s="19" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="L21" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="M21">
         <v>1</v>
@@ -4735,16 +4735,16 @@
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
+        <v>234</v>
+      </c>
+      <c r="B22" t="s">
         <v>235</v>
       </c>
-      <c r="B22" t="s">
-        <v>236</v>
-      </c>
       <c r="C22" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="D22" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="F22" s="3">
         <v>0</v>
@@ -4756,7 +4756,7 @@
         <v>23</v>
       </c>
       <c r="L22" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="M22">
         <v>1</v>
@@ -4764,16 +4764,16 @@
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
+        <v>236</v>
+      </c>
+      <c r="B23" t="s">
         <v>237</v>
       </c>
-      <c r="B23" t="s">
-        <v>238</v>
-      </c>
       <c r="C23" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="D23" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="F23" s="3">
         <v>0</v>
@@ -4782,16 +4782,16 @@
         <v>0.5</v>
       </c>
       <c r="I23" t="s">
+        <v>238</v>
+      </c>
+      <c r="J23" t="s">
         <v>239</v>
-      </c>
-      <c r="J23" t="s">
-        <v>240</v>
       </c>
       <c r="K23" s="21" t="s">
         <v>35</v>
       </c>
       <c r="L23" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="M23">
         <v>1</v>
@@ -4799,30 +4799,30 @@
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
+        <v>240</v>
+      </c>
+      <c r="B24" t="s">
         <v>241</v>
       </c>
-      <c r="B24" t="s">
+      <c r="C24" t="s">
         <v>242</v>
       </c>
-      <c r="C24" t="s">
-        <v>243</v>
-      </c>
       <c r="D24" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="E24" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="F24" s="3"/>
       <c r="G24" s="3"/>
       <c r="I24" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="K24" s="22" t="s">
         <v>37</v>
       </c>
       <c r="L24" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="M24">
         <v>1</v>
@@ -4830,19 +4830,19 @@
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
+        <v>243</v>
+      </c>
+      <c r="B25" t="s">
         <v>244</v>
       </c>
-      <c r="B25" t="s">
-        <v>245</v>
-      </c>
       <c r="C25" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="D25" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="E25" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="F25" s="3">
         <v>4</v>
@@ -4851,13 +4851,13 @@
         <v>12</v>
       </c>
       <c r="I25" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="K25" s="24" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="L25" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="M25">
         <v>2</v>
@@ -4871,39 +4871,39 @@
         <v>1</v>
       </c>
       <c r="D26" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="E26" t="s">
+        <v>192</v>
+      </c>
+      <c r="I26" t="s">
         <v>193</v>
       </c>
-      <c r="I26" t="s">
-        <v>194</v>
-      </c>
       <c r="K26" s="24" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
     </row>
     <row r="27" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B27" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="C27" t="s">
         <v>1</v>
       </c>
       <c r="D27" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="E27" t="s">
+        <v>192</v>
+      </c>
+      <c r="I27" t="s">
         <v>193</v>
       </c>
-      <c r="I27" t="s">
-        <v>194</v>
-      </c>
       <c r="K27" s="36" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="L27" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="M27">
         <v>1</v>
@@ -4911,25 +4911,25 @@
     </row>
     <row r="28" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B28" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="C28" t="s">
         <v>1</v>
       </c>
       <c r="D28" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="E28" t="s">
+        <v>192</v>
+      </c>
+      <c r="I28" t="s">
         <v>193</v>
       </c>
-      <c r="I28" t="s">
+      <c r="K28" s="24" t="s">
+        <v>220</v>
+      </c>
+      <c r="L28" t="s">
         <v>194</v>
-      </c>
-      <c r="K28" s="24" t="s">
-        <v>221</v>
-      </c>
-      <c r="L28" t="s">
-        <v>195</v>
       </c>
       <c r="M28">
         <v>1</v>
@@ -4937,28 +4937,28 @@
     </row>
     <row r="29" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
+        <v>246</v>
+      </c>
+      <c r="B29" t="s">
         <v>247</v>
-      </c>
-      <c r="B29" t="s">
-        <v>248</v>
       </c>
       <c r="C29" t="s">
         <v>17</v>
       </c>
       <c r="D29" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="E29" t="s">
+        <v>192</v>
+      </c>
+      <c r="I29" t="s">
         <v>193</v>
-      </c>
-      <c r="I29" t="s">
-        <v>194</v>
       </c>
       <c r="K29" s="21" t="s">
         <v>35</v>
       </c>
       <c r="L29" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="M29">
         <v>1</v>
@@ -4966,28 +4966,28 @@
     </row>
     <row r="30" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
+        <v>248</v>
+      </c>
+      <c r="B30" t="s">
         <v>249</v>
-      </c>
-      <c r="B30" t="s">
-        <v>250</v>
       </c>
       <c r="C30" t="s">
         <v>17</v>
       </c>
       <c r="D30" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="E30" t="s">
+        <v>192</v>
+      </c>
+      <c r="I30" t="s">
         <v>193</v>
-      </c>
-      <c r="I30" t="s">
-        <v>194</v>
       </c>
       <c r="K30" s="22" t="s">
         <v>37</v>
       </c>
       <c r="L30" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="M30">
         <v>1</v>
@@ -4995,25 +4995,25 @@
     </row>
     <row r="31" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B31" t="s">
+        <v>250</v>
+      </c>
+      <c r="C31" t="s">
+        <v>388</v>
+      </c>
+      <c r="D31" t="s">
+        <v>196</v>
+      </c>
+      <c r="E31" t="s">
+        <v>192</v>
+      </c>
+      <c r="I31" t="s">
         <v>251</v>
       </c>
-      <c r="C31" t="s">
-        <v>389</v>
-      </c>
-      <c r="D31" t="s">
-        <v>197</v>
-      </c>
-      <c r="E31" t="s">
-        <v>193</v>
-      </c>
-      <c r="I31" t="s">
+      <c r="K31" s="36" t="s">
         <v>252</v>
       </c>
-      <c r="K31" s="36" t="s">
-        <v>253</v>
-      </c>
       <c r="L31" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="M31">
         <v>1</v>
@@ -6191,7 +6191,7 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C4" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
@@ -6199,13 +6199,13 @@
         <v>2</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="C5" s="12" t="s">
+        <v>389</v>
+      </c>
+      <c r="D5" s="1" t="s">
         <v>390</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>391</v>
       </c>
       <c r="E5" s="1" t="s">
         <v>157</v>
@@ -6242,7 +6242,7 @@
         <v>1</v>
       </c>
       <c r="F7" s="26" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
@@ -6284,7 +6284,7 @@
         <v>1</v>
       </c>
       <c r="F10" s="27" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
@@ -6298,7 +6298,7 @@
         <v>1</v>
       </c>
       <c r="F11" s="24" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
@@ -6312,7 +6312,7 @@
         <v>1</v>
       </c>
       <c r="F12" s="25" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
@@ -6354,7 +6354,7 @@
         <v>1</v>
       </c>
       <c r="F15" s="26" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
@@ -6396,7 +6396,7 @@
         <v>1</v>
       </c>
       <c r="F18" s="27" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
@@ -6410,7 +6410,7 @@
         <v>1</v>
       </c>
       <c r="F19" s="24" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
@@ -6424,7 +6424,7 @@
         <v>1</v>
       </c>
       <c r="F20" s="25" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
@@ -6477,67 +6477,67 @@
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
+        <v>253</v>
+      </c>
+      <c r="E1" s="7" t="s">
         <v>254</v>
-      </c>
-      <c r="E1" s="7" t="s">
-        <v>255</v>
       </c>
     </row>
     <row r="2" spans="1:15" s="8" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="8" t="s">
+        <v>255</v>
+      </c>
+      <c r="B2" s="9" t="s">
         <v>256</v>
       </c>
-      <c r="B2" s="9" t="s">
+      <c r="C2" s="9" t="s">
         <v>257</v>
       </c>
-      <c r="C2" s="9" t="s">
+      <c r="D2" s="9" t="s">
         <v>258</v>
       </c>
-      <c r="D2" s="9" t="s">
+      <c r="E2" s="8" t="s">
         <v>259</v>
       </c>
-      <c r="E2" s="8" t="s">
+      <c r="F2" s="8" t="s">
         <v>260</v>
       </c>
-      <c r="F2" s="8" t="s">
+      <c r="G2" s="8" t="s">
         <v>261</v>
       </c>
-      <c r="G2" s="8" t="s">
+      <c r="H2" s="8" t="s">
         <v>262</v>
       </c>
-      <c r="H2" s="8" t="s">
+      <c r="I2" s="8" t="s">
         <v>263</v>
       </c>
-      <c r="I2" s="8" t="s">
+      <c r="J2" s="8" t="s">
         <v>264</v>
       </c>
-      <c r="J2" s="8" t="s">
+      <c r="K2" s="8" t="s">
         <v>265</v>
       </c>
-      <c r="K2" s="8" t="s">
+      <c r="L2" s="8" t="s">
         <v>266</v>
       </c>
-      <c r="L2" s="8" t="s">
+      <c r="M2" s="8" t="s">
         <v>267</v>
       </c>
-      <c r="M2" s="8" t="s">
+      <c r="N2" s="8" t="s">
         <v>268</v>
       </c>
-      <c r="N2" s="8" t="s">
+      <c r="O2" s="8" t="s">
         <v>269</v>
-      </c>
-      <c r="O2" s="8" t="s">
-        <v>270</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="B3" s="3"/>
       <c r="C3" s="3"/>
       <c r="E3" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="F3">
         <v>0.03</v>
@@ -6564,7 +6564,7 @@
         <v>0.6</v>
       </c>
       <c r="N3" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="O3">
         <v>2</v>
@@ -6572,7 +6572,7 @@
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="B4" s="3">
         <v>2.68</v>
@@ -6582,7 +6582,7 @@
         <v>1.0229999999999999</v>
       </c>
       <c r="E4" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
@@ -6627,7 +6627,7 @@
         <v>0</v>
       </c>
       <c r="G1" s="7" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
     </row>
     <row r="2" spans="1:8" s="8" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -6635,25 +6635,25 @@
         <v>2</v>
       </c>
       <c r="B2" s="9" t="s">
+        <v>276</v>
+      </c>
+      <c r="C2" s="9" t="s">
         <v>277</v>
-      </c>
-      <c r="C2" s="9" t="s">
-        <v>278</v>
       </c>
       <c r="D2" s="9" t="s">
         <v>116</v>
       </c>
       <c r="E2" s="9" t="s">
+        <v>278</v>
+      </c>
+      <c r="F2" s="8" t="s">
         <v>279</v>
       </c>
-      <c r="F2" s="8" t="s">
+      <c r="G2" s="9" t="s">
         <v>280</v>
       </c>
-      <c r="G2" s="9" t="s">
-        <v>281</v>
-      </c>
       <c r="H2" s="8" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -6664,10 +6664,10 @@
       <c r="C3" s="31"/>
       <c r="D3" s="31"/>
       <c r="E3" s="31" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="F3" s="31" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="G3" s="32"/>
     </row>
@@ -6676,7 +6676,7 @@
         <v>21</v>
       </c>
       <c r="B4" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="C4" t="s">
         <v>28</v>
@@ -6685,16 +6685,16 @@
         <v>162</v>
       </c>
       <c r="E4" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="F4" t="s">
+        <v>282</v>
+      </c>
+      <c r="G4" t="s">
         <v>283</v>
       </c>
-      <c r="G4" t="s">
-        <v>284</v>
-      </c>
       <c r="H4" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -6702,7 +6702,7 @@
         <v>21</v>
       </c>
       <c r="B5" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="C5" t="s">
         <v>28</v>
@@ -6711,16 +6711,16 @@
         <v>162</v>
       </c>
       <c r="E5" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="F5" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="G5" t="s">
         <v>87</v>
       </c>
       <c r="H5" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -6728,7 +6728,7 @@
         <v>21</v>
       </c>
       <c r="B6" s="31" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="C6" s="31" t="s">
         <v>28</v>
@@ -6737,14 +6737,14 @@
         <v>162</v>
       </c>
       <c r="E6" s="31" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="F6" s="31"/>
       <c r="G6" s="31">
         <v>1</v>
       </c>
       <c r="H6" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
@@ -6752,7 +6752,7 @@
         <v>11</v>
       </c>
       <c r="B7" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="C7" t="s">
         <v>28</v>
@@ -6761,16 +6761,16 @@
         <v>162</v>
       </c>
       <c r="E7" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="F7" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="G7" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="H7" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
@@ -6778,7 +6778,7 @@
         <v>11</v>
       </c>
       <c r="B8" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="C8" t="s">
         <v>28</v>
@@ -6787,16 +6787,16 @@
         <v>162</v>
       </c>
       <c r="E8" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="F8" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="G8">
         <v>0.2</v>
       </c>
       <c r="H8" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -6804,7 +6804,7 @@
         <v>11</v>
       </c>
       <c r="B9" s="31" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="C9" s="31" t="s">
         <v>28</v>
@@ -6813,19 +6813,19 @@
         <v>162</v>
       </c>
       <c r="E9" s="31" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="F9" s="31"/>
       <c r="G9" s="31">
         <v>1</v>
       </c>
       <c r="H9" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
     </row>
     <row r="21" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H21" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Trying to clean up the rename_log functionality. Added a rename_log variable to well_reader in io.py. It works, but it has not been implemented in read_las
</commit_message>
<xml_diff>
--- a/excels/project_table_new.xlsx
+++ b/excels/project_table_new.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marte\PycharmProjects\blixt_rp\excels\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\emb\Documents\PycharmProjects\blixt_rp\excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E980F469-474F-4B73-B796-7F6A4284919D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E11869BF-D175-4BAA-AF93-CF6DA91B6E8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="750" yWindow="2985" windowWidth="21495" windowHeight="12720" tabRatio="685" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1950" yWindow="1950" windowWidth="28800" windowHeight="17145" tabRatio="685" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Well settings" sheetId="1" r:id="rId1"/>
@@ -3436,7 +3436,7 @@
         <v>12</v>
       </c>
       <c r="B3" t="s">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="C3" s="4" t="s">
         <v>59</v>
@@ -3482,7 +3482,7 @@
         <v>15</v>
       </c>
       <c r="B5" t="s">
-        <v>11</v>
+        <v>21</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>69</v>
@@ -3508,7 +3508,7 @@
         <v>18</v>
       </c>
       <c r="B6" t="s">
-        <v>11</v>
+        <v>21</v>
       </c>
       <c r="C6" s="4" t="s">
         <v>73</v>
@@ -3534,7 +3534,7 @@
         <v>22</v>
       </c>
       <c r="B7" t="s">
-        <v>11</v>
+        <v>21</v>
       </c>
       <c r="C7" s="4" t="s">
         <v>74</v>
@@ -3563,7 +3563,7 @@
         <v>25</v>
       </c>
       <c r="B8" t="s">
-        <v>11</v>
+        <v>21</v>
       </c>
       <c r="C8" s="4" t="s">
         <v>81</v>
@@ -3580,7 +3580,7 @@
         <v>25</v>
       </c>
       <c r="B9" t="s">
-        <v>11</v>
+        <v>21</v>
       </c>
       <c r="C9" s="4" t="s">
         <v>84</v>
@@ -3603,7 +3603,7 @@
         <v>28</v>
       </c>
       <c r="B10" t="s">
-        <v>11</v>
+        <v>21</v>
       </c>
       <c r="C10" s="4" t="s">
         <v>89</v>
@@ -3635,7 +3635,7 @@
         <v>31</v>
       </c>
       <c r="B11" t="s">
-        <v>11</v>
+        <v>21</v>
       </c>
       <c r="C11" s="4" t="s">
         <v>91</v>

</xml_diff>

<commit_message>
Ongoing work. Focus on updating fluids_new.py so that the fluid substitution becomes more manageable
</commit_message>
<xml_diff>
--- a/excels/project_table_new.xlsx
+++ b/excels/project_table_new.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\emb\Documents\PycharmProjects\blixt_rp\excels\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="T:\Python\EMB\blixt_rp\excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E11869BF-D175-4BAA-AF93-CF6DA91B6E8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE2D827C-0E2B-4F55-B610-6C2A742D08A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1950" yWindow="1950" windowWidth="28800" windowHeight="17145" tabRatio="685" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="685" firstSheet="7" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Well settings" sheetId="1" r:id="rId1"/>
@@ -32,6 +32,7 @@
     <definedName name="AvoClasses">Utils!$Q$3:$Q$7</definedName>
     <definedName name="CheckshotFormat">Utils!$M$3:$M$4</definedName>
     <definedName name="FluidNames">Fluids!$A$3:$A$8</definedName>
+    <definedName name="FluidTypes">Utils!$E$3:$E$6</definedName>
     <definedName name="IntervalNames">Utils!$H$3:$H$18</definedName>
     <definedName name="LineStyles">Utils!$G$3:$G$6</definedName>
     <definedName name="LogTypes">Templates!$B$3:$B48</definedName>
@@ -63,7 +64,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="978" uniqueCount="395">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="982" uniqueCount="396">
   <si>
     <t>Select Yes or No</t>
   </si>
@@ -947,9 +948,6 @@
     <t>Interval average</t>
   </si>
   <si>
-    <t>VCL&gt;0.8, PHIE&lt;0.1</t>
-  </si>
-  <si>
     <t>Calcite</t>
   </si>
   <si>
@@ -1257,6 +1255,12 @@
   </si>
   <si>
     <t>Ohm m</t>
+  </si>
+  <si>
+    <t>VCL&gt;0.8[], PHIE&lt;0.1[]</t>
+  </si>
+  <si>
+    <t>"log_name" "operator" "limit(s)" "[units]"</t>
   </si>
 </sst>
 </file>
@@ -2024,7 +2028,7 @@
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>11</v>
+        <v>21</v>
       </c>
       <c r="B3" s="13" t="s">
         <v>12</v>
@@ -2100,7 +2104,7 @@
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="B8" s="13" t="s">
         <v>28</v>
@@ -2140,7 +2144,7 @@
         <v>21</v>
       </c>
       <c r="B10" s="13" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="C10" s="20" t="s">
         <v>23</v>
@@ -2199,6 +2203,9 @@
       <c r="F1" s="7" t="s">
         <v>286</v>
       </c>
+      <c r="G1" s="2" t="s">
+        <v>395</v>
+      </c>
     </row>
     <row r="2" spans="1:7" s="8" customFormat="1" ht="30.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="33" t="s">
@@ -2260,12 +2267,12 @@
         <v>291</v>
       </c>
       <c r="G4" t="s">
-        <v>292</v>
+        <v>394</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="B5">
         <v>76.8</v>
@@ -2282,7 +2289,7 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="B6">
         <v>94.9</v>
@@ -2299,7 +2306,7 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="B7">
         <v>26</v>
@@ -2316,7 +2323,7 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="B8">
         <v>47</v>
@@ -2333,7 +2340,7 @@
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="B9">
         <v>114</v>
@@ -2350,7 +2357,7 @@
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="B10">
         <v>55</v>
@@ -2367,7 +2374,7 @@
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="B11">
         <v>48</v>
@@ -2384,7 +2391,7 @@
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="B12">
         <v>85</v>
@@ -2401,7 +2408,7 @@
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="B13">
         <v>52</v>
@@ -2418,7 +2425,7 @@
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="B14">
         <v>50</v>
@@ -2435,7 +2442,7 @@
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="B15">
         <v>25.2</v>
@@ -2452,7 +2459,7 @@
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="B16">
         <v>66.5</v>
@@ -2469,7 +2476,7 @@
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="B17">
         <v>58</v>
@@ -2486,7 +2493,7 @@
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="B18">
         <v>158</v>
@@ -2503,7 +2510,7 @@
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="B19">
         <v>27</v>
@@ -2520,7 +2527,7 @@
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="B20">
         <v>123.7</v>
@@ -2537,7 +2544,7 @@
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="B21">
         <v>15</v>
@@ -2554,7 +2561,7 @@
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="B22">
         <v>17.96</v>
@@ -2571,7 +2578,7 @@
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="B23">
         <v>55.8</v>
@@ -2588,7 +2595,7 @@
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="B24">
         <v>87</v>
@@ -2605,7 +2612,7 @@
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="B25">
         <v>103.67</v>
@@ -2622,7 +2629,7 @@
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="B26">
         <v>129.13999999999999</v>
@@ -2639,7 +2646,7 @@
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="B27">
         <v>4.5199999999999996</v>
@@ -2656,7 +2663,7 @@
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="B28">
         <v>160.29</v>
@@ -2673,7 +2680,7 @@
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="B29">
         <v>62.2</v>
@@ -2690,7 +2697,7 @@
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="B30">
         <v>146.25</v>
@@ -2707,7 +2714,7 @@
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="B31">
         <v>48.35</v>
@@ -2724,7 +2731,7 @@
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="B32">
         <v>2.9</v>
@@ -2741,7 +2748,7 @@
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="B33">
         <v>12.3</v>
@@ -2758,7 +2765,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0"/>
+  <pageSetup paperSize="9" orientation="portrait" verticalDpi="300" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -2774,7 +2781,7 @@
   <sheetData>
     <row r="1" spans="1:4" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D1" s="5" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
     </row>
     <row r="2" spans="1:4" s="8" customFormat="1" ht="30.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -2785,7 +2792,7 @@
         <v>116</v>
       </c>
       <c r="C2" s="8" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="D2" s="10" t="s">
         <v>280</v>
@@ -2866,49 +2873,49 @@
       <c r="J1" s="2"/>
       <c r="K1" s="2"/>
       <c r="L1" s="2" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="M1" s="2" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="O1" s="2"/>
     </row>
     <row r="2" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>360</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>367</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>368</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>369</v>
+      </c>
+      <c r="F2" s="1" t="s">
         <v>361</v>
       </c>
-      <c r="C2" s="1" t="s">
-        <v>368</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>369</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>370</v>
-      </c>
-      <c r="F2" s="1" t="s">
+      <c r="G2" s="1" t="s">
         <v>362</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="H2" s="1" t="s">
         <v>363</v>
-      </c>
-      <c r="H2" s="1" t="s">
-        <v>364</v>
       </c>
       <c r="I2" s="1" t="s">
         <v>157</v>
       </c>
       <c r="J2" s="1" t="s">
+        <v>364</v>
+      </c>
+      <c r="K2" s="1" t="s">
         <v>365</v>
       </c>
-      <c r="K2" s="1" t="s">
+      <c r="L2" s="1" t="s">
         <v>366</v>
-      </c>
-      <c r="L2" s="1" t="s">
-        <v>367</v>
       </c>
       <c r="M2" s="1" t="s">
         <v>8</v>
@@ -2931,7 +2938,7 @@
     <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" s="2"/>
       <c r="B1" s="2" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="C1" s="2"/>
       <c r="D1" s="2"/>
@@ -2943,22 +2950,22 @@
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>99</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="D2" s="1" t="s">
+        <v>373</v>
+      </c>
+      <c r="E2" s="1" t="s">
         <v>374</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="F2" s="1" t="s">
         <v>375</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>376</v>
       </c>
       <c r="G2" s="1"/>
       <c r="H2" s="1"/>
@@ -2996,12 +3003,12 @@
   <sheetData>
     <row r="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="H1" s="2" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
     </row>
     <row r="2" spans="1:17" s="6" customFormat="1" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2" s="6" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="C2" s="6" t="s">
         <v>268</v>
@@ -3010,43 +3017,43 @@
         <v>276</v>
       </c>
       <c r="E2" t="s">
+        <v>324</v>
+      </c>
+      <c r="F2" s="6" t="s">
         <v>325</v>
       </c>
-      <c r="F2" s="6" t="s">
+      <c r="G2" s="6" t="s">
         <v>326</v>
-      </c>
-      <c r="G2" s="6" t="s">
-        <v>327</v>
       </c>
       <c r="H2" s="1" t="s">
         <v>116</v>
       </c>
       <c r="I2" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="J2" s="6" t="s">
+        <v>327</v>
+      </c>
+      <c r="K2" t="s">
         <v>328</v>
       </c>
-      <c r="K2" t="s">
+      <c r="L2" t="s">
         <v>329</v>
       </c>
-      <c r="L2" t="s">
+      <c r="M2" t="s">
         <v>330</v>
       </c>
-      <c r="M2" t="s">
+      <c r="N2" t="s">
         <v>331</v>
-      </c>
-      <c r="N2" t="s">
-        <v>332</v>
       </c>
       <c r="O2" t="s">
         <v>102</v>
       </c>
       <c r="P2" t="s">
+        <v>346</v>
+      </c>
+      <c r="Q2" t="s">
         <v>347</v>
-      </c>
-      <c r="Q2" t="s">
-        <v>348</v>
       </c>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.25">
@@ -3057,7 +3064,7 @@
         <v>271</v>
       </c>
       <c r="C3" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="D3" t="s">
         <v>284</v>
@@ -3082,13 +3089,13 @@
         <v>291</v>
       </c>
       <c r="K3" t="s">
+        <v>333</v>
+      </c>
+      <c r="L3" t="s">
         <v>334</v>
       </c>
-      <c r="L3" t="s">
+      <c r="M3" t="s">
         <v>335</v>
-      </c>
-      <c r="M3" t="s">
-        <v>336</v>
       </c>
       <c r="N3" t="s">
         <v>128</v>
@@ -3097,10 +3104,10 @@
         <v>106</v>
       </c>
       <c r="P3" t="s">
+        <v>348</v>
+      </c>
+      <c r="Q3" t="s">
         <v>349</v>
-      </c>
-      <c r="Q3" t="s">
-        <v>350</v>
       </c>
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.25">
@@ -3139,30 +3146,30 @@
         <v>103</v>
       </c>
       <c r="L4" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="M4" t="s">
         <v>105</v>
       </c>
       <c r="O4" t="s">
+        <v>350</v>
+      </c>
+      <c r="P4" t="s">
         <v>351</v>
       </c>
-      <c r="P4" t="s">
+      <c r="Q4" t="s">
         <v>352</v>
-      </c>
-      <c r="Q4" t="s">
-        <v>353</v>
       </c>
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.25">
       <c r="E5" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="F5" t="s">
         <v>20</v>
       </c>
       <c r="G5" s="13" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="H5" t="s">
         <v>161</v>
@@ -3175,18 +3182,21 @@
         <v>105</v>
       </c>
       <c r="O5" t="s">
+        <v>353</v>
+      </c>
+      <c r="Q5" t="s">
         <v>354</v>
       </c>
-      <c r="Q5" t="s">
-        <v>355</v>
-      </c>
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="E6" t="s">
+        <v>274</v>
+      </c>
       <c r="F6" t="s">
         <v>27</v>
       </c>
       <c r="G6" s="13" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="H6" t="s">
         <v>162</v>
@@ -3196,10 +3206,10 @@
         <v>4</v>
       </c>
       <c r="O6" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="Q6" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
     </row>
     <row r="7" spans="1:17" x14ac:dyDescent="0.25">
@@ -3214,10 +3224,10 @@
         <v>4</v>
       </c>
       <c r="O7" t="s">
+        <v>356</v>
+      </c>
+      <c r="Q7" t="s">
         <v>357</v>
-      </c>
-      <c r="Q7" t="s">
-        <v>358</v>
       </c>
     </row>
     <row r="8" spans="1:17" x14ac:dyDescent="0.25">
@@ -3282,7 +3292,7 @@
     </row>
     <row r="13" spans="1:17" x14ac:dyDescent="0.25">
       <c r="F13" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="H13" s="30" t="s">
         <v>169</v>
@@ -3294,7 +3304,7 @@
     </row>
     <row r="14" spans="1:17" x14ac:dyDescent="0.25">
       <c r="F14" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="H14" s="30" t="s">
         <v>170</v>
@@ -3318,7 +3328,7 @@
     </row>
     <row r="16" spans="1:17" x14ac:dyDescent="0.25">
       <c r="F16" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="H16" s="30" t="s">
         <v>172</v>
@@ -3436,7 +3446,7 @@
         <v>12</v>
       </c>
       <c r="B3" t="s">
-        <v>11</v>
+        <v>21</v>
       </c>
       <c r="C3" s="4" t="s">
         <v>59</v>
@@ -3465,7 +3475,7 @@
         <v>12</v>
       </c>
       <c r="B4" t="s">
-        <v>11</v>
+        <v>21</v>
       </c>
       <c r="C4" s="4" t="s">
         <v>66</v>
@@ -3603,7 +3613,7 @@
         <v>28</v>
       </c>
       <c r="B10" t="s">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="C10" s="4" t="s">
         <v>89</v>
@@ -3689,7 +3699,7 @@
   <dimension ref="A1:M20"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="3" max="3" width="15.28515625" customWidth="1"/>
+    <col min="3" max="3" width="20.85546875" customWidth="1"/>
     <col min="4" max="4" width="14.5703125" customWidth="1"/>
   </cols>
   <sheetData>
@@ -3704,7 +3714,7 @@
         <v>98</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
     </row>
     <row r="2" spans="1:13" ht="30" x14ac:dyDescent="0.25">
@@ -3727,7 +3737,7 @@
         <v>245</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="H2" s="1" t="s">
         <v>241</v>
@@ -3761,13 +3771,13 @@
         <v>106</v>
       </c>
       <c r="F3" t="s">
+        <v>380</v>
+      </c>
+      <c r="G3" t="s">
         <v>381</v>
       </c>
-      <c r="G3" t="s">
+      <c r="H3" t="s">
         <v>382</v>
-      </c>
-      <c r="H3" t="s">
-        <v>383</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
@@ -3787,10 +3797,10 @@
         <v>106</v>
       </c>
       <c r="G4" t="s">
+        <v>383</v>
+      </c>
+      <c r="I4" t="s">
         <v>384</v>
-      </c>
-      <c r="I4" t="s">
-        <v>385</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
@@ -3814,13 +3824,13 @@
         <v>106</v>
       </c>
       <c r="F6" t="s">
+        <v>380</v>
+      </c>
+      <c r="G6" t="s">
         <v>381</v>
       </c>
-      <c r="G6" t="s">
+      <c r="H6" t="s">
         <v>382</v>
-      </c>
-      <c r="H6" t="s">
-        <v>383</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
@@ -3840,10 +3850,10 @@
         <v>106</v>
       </c>
       <c r="G7" t="s">
+        <v>383</v>
+      </c>
+      <c r="I7" t="s">
         <v>384</v>
-      </c>
-      <c r="I7" t="s">
-        <v>385</v>
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.25">
@@ -3867,13 +3877,13 @@
         <v>106</v>
       </c>
       <c r="F9" t="s">
+        <v>380</v>
+      </c>
+      <c r="G9" t="s">
         <v>381</v>
       </c>
-      <c r="G9" t="s">
+      <c r="H9" t="s">
         <v>382</v>
-      </c>
-      <c r="H9" t="s">
-        <v>383</v>
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.25">
@@ -3893,10 +3903,10 @@
         <v>106</v>
       </c>
       <c r="G10" t="s">
+        <v>383</v>
+      </c>
+      <c r="I10" t="s">
         <v>384</v>
-      </c>
-      <c r="I10" t="s">
-        <v>385</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.25">
@@ -3955,16 +3965,16 @@
         <v>106</v>
       </c>
       <c r="F17" t="s">
+        <v>380</v>
+      </c>
+      <c r="G17" t="s">
         <v>381</v>
       </c>
-      <c r="G17" t="s">
+      <c r="H17" t="s">
         <v>382</v>
       </c>
-      <c r="H17" t="s">
-        <v>383</v>
-      </c>
       <c r="K17" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.25">
@@ -3984,10 +3994,10 @@
         <v>106</v>
       </c>
       <c r="G18" t="s">
+        <v>383</v>
+      </c>
+      <c r="I18" t="s">
         <v>384</v>
-      </c>
-      <c r="I18" t="s">
-        <v>385</v>
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.25">
@@ -4085,7 +4095,7 @@
         <v>188</v>
       </c>
       <c r="N2" s="1" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="O2" s="1" t="s">
         <v>189</v>
@@ -4099,7 +4109,7 @@
         <v>55</v>
       </c>
       <c r="C3" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="D3" t="s">
         <v>191</v>
@@ -4233,7 +4243,7 @@
         <v>201</v>
       </c>
       <c r="C7" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="D7" t="s">
         <v>196</v>
@@ -4353,7 +4363,7 @@
         <v>52</v>
       </c>
       <c r="C11" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="D11" t="s">
         <v>196</v>
@@ -4388,7 +4398,7 @@
         <v>53</v>
       </c>
       <c r="C12" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="D12" t="s">
         <v>196</v>
@@ -4423,7 +4433,7 @@
         <v>54</v>
       </c>
       <c r="C13" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="D13" t="s">
         <v>196</v>
@@ -4598,7 +4608,7 @@
         <v>46</v>
       </c>
       <c r="C18" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="D18" t="s">
         <v>196</v>
@@ -4633,7 +4643,7 @@
         <v>226</v>
       </c>
       <c r="C19" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="D19" t="s">
         <v>196</v>
@@ -4741,7 +4751,7 @@
         <v>235</v>
       </c>
       <c r="C22" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="D22" t="s">
         <v>196</v>
@@ -4770,7 +4780,7 @@
         <v>237</v>
       </c>
       <c r="C23" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="D23" t="s">
         <v>231</v>
@@ -4885,7 +4895,7 @@
     </row>
     <row r="27" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B27" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="C27" t="s">
         <v>1</v>
@@ -4998,7 +5008,7 @@
         <v>250</v>
       </c>
       <c r="C31" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="D31" t="s">
         <v>196</v>
@@ -6191,7 +6201,7 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C4" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
@@ -6202,10 +6212,10 @@
         <v>255</v>
       </c>
       <c r="C5" s="12" t="s">
+        <v>388</v>
+      </c>
+      <c r="D5" s="1" t="s">
         <v>389</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>390</v>
       </c>
       <c r="E5" s="1" t="s">
         <v>157</v>
@@ -6653,7 +6663,7 @@
         <v>280</v>
       </c>
       <c r="H2" s="8" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -6694,7 +6704,7 @@
         <v>283</v>
       </c>
       <c r="H4" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -6720,7 +6730,7 @@
         <v>87</v>
       </c>
       <c r="H5" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -6739,12 +6749,14 @@
       <c r="E6" s="31" t="s">
         <v>273</v>
       </c>
-      <c r="F6" s="31"/>
+      <c r="F6" s="31" t="s">
+        <v>274</v>
+      </c>
       <c r="G6" s="31">
         <v>1</v>
       </c>
       <c r="H6" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
@@ -6764,13 +6776,13 @@
         <v>270</v>
       </c>
       <c r="F7" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="G7" t="s">
         <v>283</v>
       </c>
       <c r="H7" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
@@ -6796,7 +6808,7 @@
         <v>0.2</v>
       </c>
       <c r="H8" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -6815,12 +6827,14 @@
       <c r="E9" s="31" t="s">
         <v>273</v>
       </c>
-      <c r="F9" s="31"/>
+      <c r="F9" s="31" t="s">
+        <v>274</v>
+      </c>
       <c r="G9" s="31">
         <v>1</v>
       </c>
       <c r="H9" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
     </row>
     <row r="21" spans="8:8" x14ac:dyDescent="0.25">
@@ -6850,7 +6864,7 @@
       <formula>"Final"</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="3">
+  <dataValidations count="4">
     <dataValidation type="list" showInputMessage="1" showErrorMessage="1" prompt="Select well name from &quot;Well settings&quot; sheet " sqref="C3:C38" xr:uid="{00000000-0002-0000-0800-000000000000}">
       <formula1>WellNames</formula1>
     </dataValidation>
@@ -6858,6 +6872,9 @@
       <formula1>FluidNames</formula1>
     </dataValidation>
     <dataValidation showInputMessage="1" showErrorMessage="1" prompt="'1.0' (or other number) for constant saturation (Volume fraction)_x000a_'complement' for complement volume fraction _x000a_log name, e.g. SW, for using a log for volume fraction" sqref="G3:G39" xr:uid="{00000000-0002-0000-0800-000002000000}"/>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F3:F26" xr:uid="{4C19012F-49C5-43F5-A296-8CC8E33A6DE3}">
+      <formula1>FluidTypes</formula1>
+    </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Ongoing work. Introduced a new fluids_and_minerals.py library that is intended to replace fluids_new.py and minerals_new.py
</commit_message>
<xml_diff>
--- a/excels/project_table_new.xlsx
+++ b/excels/project_table_new.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="T:\Python\EMB\blixt_rp\excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE2D827C-0E2B-4F55-B610-6C2A742D08A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4FACC36E-0721-4EE3-A59C-47CFE26A7F3E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="685" firstSheet="7" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="685" firstSheet="5" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Well settings" sheetId="1" r:id="rId1"/>
@@ -64,7 +64,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="982" uniqueCount="396">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1024" uniqueCount="397">
   <si>
     <t>Select Yes or No</t>
   </si>
@@ -1261,6 +1261,9 @@
   </si>
   <si>
     <t>"log_name" "operator" "limit(s)" "[units]"</t>
+  </si>
+  <si>
+    <t>TESTFLUID</t>
   </si>
 </sst>
 </file>
@@ -1980,13 +1983,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:I13"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" customWidth="1"/>
-    <col min="2" max="2" width="12.42578125" customWidth="1"/>
+    <col min="1" max="1" width="5.6640625" customWidth="1"/>
+    <col min="2" max="2" width="12.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1997,7 +2000,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:9" s="1" customFormat="1" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" s="1" customFormat="1" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
@@ -2026,7 +2029,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>21</v>
       </c>
@@ -2046,7 +2049,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>21</v>
       </c>
@@ -2060,7 +2063,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>21</v>
       </c>
@@ -2074,7 +2077,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>21</v>
       </c>
@@ -2088,7 +2091,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>21</v>
       </c>
@@ -2102,7 +2105,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>11</v>
       </c>
@@ -2122,7 +2125,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>21</v>
       </c>
@@ -2139,7 +2142,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>21</v>
       </c>
@@ -2153,7 +2156,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
       <c r="C11" s="21" t="s">
         <v>35</v>
       </c>
@@ -2161,7 +2164,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
       <c r="C12" s="22" t="s">
         <v>37</v>
       </c>
@@ -2169,7 +2172,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
       <c r="C13" s="23" t="s">
         <v>39</v>
       </c>
@@ -2193,13 +2196,13 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
   <dimension ref="A1:G33"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="17.42578125" customWidth="1"/>
+    <col min="1" max="1" width="17.44140625" customWidth="1"/>
     <col min="6" max="6" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" ht="26.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="F1" s="7" t="s">
         <v>286</v>
       </c>
@@ -2207,7 +2210,7 @@
         <v>395</v>
       </c>
     </row>
-    <row r="2" spans="1:7" s="8" customFormat="1" ht="30.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" s="8" customFormat="1" ht="30.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="33" t="s">
         <v>255</v>
       </c>
@@ -2230,7 +2233,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>289</v>
       </c>
@@ -2247,7 +2250,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>290</v>
       </c>
@@ -2270,7 +2273,7 @@
         <v>394</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>292</v>
       </c>
@@ -2287,7 +2290,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>293</v>
       </c>
@@ -2304,7 +2307,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>294</v>
       </c>
@@ -2321,7 +2324,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>295</v>
       </c>
@@ -2338,7 +2341,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>296</v>
       </c>
@@ -2355,7 +2358,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>297</v>
       </c>
@@ -2372,7 +2375,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>298</v>
       </c>
@@ -2389,7 +2392,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>299</v>
       </c>
@@ -2406,7 +2409,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>300</v>
       </c>
@@ -2423,7 +2426,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>301</v>
       </c>
@@ -2440,7 +2443,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>302</v>
       </c>
@@ -2457,7 +2460,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>303</v>
       </c>
@@ -2474,7 +2477,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>304</v>
       </c>
@@ -2491,7 +2494,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>305</v>
       </c>
@@ -2508,7 +2511,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>306</v>
       </c>
@@ -2525,7 +2528,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>307</v>
       </c>
@@ -2542,7 +2545,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>308</v>
       </c>
@@ -2559,7 +2562,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>309</v>
       </c>
@@ -2576,7 +2579,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>310</v>
       </c>
@@ -2593,7 +2596,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>311</v>
       </c>
@@ -2610,7 +2613,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>312</v>
       </c>
@@ -2627,7 +2630,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>313</v>
       </c>
@@ -2644,7 +2647,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>314</v>
       </c>
@@ -2661,7 +2664,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>315</v>
       </c>
@@ -2678,7 +2681,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>316</v>
       </c>
@@ -2695,7 +2698,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>317</v>
       </c>
@@ -2712,7 +2715,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>318</v>
       </c>
@@ -2729,7 +2732,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>319</v>
       </c>
@@ -2746,7 +2749,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>320</v>
       </c>
@@ -2772,19 +2775,19 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
   <dimension ref="A1:D4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="2" width="10.28515625" customWidth="1"/>
-    <col min="3" max="3" width="17.42578125" customWidth="1"/>
+    <col min="1" max="2" width="10.33203125" customWidth="1"/>
+    <col min="3" max="3" width="17.44140625" customWidth="1"/>
     <col min="4" max="4" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" ht="26.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D1" s="5" t="s">
         <v>321</v>
       </c>
     </row>
-    <row r="2" spans="1:4" s="8" customFormat="1" ht="30.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" s="8" customFormat="1" ht="30.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="9" t="s">
         <v>277</v>
       </c>
@@ -2798,7 +2801,7 @@
         <v>280</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>28</v>
       </c>
@@ -2812,7 +2815,7 @@
         <v>283</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>28</v>
       </c>
@@ -2857,9 +2860,9 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CCD9C215-DCD2-40A2-A7D5-172DC530BE0E}">
   <dimension ref="A1:Q2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.3">
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
       <c r="D1" s="2"/>
@@ -2880,7 +2883,7 @@
       </c>
       <c r="O1" s="2"/>
     </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>371</v>
       </c>
@@ -2933,9 +2936,9 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3CCC2506-3BD3-4476-A9AA-1673C259914E}">
   <dimension ref="A1:M2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A1" s="2"/>
       <c r="B1" s="2" t="s">
         <v>376</v>
@@ -2948,7 +2951,7 @@
       <c r="I1" s="2"/>
       <c r="K1" s="2"/>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>372</v>
       </c>
@@ -2994,19 +2997,19 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
   <dimension ref="A1:Q18"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="16.28515625" customWidth="1"/>
-    <col min="3" max="3" width="12.28515625" customWidth="1"/>
-    <col min="4" max="4" width="9.85546875" customWidth="1"/>
+    <col min="2" max="2" width="16.33203125" customWidth="1"/>
+    <col min="3" max="3" width="12.33203125" customWidth="1"/>
+    <col min="4" max="4" width="9.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.3">
       <c r="H1" s="2" t="s">
         <v>359</v>
       </c>
     </row>
-    <row r="2" spans="1:17" s="6" customFormat="1" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:17" s="6" customFormat="1" ht="42.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B2" s="6" t="s">
         <v>323</v>
       </c>
@@ -3056,7 +3059,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>11</v>
       </c>
@@ -3110,7 +3113,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>21</v>
       </c>
@@ -3161,7 +3164,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:17" x14ac:dyDescent="0.3">
       <c r="E5" t="s">
         <v>337</v>
       </c>
@@ -3188,7 +3191,7 @@
         <v>354</v>
       </c>
     </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:17" x14ac:dyDescent="0.3">
       <c r="E6" t="s">
         <v>274</v>
       </c>
@@ -3212,7 +3215,7 @@
         <v>355</v>
       </c>
     </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:17" x14ac:dyDescent="0.3">
       <c r="F7" t="s">
         <v>30</v>
       </c>
@@ -3230,7 +3233,7 @@
         <v>357</v>
       </c>
     </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:17" x14ac:dyDescent="0.3">
       <c r="F8" t="s">
         <v>33</v>
       </c>
@@ -3242,7 +3245,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:17" x14ac:dyDescent="0.3">
       <c r="F9" t="s">
         <v>24</v>
       </c>
@@ -3254,7 +3257,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="10" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:17" x14ac:dyDescent="0.3">
       <c r="F10" t="s">
         <v>36</v>
       </c>
@@ -3266,7 +3269,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:17" x14ac:dyDescent="0.3">
       <c r="F11" t="s">
         <v>38</v>
       </c>
@@ -3278,7 +3281,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:17" x14ac:dyDescent="0.3">
       <c r="F12" t="s">
         <v>40</v>
       </c>
@@ -3290,7 +3293,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:17" x14ac:dyDescent="0.3">
       <c r="F13" t="s">
         <v>340</v>
       </c>
@@ -3302,7 +3305,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:17" x14ac:dyDescent="0.3">
       <c r="F14" t="s">
         <v>341</v>
       </c>
@@ -3314,7 +3317,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:17" x14ac:dyDescent="0.3">
       <c r="F15" t="s">
         <v>121</v>
       </c>
@@ -3326,7 +3329,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:17" x14ac:dyDescent="0.3">
       <c r="F16" t="s">
         <v>342</v>
       </c>
@@ -3338,7 +3341,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="8:9" x14ac:dyDescent="0.25">
+    <row r="17" spans="8:9" x14ac:dyDescent="0.3">
       <c r="H17" s="30" t="s">
         <v>173</v>
       </c>
@@ -3347,7 +3350,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="8:9" x14ac:dyDescent="0.25">
+    <row r="18" spans="8:9" x14ac:dyDescent="0.3">
       <c r="H18" s="30" t="s">
         <v>174</v>
       </c>
@@ -3365,19 +3368,19 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:R11"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="2" width="9.7109375" style="13" customWidth="1"/>
-    <col min="3" max="3" width="15.85546875" customWidth="1"/>
-    <col min="4" max="5" width="11.5703125" customWidth="1"/>
+    <col min="1" max="2" width="9.6640625" style="13" customWidth="1"/>
+    <col min="3" max="3" width="15.88671875" customWidth="1"/>
+    <col min="4" max="5" width="11.5546875" customWidth="1"/>
     <col min="6" max="7" width="10" customWidth="1"/>
-    <col min="11" max="11" width="16.140625" customWidth="1"/>
+    <col min="11" max="11" width="16.109375" customWidth="1"/>
     <col min="13" max="13" width="7" customWidth="1"/>
-    <col min="16" max="16" width="6.5703125" customWidth="1"/>
-    <col min="17" max="17" width="4.7109375" customWidth="1"/>
+    <col min="16" max="16" width="6.5546875" customWidth="1"/>
+    <col min="17" max="17" width="4.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A1" s="11" t="s">
         <v>41</v>
       </c>
@@ -3385,7 +3388,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="2" spans="1:18" s="1" customFormat="1" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:18" s="1" customFormat="1" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="12" t="s">
         <v>3</v>
       </c>
@@ -3441,7 +3444,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A3" s="13" t="s">
         <v>12</v>
       </c>
@@ -3470,7 +3473,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A4" s="13" t="s">
         <v>12</v>
       </c>
@@ -3487,7 +3490,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A5" s="13" t="s">
         <v>15</v>
       </c>
@@ -3513,7 +3516,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A6" s="13" t="s">
         <v>18</v>
       </c>
@@ -3539,7 +3542,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A7" s="13" t="s">
         <v>22</v>
       </c>
@@ -3568,7 +3571,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A8" s="13" t="s">
         <v>25</v>
       </c>
@@ -3585,7 +3588,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A9" s="13" t="s">
         <v>25</v>
       </c>
@@ -3608,7 +3611,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A10" s="13" t="s">
         <v>28</v>
       </c>
@@ -3640,7 +3643,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A11" s="13" t="s">
         <v>31</v>
       </c>
@@ -3697,13 +3700,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{725EDE5F-2F74-4F10-B375-EE1EEF8AD52D}">
   <dimension ref="A1:M20"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="3" max="3" width="20.85546875" customWidth="1"/>
-    <col min="4" max="4" width="14.5703125" customWidth="1"/>
+    <col min="3" max="3" width="20.88671875" customWidth="1"/>
+    <col min="4" max="4" width="14.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A1" s="11" t="s">
         <v>41</v>
       </c>
@@ -3717,7 +3720,7 @@
         <v>379</v>
       </c>
     </row>
-    <row r="2" spans="1:13" ht="30" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A2" s="12" t="s">
         <v>3</v>
       </c>
@@ -3754,7 +3757,7 @@
       <c r="L2" s="1"/>
       <c r="M2" s="1"/>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A3" s="13" t="s">
         <v>12</v>
       </c>
@@ -3780,7 +3783,7 @@
         <v>382</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A4" s="13" t="s">
         <v>12</v>
       </c>
@@ -3803,11 +3806,11 @@
         <v>384</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A5" s="13"/>
       <c r="C5" s="4"/>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A6" s="13" t="s">
         <v>15</v>
       </c>
@@ -3833,7 +3836,7 @@
         <v>382</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A7" s="13" t="s">
         <v>15</v>
       </c>
@@ -3856,11 +3859,11 @@
         <v>384</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A8" s="13"/>
       <c r="C8" s="4"/>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A9" s="13" t="s">
         <v>18</v>
       </c>
@@ -3886,7 +3889,7 @@
         <v>382</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A10" s="13" t="s">
         <v>18</v>
       </c>
@@ -3909,11 +3912,11 @@
         <v>384</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A11" s="13"/>
       <c r="C11" s="4"/>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A12" s="13" t="s">
         <v>22</v>
       </c>
@@ -3922,11 +3925,11 @@
       </c>
       <c r="C12" s="4"/>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A13" s="13"/>
       <c r="C13" s="4"/>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A14" s="13" t="s">
         <v>25</v>
       </c>
@@ -3935,7 +3938,7 @@
       </c>
       <c r="C14" s="4"/>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A15" s="13" t="s">
         <v>25</v>
       </c>
@@ -3944,11 +3947,11 @@
       </c>
       <c r="C15" s="4"/>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A16" s="13"/>
       <c r="C16" s="4"/>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A17" s="13" t="s">
         <v>28</v>
       </c>
@@ -3977,7 +3980,7 @@
         <v>385</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A18" s="13" t="s">
         <v>28</v>
       </c>
@@ -4000,11 +4003,11 @@
         <v>384</v>
       </c>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A19" s="13"/>
       <c r="C19" s="4"/>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A20" s="13" t="s">
         <v>31</v>
       </c>
@@ -4042,19 +4045,19 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:O31"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="11.42578125" customWidth="1"/>
-    <col min="2" max="2" width="14.140625" customWidth="1"/>
-    <col min="3" max="3" width="14.5703125" customWidth="1"/>
+    <col min="1" max="1" width="11.44140625" customWidth="1"/>
+    <col min="2" max="2" width="14.109375" customWidth="1"/>
+    <col min="3" max="3" width="14.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>175</v>
       </c>
     </row>
-    <row r="2" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>176</v>
       </c>
@@ -4101,7 +4104,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>190</v>
       </c>
@@ -4136,7 +4139,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
       <c r="B4" t="s">
         <v>45</v>
       </c>
@@ -4168,7 +4171,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
       <c r="B5" t="s">
         <v>47</v>
       </c>
@@ -4200,7 +4203,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>197</v>
       </c>
@@ -4235,7 +4238,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>200</v>
       </c>
@@ -4270,7 +4273,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>202</v>
       </c>
@@ -4305,7 +4308,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.3">
       <c r="B9" t="s">
         <v>206</v>
       </c>
@@ -4330,7 +4333,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.3">
       <c r="B10" t="s">
         <v>208</v>
       </c>
@@ -4355,7 +4358,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>209</v>
       </c>
@@ -4390,7 +4393,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>210</v>
       </c>
@@ -4425,7 +4428,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>213</v>
       </c>
@@ -4460,7 +4463,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>77</v>
       </c>
@@ -4495,7 +4498,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>215</v>
       </c>
@@ -4530,7 +4533,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>218</v>
       </c>
@@ -4565,7 +4568,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>221</v>
       </c>
@@ -4600,7 +4603,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>224</v>
       </c>
@@ -4635,7 +4638,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>225</v>
       </c>
@@ -4670,7 +4673,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>227</v>
       </c>
@@ -4705,7 +4708,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>229</v>
       </c>
@@ -4743,7 +4746,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>234</v>
       </c>
@@ -4772,7 +4775,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>236</v>
       </c>
@@ -4807,7 +4810,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>240</v>
       </c>
@@ -4838,7 +4841,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>243</v>
       </c>
@@ -4873,7 +4876,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:13" x14ac:dyDescent="0.3">
       <c r="B26" t="s">
         <v>57</v>
       </c>
@@ -4893,7 +4896,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:13" x14ac:dyDescent="0.3">
       <c r="B27" t="s">
         <v>378</v>
       </c>
@@ -4919,7 +4922,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:13" x14ac:dyDescent="0.3">
       <c r="B28" t="s">
         <v>245</v>
       </c>
@@ -4945,7 +4948,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>246</v>
       </c>
@@ -4974,7 +4977,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>248</v>
       </c>
@@ -5003,7 +5006,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:13" x14ac:dyDescent="0.3">
       <c r="B31" t="s">
         <v>250</v>
       </c>
@@ -5043,13 +5046,13 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:M17"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
-    <col min="6" max="6" width="15.5703125" customWidth="1"/>
+    <col min="6" max="6" width="15.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A1" s="2"/>
       <c r="B1" s="2" t="s">
         <v>112</v>
@@ -5066,7 +5069,7 @@
       <c r="I1" s="2"/>
       <c r="K1" s="2"/>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>115</v>
       </c>
@@ -5107,7 +5110,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>125</v>
       </c>
@@ -5133,7 +5136,7 @@
         <v>-18877.708702820371</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>131</v>
       </c>
@@ -5159,7 +5162,7 @@
         <v>-19045.139985898601</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>133</v>
       </c>
@@ -5185,7 +5188,7 @@
         <v>-5.4445188599886638</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>135</v>
       </c>
@@ -5211,7 +5214,7 @@
         <v>2.671411511624413</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>137</v>
       </c>
@@ -5237,7 +5240,7 @@
         <v>9.5532474786010475</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>125</v>
       </c>
@@ -5263,7 +5266,7 @@
         <v>2866.0938229725748</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>131</v>
       </c>
@@ -5289,7 +5292,7 @@
         <v>1490.761502865475</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>133</v>
       </c>
@@ -5315,7 +5318,7 @@
         <v>2.217459469264154</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>135</v>
       </c>
@@ -5341,7 +5344,7 @@
         <v>0.2337935274525294</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>137</v>
       </c>
@@ -5367,7 +5370,7 @@
         <v>2.0873115011979051E-2</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>125</v>
       </c>
@@ -5393,7 +5396,7 @@
         <v>1351.711647219304</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>131</v>
       </c>
@@ -5419,7 +5422,7 @@
         <v>150.9391394665019</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>133</v>
       </c>
@@ -5445,7 +5448,7 @@
         <v>1.940117188288828</v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>135</v>
       </c>
@@ -5471,7 +5474,7 @@
         <v>-2.0146865510893688E-2</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>137</v>
       </c>
@@ -5505,22 +5508,22 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:G42"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="3" max="3" width="16.7109375" customWidth="1"/>
+    <col min="3" max="3" width="16.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>153</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="5" spans="1:7" s="1" customFormat="1" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" s="1" customFormat="1" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>2</v>
       </c>
@@ -5543,7 +5546,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B6" t="s">
         <v>12</v>
       </c>
@@ -5563,7 +5566,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="7" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="B7" t="s">
         <v>12</v>
       </c>
@@ -5580,7 +5583,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="8" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="B8" t="s">
         <v>12</v>
       </c>
@@ -5597,7 +5600,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="9" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="B9" t="s">
         <v>12</v>
       </c>
@@ -5614,7 +5617,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="10" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="B10" t="s">
         <v>12</v>
       </c>
@@ -5631,7 +5634,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="11" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="B11" t="s">
         <v>12</v>
       </c>
@@ -5648,7 +5651,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B12" t="s">
         <v>12</v>
       </c>
@@ -5665,7 +5668,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B13" t="s">
         <v>15</v>
       </c>
@@ -5682,7 +5685,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="14" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="B14" t="s">
         <v>15</v>
       </c>
@@ -5699,7 +5702,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="15" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="B15" t="s">
         <v>15</v>
       </c>
@@ -5716,7 +5719,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="16" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="B16" t="s">
         <v>15</v>
       </c>
@@ -5733,7 +5736,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="17" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B17" t="s">
         <v>15</v>
       </c>
@@ -5750,7 +5753,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="18" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B18" t="s">
         <v>15</v>
       </c>
@@ -5767,7 +5770,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="19" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B19" t="s">
         <v>15</v>
       </c>
@@ -5784,7 +5787,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="20" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B20" t="s">
         <v>18</v>
       </c>
@@ -5801,7 +5804,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="21" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B21" t="s">
         <v>18</v>
       </c>
@@ -5818,7 +5821,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="22" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B22" t="s">
         <v>18</v>
       </c>
@@ -5835,7 +5838,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="23" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B23" t="s">
         <v>18</v>
       </c>
@@ -5852,7 +5855,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="24" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B24" t="s">
         <v>18</v>
       </c>
@@ -5869,7 +5872,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="25" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B25" t="s">
         <v>18</v>
       </c>
@@ -5886,7 +5889,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="26" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B26" t="s">
         <v>18</v>
       </c>
@@ -5903,7 +5906,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="27" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B27" t="s">
         <v>28</v>
       </c>
@@ -5920,7 +5923,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="28" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B28" t="s">
         <v>28</v>
       </c>
@@ -5937,7 +5940,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="29" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B29" t="s">
         <v>28</v>
       </c>
@@ -5954,7 +5957,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="30" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B30" t="s">
         <v>28</v>
       </c>
@@ -5971,7 +5974,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="31" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B31" t="s">
         <v>28</v>
       </c>
@@ -5988,7 +5991,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="32" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B32" t="s">
         <v>28</v>
       </c>
@@ -6005,7 +6008,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="33" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B33" t="s">
         <v>28</v>
       </c>
@@ -6022,7 +6025,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="34" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B34" t="s">
         <v>31</v>
       </c>
@@ -6039,7 +6042,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="35" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B35" t="s">
         <v>31</v>
       </c>
@@ -6056,7 +6059,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="36" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B36" t="s">
         <v>31</v>
       </c>
@@ -6073,7 +6076,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="37" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B37" t="s">
         <v>31</v>
       </c>
@@ -6090,7 +6093,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="38" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B38" t="s">
         <v>31</v>
       </c>
@@ -6107,7 +6110,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="39" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B39" t="s">
         <v>31</v>
       </c>
@@ -6124,7 +6127,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="40" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B40" t="s">
         <v>31</v>
       </c>
@@ -6141,7 +6144,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="41" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="41" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B41" t="s">
         <v>31</v>
       </c>
@@ -6158,7 +6161,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="42" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="42" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B42" t="s">
         <v>31</v>
       </c>
@@ -6192,19 +6195,19 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9DE0C751-ACC1-462A-82AF-4CE9BB91C06B}">
   <dimension ref="A2:G21"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="C4" t="s">
         <v>390</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>2</v>
       </c>
@@ -6227,7 +6230,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>21</v>
       </c>
@@ -6241,7 +6244,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>11</v>
       </c>
@@ -6255,7 +6258,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>11</v>
       </c>
@@ -6269,7 +6272,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>11</v>
       </c>
@@ -6283,7 +6286,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>11</v>
       </c>
@@ -6297,7 +6300,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>11</v>
       </c>
@@ -6311,7 +6314,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>21</v>
       </c>
@@ -6325,7 +6328,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>11</v>
       </c>
@@ -6339,7 +6342,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>11</v>
       </c>
@@ -6353,7 +6356,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>11</v>
       </c>
@@ -6367,7 +6370,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>11</v>
       </c>
@@ -6381,7 +6384,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>11</v>
       </c>
@@ -6395,7 +6398,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>11</v>
       </c>
@@ -6409,7 +6412,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>11</v>
       </c>
@@ -6423,7 +6426,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>11</v>
       </c>
@@ -6437,7 +6440,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>11</v>
       </c>
@@ -6467,25 +6470,25 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:O8"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="8.5703125" customWidth="1"/>
+    <col min="1" max="1" width="8.5546875" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
-    <col min="3" max="3" width="12.85546875" customWidth="1"/>
+    <col min="3" max="3" width="12.88671875" customWidth="1"/>
     <col min="4" max="4" width="10" customWidth="1"/>
-    <col min="6" max="6" width="6.7109375" customWidth="1"/>
-    <col min="7" max="7" width="6.5703125" customWidth="1"/>
-    <col min="8" max="8" width="8.28515625" customWidth="1"/>
-    <col min="9" max="9" width="5.5703125" customWidth="1"/>
-    <col min="10" max="10" width="6.5703125" customWidth="1"/>
-    <col min="11" max="11" width="6.140625" customWidth="1"/>
-    <col min="12" max="12" width="5.140625" customWidth="1"/>
-    <col min="13" max="13" width="5.5703125" customWidth="1"/>
-    <col min="14" max="14" width="5.140625" customWidth="1"/>
-    <col min="15" max="15" width="4.42578125" customWidth="1"/>
+    <col min="6" max="6" width="6.6640625" customWidth="1"/>
+    <col min="7" max="7" width="6.5546875" customWidth="1"/>
+    <col min="8" max="8" width="8.33203125" customWidth="1"/>
+    <col min="9" max="9" width="5.5546875" customWidth="1"/>
+    <col min="10" max="10" width="6.5546875" customWidth="1"/>
+    <col min="11" max="11" width="6.109375" customWidth="1"/>
+    <col min="12" max="12" width="5.109375" customWidth="1"/>
+    <col min="13" max="13" width="5.5546875" customWidth="1"/>
+    <col min="14" max="14" width="5.109375" customWidth="1"/>
+    <col min="15" max="15" width="4.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>253</v>
       </c>
@@ -6493,7 +6496,7 @@
         <v>254</v>
       </c>
     </row>
-    <row r="2" spans="1:15" s="8" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:15" s="8" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="8" t="s">
         <v>255</v>
       </c>
@@ -6540,7 +6543,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>270</v>
       </c>
@@ -6580,7 +6583,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>273</v>
       </c>
@@ -6595,19 +6598,55 @@
         <v>274</v>
       </c>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>396</v>
+      </c>
       <c r="B5" s="3"/>
       <c r="C5" s="3"/>
-    </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="E5" t="s">
+        <v>271</v>
+      </c>
+      <c r="F5">
+        <v>0.03</v>
+      </c>
+      <c r="G5">
+        <v>5</v>
+      </c>
+      <c r="H5">
+        <v>1.0699999999999999E-2</v>
+      </c>
+      <c r="I5">
+        <v>0</v>
+      </c>
+      <c r="J5">
+        <v>70000</v>
+      </c>
+      <c r="K5">
+        <v>1</v>
+      </c>
+      <c r="L5">
+        <v>30</v>
+      </c>
+      <c r="M5">
+        <v>0.6</v>
+      </c>
+      <c r="N5" t="s">
+        <v>272</v>
+      </c>
+      <c r="O5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
       <c r="B7" s="3"/>
       <c r="C7" s="3"/>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.3">
       <c r="B8" s="3"/>
       <c r="C8" s="3"/>
     </row>
@@ -6626,13 +6665,13 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
   <dimension ref="A1:H21"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="4" width="10.28515625" customWidth="1"/>
-    <col min="5" max="6" width="8.5703125" customWidth="1"/>
+    <col min="2" max="4" width="10.33203125" customWidth="1"/>
+    <col min="5" max="6" width="8.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -6640,7 +6679,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="2" spans="1:8" s="8" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" s="8" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
@@ -6666,7 +6705,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="31" t="s">
         <v>21</v>
       </c>
@@ -6681,7 +6720,7 @@
       </c>
       <c r="G3" s="32"/>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>21</v>
       </c>
@@ -6707,7 +6746,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>21</v>
       </c>
@@ -6733,7 +6772,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" s="31" t="s">
         <v>21</v>
       </c>
@@ -6759,7 +6798,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>11</v>
       </c>
@@ -6785,7 +6824,7 @@
         <v>345</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>11</v>
       </c>
@@ -6799,7 +6838,7 @@
         <v>162</v>
       </c>
       <c r="E8" t="s">
-        <v>270</v>
+        <v>396</v>
       </c>
       <c r="F8" t="s">
         <v>273</v>
@@ -6811,7 +6850,7 @@
         <v>345</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A9" s="31" t="s">
         <v>11</v>
       </c>
@@ -6837,7 +6876,145 @@
         <v>345</v>
       </c>
     </row>
-    <row r="21" spans="8:8" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>11</v>
+      </c>
+      <c r="B10" t="s">
+        <v>281</v>
+      </c>
+      <c r="C10" t="s">
+        <v>28</v>
+      </c>
+      <c r="D10" t="s">
+        <v>161</v>
+      </c>
+      <c r="E10" t="s">
+        <v>396</v>
+      </c>
+      <c r="F10" t="s">
+        <v>282</v>
+      </c>
+      <c r="G10">
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>11</v>
+      </c>
+      <c r="B11" t="s">
+        <v>281</v>
+      </c>
+      <c r="C11" t="s">
+        <v>28</v>
+      </c>
+      <c r="D11" t="s">
+        <v>161</v>
+      </c>
+      <c r="E11" t="s">
+        <v>270</v>
+      </c>
+      <c r="F11" t="s">
+        <v>273</v>
+      </c>
+      <c r="G11" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="31" t="s">
+        <v>11</v>
+      </c>
+      <c r="B12" s="31" t="s">
+        <v>284</v>
+      </c>
+      <c r="C12" s="31" t="s">
+        <v>28</v>
+      </c>
+      <c r="D12" s="31" t="s">
+        <v>161</v>
+      </c>
+      <c r="E12" s="31" t="s">
+        <v>270</v>
+      </c>
+      <c r="F12" s="31" t="s">
+        <v>273</v>
+      </c>
+      <c r="G12" s="31">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>11</v>
+      </c>
+      <c r="B13" t="s">
+        <v>281</v>
+      </c>
+      <c r="C13" t="s">
+        <v>28</v>
+      </c>
+      <c r="D13" t="s">
+        <v>163</v>
+      </c>
+      <c r="E13" t="s">
+        <v>270</v>
+      </c>
+      <c r="F13" t="s">
+        <v>282</v>
+      </c>
+      <c r="G13" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>11</v>
+      </c>
+      <c r="B14" t="s">
+        <v>281</v>
+      </c>
+      <c r="C14" t="s">
+        <v>28</v>
+      </c>
+      <c r="D14" t="s">
+        <v>163</v>
+      </c>
+      <c r="E14" t="s">
+        <v>270</v>
+      </c>
+      <c r="F14" t="s">
+        <v>273</v>
+      </c>
+      <c r="G14" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A15" s="31" t="s">
+        <v>11</v>
+      </c>
+      <c r="B15" s="31" t="s">
+        <v>284</v>
+      </c>
+      <c r="C15" s="31" t="s">
+        <v>28</v>
+      </c>
+      <c r="D15" s="31" t="s">
+        <v>163</v>
+      </c>
+      <c r="E15" s="31" t="s">
+        <v>273</v>
+      </c>
+      <c r="F15" s="31" t="s">
+        <v>274</v>
+      </c>
+      <c r="G15" s="31">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H21" t="s">
         <v>285</v>
       </c>
@@ -6864,7 +7041,7 @@
       <formula>"Final"</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="4">
+  <dataValidations count="5">
     <dataValidation type="list" showInputMessage="1" showErrorMessage="1" prompt="Select well name from &quot;Well settings&quot; sheet " sqref="C3:C38" xr:uid="{00000000-0002-0000-0800-000000000000}">
       <formula1>WellNames</formula1>
     </dataValidation>
@@ -6875,6 +7052,9 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F3:F26" xr:uid="{4C19012F-49C5-43F5-A296-8CC8E33A6DE3}">
       <formula1>FluidTypes</formula1>
     </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D3:D26" xr:uid="{7DE5147A-C027-4ABD-8AB8-B6B76F43DBCB}">
+      <formula1>IntervalNames</formula1>
+    </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Ongoing work.  Continued work on fluids_and_minerals.py library which I'm trying to generalize so that it can handle both fluids and minerals consistently
</commit_message>
<xml_diff>
--- a/excels/project_table_new.xlsx
+++ b/excels/project_table_new.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="T:\Python\EMB\blixt_rp\excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4FACC36E-0721-4EE3-A59C-47CFE26A7F3E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93759F2E-467B-4E29-84F7-FECAE662F40D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="685" firstSheet="5" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="685" firstSheet="5" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Well settings" sheetId="1" r:id="rId1"/>
@@ -64,7 +64,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1024" uniqueCount="397">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1048" uniqueCount="397">
   <si>
     <t>Select Yes or No</t>
   </si>
@@ -1475,7 +1475,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1527,11 +1527,251 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="17">
+  <dxfs count="39">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C5700"/>
@@ -1983,13 +2223,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:I13"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="5.6640625" customWidth="1"/>
-    <col min="2" max="2" width="12.44140625" customWidth="1"/>
+    <col min="1" max="1" width="5.7109375" customWidth="1"/>
+    <col min="2" max="2" width="12.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -2000,7 +2240,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:9" s="1" customFormat="1" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:9" s="1" customFormat="1" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
@@ -2029,7 +2269,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>21</v>
       </c>
@@ -2049,7 +2289,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>21</v>
       </c>
@@ -2063,7 +2303,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>21</v>
       </c>
@@ -2077,7 +2317,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>21</v>
       </c>
@@ -2091,7 +2331,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>21</v>
       </c>
@@ -2105,7 +2345,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>11</v>
       </c>
@@ -2125,7 +2365,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>21</v>
       </c>
@@ -2142,7 +2382,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>21</v>
       </c>
@@ -2156,7 +2396,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="C11" s="21" t="s">
         <v>35</v>
       </c>
@@ -2164,7 +2404,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="C12" s="22" t="s">
         <v>37</v>
       </c>
@@ -2172,7 +2412,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="C13" s="23" t="s">
         <v>39</v>
       </c>
@@ -2182,10 +2422,10 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A3:A20">
-    <cfRule type="cellIs" dxfId="16" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="38" priority="1" operator="equal">
       <formula>"Yes"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="15" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="37" priority="2" operator="equal">
       <formula>"No"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -2196,13 +2436,13 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
   <dimension ref="A1:G33"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.44140625" customWidth="1"/>
+    <col min="1" max="1" width="17.42578125" customWidth="1"/>
     <col min="6" max="6" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="26.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F1" s="7" t="s">
         <v>286</v>
       </c>
@@ -2210,7 +2450,7 @@
         <v>395</v>
       </c>
     </row>
-    <row r="2" spans="1:7" s="8" customFormat="1" ht="30.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:7" s="8" customFormat="1" ht="30.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="33" t="s">
         <v>255</v>
       </c>
@@ -2233,7 +2473,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>289</v>
       </c>
@@ -2250,7 +2490,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>290</v>
       </c>
@@ -2273,7 +2513,7 @@
         <v>394</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>292</v>
       </c>
@@ -2290,7 +2530,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>293</v>
       </c>
@@ -2307,7 +2547,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>294</v>
       </c>
@@ -2324,7 +2564,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>295</v>
       </c>
@@ -2341,7 +2581,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>296</v>
       </c>
@@ -2358,7 +2598,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>297</v>
       </c>
@@ -2375,7 +2615,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>298</v>
       </c>
@@ -2392,7 +2632,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>299</v>
       </c>
@@ -2409,7 +2649,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>300</v>
       </c>
@@ -2426,7 +2666,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>301</v>
       </c>
@@ -2443,7 +2683,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>302</v>
       </c>
@@ -2460,7 +2700,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>303</v>
       </c>
@@ -2477,7 +2717,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>304</v>
       </c>
@@ -2494,7 +2734,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>305</v>
       </c>
@@ -2511,7 +2751,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>306</v>
       </c>
@@ -2528,7 +2768,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>307</v>
       </c>
@@ -2545,7 +2785,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>308</v>
       </c>
@@ -2562,7 +2802,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>309</v>
       </c>
@@ -2579,7 +2819,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>310</v>
       </c>
@@ -2596,7 +2836,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>311</v>
       </c>
@@ -2613,7 +2853,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>312</v>
       </c>
@@ -2630,7 +2870,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>313</v>
       </c>
@@ -2647,7 +2887,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>314</v>
       </c>
@@ -2664,7 +2904,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>315</v>
       </c>
@@ -2681,7 +2921,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>316</v>
       </c>
@@ -2698,7 +2938,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>317</v>
       </c>
@@ -2715,7 +2955,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>318</v>
       </c>
@@ -2732,7 +2972,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>319</v>
       </c>
@@ -2749,7 +2989,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>320</v>
       </c>
@@ -2774,83 +3014,211 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
-  <dimension ref="A1:D4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:E8"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="2" width="10.33203125" customWidth="1"/>
-    <col min="3" max="3" width="17.44140625" customWidth="1"/>
-    <col min="4" max="4" width="12" customWidth="1"/>
+    <col min="2" max="3" width="10.28515625" customWidth="1"/>
+    <col min="4" max="4" width="17.42578125" customWidth="1"/>
+    <col min="5" max="5" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="26.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D1" s="5" t="s">
+    <row r="1" spans="1:5" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="37" t="s">
+        <v>0</v>
+      </c>
+      <c r="E1" s="5" t="s">
         <v>321</v>
       </c>
     </row>
-    <row r="2" spans="1:4" s="8" customFormat="1" ht="30.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="9" t="s">
+    <row r="2" spans="1:5" s="8" customFormat="1" ht="30.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="38" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="9" t="s">
         <v>277</v>
       </c>
-      <c r="B2" s="9" t="s">
+      <c r="C2" s="9" t="s">
         <v>116</v>
       </c>
-      <c r="C2" s="8" t="s">
+      <c r="D2" s="8" t="s">
         <v>322</v>
       </c>
-      <c r="D2" s="10" t="s">
+      <c r="E2" s="10" t="s">
         <v>280</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
+    <row r="3" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="39" t="s">
+        <v>11</v>
+      </c>
+      <c r="B3" t="s">
         <v>28</v>
       </c>
-      <c r="B3" t="s">
+      <c r="C3" t="s">
         <v>162</v>
       </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
         <v>289</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="E3" s="6" t="s">
         <v>283</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
+    <row r="4" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="41" t="s">
+        <v>11</v>
+      </c>
+      <c r="B4" s="41" t="s">
         <v>28</v>
       </c>
-      <c r="B4" t="s">
+      <c r="C4" s="41" t="s">
         <v>162</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" s="41" t="s">
         <v>290</v>
       </c>
-      <c r="D4" t="s">
+      <c r="E4" s="41" t="s">
         <v>64</v>
       </c>
     </row>
+    <row r="5" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A5" s="39" t="s">
+        <v>11</v>
+      </c>
+      <c r="B5" s="39" t="s">
+        <v>28</v>
+      </c>
+      <c r="C5" s="39" t="s">
+        <v>161</v>
+      </c>
+      <c r="D5" s="39" t="s">
+        <v>289</v>
+      </c>
+      <c r="E5" s="40" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="41" t="s">
+        <v>11</v>
+      </c>
+      <c r="B6" s="41" t="s">
+        <v>28</v>
+      </c>
+      <c r="C6" s="41" t="s">
+        <v>161</v>
+      </c>
+      <c r="D6" s="41" t="s">
+        <v>290</v>
+      </c>
+      <c r="E6" s="41" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A7" s="39" t="s">
+        <v>11</v>
+      </c>
+      <c r="B7" s="39" t="s">
+        <v>28</v>
+      </c>
+      <c r="C7" s="39" t="s">
+        <v>163</v>
+      </c>
+      <c r="D7" s="39" t="s">
+        <v>289</v>
+      </c>
+      <c r="E7" s="40" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="41" t="s">
+        <v>11</v>
+      </c>
+      <c r="B8" s="41" t="s">
+        <v>28</v>
+      </c>
+      <c r="C8" s="41" t="s">
+        <v>163</v>
+      </c>
+      <c r="D8" s="41" t="s">
+        <v>290</v>
+      </c>
+      <c r="E8" s="41" t="s">
+        <v>64</v>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="A3:C15 D5:D6">
-    <cfRule type="cellIs" dxfId="2" priority="1" operator="equal">
+  <conditionalFormatting sqref="B3:D15 E5:E6">
+    <cfRule type="cellIs" dxfId="24" priority="13" operator="equal">
       <formula>"Initial"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A3:C17 D5:D6">
-    <cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
+  <conditionalFormatting sqref="B3:D17 E5:E6">
+    <cfRule type="cellIs" dxfId="23" priority="14" operator="equal">
       <formula>"Inital"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="22" priority="15" operator="equal">
       <formula>"Final"</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="A3">
+    <cfRule type="cellIs" dxfId="17" priority="11" operator="equal">
+      <formula>"Yes"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="16" priority="12" operator="equal">
+      <formula>"No"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A4">
+    <cfRule type="cellIs" dxfId="13" priority="9" operator="equal">
+      <formula>"Yes"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="12" priority="10" operator="equal">
+      <formula>"No"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A5">
+    <cfRule type="cellIs" dxfId="9" priority="7" operator="equal">
+      <formula>"Yes"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="8" priority="8" operator="equal">
+      <formula>"No"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A6">
+    <cfRule type="cellIs" dxfId="7" priority="5" operator="equal">
+      <formula>"Yes"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="6" priority="6" operator="equal">
+      <formula>"No"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A7">
+    <cfRule type="cellIs" dxfId="5" priority="3" operator="equal">
+      <formula>"Yes"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="4" priority="4" operator="equal">
+      <formula>"No"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A8">
+    <cfRule type="cellIs" dxfId="1" priority="1" operator="equal">
+      <formula>"Yes"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="0" priority="2" operator="equal">
+      <formula>"No"</formula>
+    </cfRule>
+  </conditionalFormatting>
   <dataValidations count="3">
-    <dataValidation type="list" showInputMessage="1" showErrorMessage="1" prompt="Select well name from &quot;Well settings&quot; sheet " sqref="A3:A38" xr:uid="{00000000-0002-0000-0A00-000000000000}">
+    <dataValidation type="list" showInputMessage="1" showErrorMessage="1" prompt="Select well name from &quot;Well settings&quot; sheet " sqref="B3:B38" xr:uid="{00000000-0002-0000-0A00-000000000000}">
       <formula1>WellNames</formula1>
     </dataValidation>
-    <dataValidation type="list" showInputMessage="1" showErrorMessage="1" prompt="Select Mineral from &quot;Minerals&quot; sheet" sqref="C3:C40" xr:uid="{00000000-0002-0000-0A00-000001000000}">
+    <dataValidation type="list" showInputMessage="1" showErrorMessage="1" prompt="Select Mineral from &quot;Minerals&quot; sheet" sqref="D3:D40" xr:uid="{00000000-0002-0000-0A00-000001000000}">
       <formula1>MineralNames</formula1>
     </dataValidation>
-    <dataValidation showInputMessage="1" showErrorMessage="1" prompt="'1.0' (or other number) for constant Volume fraction_x000a_'complement' for complement volume fraction _x000a_log name, e.g. VCL, for using a log for volume fraction" sqref="D3:D40" xr:uid="{00000000-0002-0000-0A00-000002000000}"/>
+    <dataValidation showInputMessage="1" showErrorMessage="1" prompt="'1.0' (or other number) for constant Volume fraction_x000a_'complement' for complement volume fraction _x000a_log name, e.g. VCL, for using a log for volume fraction" sqref="E3:E40" xr:uid="{00000000-0002-0000-0A00-000002000000}"/>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" verticalDpi="0"/>
@@ -2860,9 +3228,9 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CCD9C215-DCD2-40A2-A7D5-172DC530BE0E}">
   <dimension ref="A1:Q2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
       <c r="D1" s="2"/>
@@ -2883,7 +3251,7 @@
       </c>
       <c r="O1" s="2"/>
     </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>371</v>
       </c>
@@ -2936,9 +3304,9 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3CCC2506-3BD3-4476-A9AA-1673C259914E}">
   <dimension ref="A1:M2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" s="2"/>
       <c r="B1" s="2" t="s">
         <v>376</v>
@@ -2951,7 +3319,7 @@
       <c r="I1" s="2"/>
       <c r="K1" s="2"/>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>372</v>
       </c>
@@ -2997,19 +3365,19 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
   <dimension ref="A1:Q18"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="16.33203125" customWidth="1"/>
-    <col min="3" max="3" width="12.33203125" customWidth="1"/>
-    <col min="4" max="4" width="9.88671875" customWidth="1"/>
+    <col min="2" max="2" width="16.28515625" customWidth="1"/>
+    <col min="3" max="3" width="12.28515625" customWidth="1"/>
+    <col min="4" max="4" width="9.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="H1" s="2" t="s">
         <v>359</v>
       </c>
     </row>
-    <row r="2" spans="1:17" s="6" customFormat="1" ht="42.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:17" s="6" customFormat="1" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2" s="6" t="s">
         <v>323</v>
       </c>
@@ -3059,7 +3427,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>11</v>
       </c>
@@ -3113,7 +3481,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>21</v>
       </c>
@@ -3164,7 +3532,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
       <c r="E5" t="s">
         <v>337</v>
       </c>
@@ -3191,7 +3559,7 @@
         <v>354</v>
       </c>
     </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
       <c r="E6" t="s">
         <v>274</v>
       </c>
@@ -3215,7 +3583,7 @@
         <v>355</v>
       </c>
     </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
       <c r="F7" t="s">
         <v>30</v>
       </c>
@@ -3233,7 +3601,7 @@
         <v>357</v>
       </c>
     </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
       <c r="F8" t="s">
         <v>33</v>
       </c>
@@ -3245,7 +3613,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
       <c r="F9" t="s">
         <v>24</v>
       </c>
@@ -3257,7 +3625,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="10" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:17" x14ac:dyDescent="0.25">
       <c r="F10" t="s">
         <v>36</v>
       </c>
@@ -3269,7 +3637,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:17" x14ac:dyDescent="0.25">
       <c r="F11" t="s">
         <v>38</v>
       </c>
@@ -3281,7 +3649,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:17" x14ac:dyDescent="0.25">
       <c r="F12" t="s">
         <v>40</v>
       </c>
@@ -3293,7 +3661,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:17" x14ac:dyDescent="0.25">
       <c r="F13" t="s">
         <v>340</v>
       </c>
@@ -3305,7 +3673,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:17" x14ac:dyDescent="0.25">
       <c r="F14" t="s">
         <v>341</v>
       </c>
@@ -3317,7 +3685,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:17" x14ac:dyDescent="0.25">
       <c r="F15" t="s">
         <v>121</v>
       </c>
@@ -3329,7 +3697,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:17" x14ac:dyDescent="0.25">
       <c r="F16" t="s">
         <v>342</v>
       </c>
@@ -3341,7 +3709,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="8:9" x14ac:dyDescent="0.3">
+    <row r="17" spans="8:9" x14ac:dyDescent="0.25">
       <c r="H17" s="30" t="s">
         <v>173</v>
       </c>
@@ -3350,7 +3718,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="8:9" x14ac:dyDescent="0.3">
+    <row r="18" spans="8:9" x14ac:dyDescent="0.25">
       <c r="H18" s="30" t="s">
         <v>174</v>
       </c>
@@ -3368,19 +3736,19 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:R11"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="2" width="9.6640625" style="13" customWidth="1"/>
-    <col min="3" max="3" width="15.88671875" customWidth="1"/>
-    <col min="4" max="5" width="11.5546875" customWidth="1"/>
+    <col min="1" max="2" width="9.7109375" style="13" customWidth="1"/>
+    <col min="3" max="3" width="15.85546875" customWidth="1"/>
+    <col min="4" max="5" width="11.5703125" customWidth="1"/>
     <col min="6" max="7" width="10" customWidth="1"/>
-    <col min="11" max="11" width="16.109375" customWidth="1"/>
+    <col min="11" max="11" width="16.140625" customWidth="1"/>
     <col min="13" max="13" width="7" customWidth="1"/>
-    <col min="16" max="16" width="6.5546875" customWidth="1"/>
-    <col min="17" max="17" width="4.6640625" customWidth="1"/>
+    <col min="16" max="16" width="6.5703125" customWidth="1"/>
+    <col min="17" max="17" width="4.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A1" s="11" t="s">
         <v>41</v>
       </c>
@@ -3388,7 +3756,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="2" spans="1:18" s="1" customFormat="1" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:18" s="1" customFormat="1" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="12" t="s">
         <v>3</v>
       </c>
@@ -3444,7 +3812,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A3" s="13" t="s">
         <v>12</v>
       </c>
@@ -3473,7 +3841,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A4" s="13" t="s">
         <v>12</v>
       </c>
@@ -3490,7 +3858,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A5" s="13" t="s">
         <v>15</v>
       </c>
@@ -3516,7 +3884,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A6" s="13" t="s">
         <v>18</v>
       </c>
@@ -3542,7 +3910,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A7" s="13" t="s">
         <v>22</v>
       </c>
@@ -3571,7 +3939,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A8" s="13" t="s">
         <v>25</v>
       </c>
@@ -3588,7 +3956,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A9" s="13" t="s">
         <v>25</v>
       </c>
@@ -3611,7 +3979,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A10" s="13" t="s">
         <v>28</v>
       </c>
@@ -3643,7 +4011,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A11" s="13" t="s">
         <v>31</v>
       </c>
@@ -3677,10 +4045,10 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="B3:B16">
-    <cfRule type="cellIs" dxfId="14" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="36" priority="1" operator="equal">
       <formula>"Yes"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="13" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="35" priority="2" operator="equal">
       <formula>"No"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3700,13 +4068,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{725EDE5F-2F74-4F10-B375-EE1EEF8AD52D}">
   <dimension ref="A1:M20"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="3" max="3" width="20.88671875" customWidth="1"/>
-    <col min="4" max="4" width="14.5546875" customWidth="1"/>
+    <col min="3" max="3" width="20.85546875" customWidth="1"/>
+    <col min="4" max="4" width="14.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" s="11" t="s">
         <v>41</v>
       </c>
@@ -3720,7 +4088,7 @@
         <v>379</v>
       </c>
     </row>
-    <row r="2" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="12" t="s">
         <v>3</v>
       </c>
@@ -3757,7 +4125,7 @@
       <c r="L2" s="1"/>
       <c r="M2" s="1"/>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" s="13" t="s">
         <v>12</v>
       </c>
@@ -3783,7 +4151,7 @@
         <v>382</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" s="13" t="s">
         <v>12</v>
       </c>
@@ -3806,11 +4174,11 @@
         <v>384</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" s="13"/>
       <c r="C5" s="4"/>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" s="13" t="s">
         <v>15</v>
       </c>
@@ -3836,7 +4204,7 @@
         <v>382</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" s="13" t="s">
         <v>15</v>
       </c>
@@ -3859,11 +4227,11 @@
         <v>384</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" s="13"/>
       <c r="C8" s="4"/>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" s="13" t="s">
         <v>18</v>
       </c>
@@ -3889,7 +4257,7 @@
         <v>382</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" s="13" t="s">
         <v>18</v>
       </c>
@@ -3912,11 +4280,11 @@
         <v>384</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" s="13"/>
       <c r="C11" s="4"/>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A12" s="13" t="s">
         <v>22</v>
       </c>
@@ -3925,11 +4293,11 @@
       </c>
       <c r="C12" s="4"/>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A13" s="13"/>
       <c r="C13" s="4"/>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A14" s="13" t="s">
         <v>25</v>
       </c>
@@ -3938,7 +4306,7 @@
       </c>
       <c r="C14" s="4"/>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A15" s="13" t="s">
         <v>25</v>
       </c>
@@ -3947,11 +4315,11 @@
       </c>
       <c r="C15" s="4"/>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A16" s="13"/>
       <c r="C16" s="4"/>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" s="13" t="s">
         <v>28</v>
       </c>
@@ -3980,7 +4348,7 @@
         <v>385</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" s="13" t="s">
         <v>28</v>
       </c>
@@ -4003,11 +4371,11 @@
         <v>384</v>
       </c>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" s="13"/>
       <c r="C19" s="4"/>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" s="13" t="s">
         <v>31</v>
       </c>
@@ -4019,10 +4387,10 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="B3:B20">
-    <cfRule type="cellIs" dxfId="12" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="34" priority="1" operator="equal">
       <formula>"Yes"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="11" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="33" priority="2" operator="equal">
       <formula>"No"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -4045,19 +4413,19 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:O31"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.44140625" customWidth="1"/>
-    <col min="2" max="2" width="14.109375" customWidth="1"/>
-    <col min="3" max="3" width="14.5546875" customWidth="1"/>
+    <col min="1" max="1" width="11.42578125" customWidth="1"/>
+    <col min="2" max="2" width="14.140625" customWidth="1"/>
+    <col min="3" max="3" width="14.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>175</v>
       </c>
     </row>
-    <row r="2" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>176</v>
       </c>
@@ -4104,7 +4472,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>190</v>
       </c>
@@ -4139,7 +4507,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
         <v>45</v>
       </c>
@@ -4171,7 +4539,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
         <v>47</v>
       </c>
@@ -4203,7 +4571,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>197</v>
       </c>
@@ -4238,7 +4606,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>200</v>
       </c>
@@ -4273,7 +4641,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>202</v>
       </c>
@@ -4308,7 +4676,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
         <v>206</v>
       </c>
@@ -4333,7 +4701,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
         <v>208</v>
       </c>
@@ -4358,7 +4726,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>209</v>
       </c>
@@ -4393,7 +4761,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>210</v>
       </c>
@@ -4428,7 +4796,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>213</v>
       </c>
@@ -4463,7 +4831,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>77</v>
       </c>
@@ -4498,7 +4866,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>215</v>
       </c>
@@ -4533,7 +4901,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>218</v>
       </c>
@@ -4568,7 +4936,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>221</v>
       </c>
@@ -4603,7 +4971,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>224</v>
       </c>
@@ -4638,7 +5006,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>225</v>
       </c>
@@ -4673,7 +5041,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>227</v>
       </c>
@@ -4708,7 +5076,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>229</v>
       </c>
@@ -4746,7 +5114,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>234</v>
       </c>
@@ -4775,7 +5143,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>236</v>
       </c>
@@ -4810,7 +5178,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>240</v>
       </c>
@@ -4841,7 +5209,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>243</v>
       </c>
@@ -4876,7 +5244,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B26" t="s">
         <v>57</v>
       </c>
@@ -4896,7 +5264,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B27" t="s">
         <v>378</v>
       </c>
@@ -4922,7 +5290,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B28" t="s">
         <v>245</v>
       </c>
@@ -4948,7 +5316,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>246</v>
       </c>
@@ -4977,7 +5345,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>248</v>
       </c>
@@ -5006,7 +5374,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B31" t="s">
         <v>250</v>
       </c>
@@ -5046,13 +5414,13 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:M17"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
-    <col min="6" max="6" width="15.5546875" customWidth="1"/>
+    <col min="6" max="6" width="15.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" s="2"/>
       <c r="B1" s="2" t="s">
         <v>112</v>
@@ -5069,7 +5437,7 @@
       <c r="I1" s="2"/>
       <c r="K1" s="2"/>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>115</v>
       </c>
@@ -5110,7 +5478,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>125</v>
       </c>
@@ -5136,7 +5504,7 @@
         <v>-18877.708702820371</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>131</v>
       </c>
@@ -5162,7 +5530,7 @@
         <v>-19045.139985898601</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>133</v>
       </c>
@@ -5188,7 +5556,7 @@
         <v>-5.4445188599886638</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>135</v>
       </c>
@@ -5214,7 +5582,7 @@
         <v>2.671411511624413</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>137</v>
       </c>
@@ -5240,7 +5608,7 @@
         <v>9.5532474786010475</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>125</v>
       </c>
@@ -5266,7 +5634,7 @@
         <v>2866.0938229725748</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>131</v>
       </c>
@@ -5292,7 +5660,7 @@
         <v>1490.761502865475</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>133</v>
       </c>
@@ -5318,7 +5686,7 @@
         <v>2.217459469264154</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>135</v>
       </c>
@@ -5344,7 +5712,7 @@
         <v>0.2337935274525294</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>137</v>
       </c>
@@ -5370,7 +5738,7 @@
         <v>2.0873115011979051E-2</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>125</v>
       </c>
@@ -5396,7 +5764,7 @@
         <v>1351.711647219304</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>131</v>
       </c>
@@ -5422,7 +5790,7 @@
         <v>150.9391394665019</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>133</v>
       </c>
@@ -5448,7 +5816,7 @@
         <v>1.940117188288828</v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>135</v>
       </c>
@@ -5474,7 +5842,7 @@
         <v>-2.0146865510893688E-2</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>137</v>
       </c>
@@ -5508,22 +5876,22 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:G42"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="3" max="3" width="16.6640625" customWidth="1"/>
+    <col min="3" max="3" width="16.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>153</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="5" spans="1:7" s="1" customFormat="1" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" s="1" customFormat="1" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>2</v>
       </c>
@@ -5546,7 +5914,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
         <v>12</v>
       </c>
@@ -5566,7 +5934,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="7" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
         <v>12</v>
       </c>
@@ -5583,7 +5951,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="8" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
         <v>12</v>
       </c>
@@ -5600,7 +5968,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="9" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
         <v>12</v>
       </c>
@@ -5617,7 +5985,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="10" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
         <v>12</v>
       </c>
@@ -5634,7 +6002,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="11" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
         <v>12</v>
       </c>
@@ -5651,7 +6019,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
         <v>12</v>
       </c>
@@ -5668,7 +6036,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B13" t="s">
         <v>15</v>
       </c>
@@ -5685,7 +6053,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="14" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="B14" t="s">
         <v>15</v>
       </c>
@@ -5702,7 +6070,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="15" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="B15" t="s">
         <v>15</v>
       </c>
@@ -5719,7 +6087,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="16" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="B16" t="s">
         <v>15</v>
       </c>
@@ -5736,7 +6104,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="17" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B17" t="s">
         <v>15</v>
       </c>
@@ -5753,7 +6121,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="18" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B18" t="s">
         <v>15</v>
       </c>
@@ -5770,7 +6138,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="19" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="B19" t="s">
         <v>15</v>
       </c>
@@ -5787,7 +6155,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="20" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B20" t="s">
         <v>18</v>
       </c>
@@ -5804,7 +6172,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="21" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B21" t="s">
         <v>18</v>
       </c>
@@ -5821,7 +6189,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="22" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B22" t="s">
         <v>18</v>
       </c>
@@ -5838,7 +6206,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="23" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B23" t="s">
         <v>18</v>
       </c>
@@ -5855,7 +6223,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="24" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B24" t="s">
         <v>18</v>
       </c>
@@ -5872,7 +6240,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="25" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B25" t="s">
         <v>18</v>
       </c>
@@ -5889,7 +6257,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="26" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B26" t="s">
         <v>18</v>
       </c>
@@ -5906,7 +6274,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="27" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B27" t="s">
         <v>28</v>
       </c>
@@ -5923,7 +6291,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="28" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B28" t="s">
         <v>28</v>
       </c>
@@ -5940,7 +6308,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="29" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B29" t="s">
         <v>28</v>
       </c>
@@ -5957,7 +6325,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="30" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B30" t="s">
         <v>28</v>
       </c>
@@ -5974,7 +6342,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="31" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B31" t="s">
         <v>28</v>
       </c>
@@ -5991,7 +6359,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="32" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B32" t="s">
         <v>28</v>
       </c>
@@ -6008,7 +6376,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="33" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B33" t="s">
         <v>28</v>
       </c>
@@ -6025,7 +6393,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="34" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="34" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B34" t="s">
         <v>31</v>
       </c>
@@ -6042,7 +6410,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="35" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="35" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B35" t="s">
         <v>31</v>
       </c>
@@ -6059,7 +6427,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="36" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="36" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B36" t="s">
         <v>31</v>
       </c>
@@ -6076,7 +6444,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="37" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="37" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B37" t="s">
         <v>31</v>
       </c>
@@ -6093,7 +6461,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="38" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="38" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B38" t="s">
         <v>31</v>
       </c>
@@ -6110,7 +6478,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="39" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="39" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B39" t="s">
         <v>31</v>
       </c>
@@ -6127,7 +6495,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="40" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="40" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B40" t="s">
         <v>31</v>
       </c>
@@ -6144,7 +6512,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="41" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="41" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B41" t="s">
         <v>31</v>
       </c>
@@ -6161,7 +6529,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="42" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="42" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B42" t="s">
         <v>31</v>
       </c>
@@ -6195,19 +6563,19 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9DE0C751-ACC1-462A-82AF-4CE9BB91C06B}">
   <dimension ref="A2:G21"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C4" t="s">
         <v>390</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>2</v>
       </c>
@@ -6230,7 +6598,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>21</v>
       </c>
@@ -6244,7 +6612,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>11</v>
       </c>
@@ -6258,7 +6626,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>11</v>
       </c>
@@ -6272,7 +6640,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>11</v>
       </c>
@@ -6286,7 +6654,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>11</v>
       </c>
@@ -6300,7 +6668,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>11</v>
       </c>
@@ -6314,7 +6682,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>21</v>
       </c>
@@ -6328,7 +6696,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>11</v>
       </c>
@@ -6342,7 +6710,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>11</v>
       </c>
@@ -6356,7 +6724,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>11</v>
       </c>
@@ -6370,7 +6738,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>11</v>
       </c>
@@ -6384,7 +6752,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>11</v>
       </c>
@@ -6398,7 +6766,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>11</v>
       </c>
@@ -6412,7 +6780,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>11</v>
       </c>
@@ -6426,7 +6794,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>11</v>
       </c>
@@ -6440,7 +6808,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>11</v>
       </c>
@@ -6456,10 +6824,10 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A6:A22">
-    <cfRule type="cellIs" dxfId="10" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="32" priority="1" operator="equal">
       <formula>"Yes"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="9" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="31" priority="2" operator="equal">
       <formula>"No"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -6470,25 +6838,25 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:O8"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8.5546875" customWidth="1"/>
+    <col min="1" max="1" width="8.5703125" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
-    <col min="3" max="3" width="12.88671875" customWidth="1"/>
+    <col min="3" max="3" width="12.85546875" customWidth="1"/>
     <col min="4" max="4" width="10" customWidth="1"/>
-    <col min="6" max="6" width="6.6640625" customWidth="1"/>
-    <col min="7" max="7" width="6.5546875" customWidth="1"/>
-    <col min="8" max="8" width="8.33203125" customWidth="1"/>
-    <col min="9" max="9" width="5.5546875" customWidth="1"/>
-    <col min="10" max="10" width="6.5546875" customWidth="1"/>
-    <col min="11" max="11" width="6.109375" customWidth="1"/>
-    <col min="12" max="12" width="5.109375" customWidth="1"/>
-    <col min="13" max="13" width="5.5546875" customWidth="1"/>
-    <col min="14" max="14" width="5.109375" customWidth="1"/>
-    <col min="15" max="15" width="4.44140625" customWidth="1"/>
+    <col min="6" max="6" width="6.7109375" customWidth="1"/>
+    <col min="7" max="7" width="6.5703125" customWidth="1"/>
+    <col min="8" max="8" width="8.28515625" customWidth="1"/>
+    <col min="9" max="9" width="5.5703125" customWidth="1"/>
+    <col min="10" max="10" width="6.5703125" customWidth="1"/>
+    <col min="11" max="11" width="6.140625" customWidth="1"/>
+    <col min="12" max="12" width="5.140625" customWidth="1"/>
+    <col min="13" max="13" width="5.5703125" customWidth="1"/>
+    <col min="14" max="14" width="5.140625" customWidth="1"/>
+    <col min="15" max="15" width="4.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>253</v>
       </c>
@@ -6496,7 +6864,7 @@
         <v>254</v>
       </c>
     </row>
-    <row r="2" spans="1:15" s="8" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:15" s="8" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="8" t="s">
         <v>255</v>
       </c>
@@ -6543,7 +6911,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>270</v>
       </c>
@@ -6583,7 +6951,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>273</v>
       </c>
@@ -6598,7 +6966,7 @@
         <v>274</v>
       </c>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>396</v>
       </c>
@@ -6638,21 +7006,21 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B7" s="3"/>
       <c r="C7" s="3"/>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B8" s="3"/>
       <c r="C8" s="3"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="A3:A28">
-    <cfRule type="duplicateValues" dxfId="8" priority="6"/>
+    <cfRule type="duplicateValues" dxfId="30" priority="6"/>
   </conditionalFormatting>
   <dataValidations count="1">
     <dataValidation showInputMessage="1" showErrorMessage="1" prompt="No duplicate names please" sqref="A3:A38" xr:uid="{00000000-0002-0000-0700-000000000000}"/>
@@ -6665,13 +7033,13 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
   <dimension ref="A1:H21"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="4" width="10.33203125" customWidth="1"/>
-    <col min="5" max="6" width="8.5546875" customWidth="1"/>
+    <col min="2" max="4" width="10.28515625" customWidth="1"/>
+    <col min="5" max="6" width="8.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -6679,7 +7047,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="2" spans="1:8" s="8" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:8" s="8" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
@@ -6705,7 +7073,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:8" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="31" t="s">
         <v>21</v>
       </c>
@@ -6720,7 +7088,7 @@
       </c>
       <c r="G3" s="32"/>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>21</v>
       </c>
@@ -6746,7 +7114,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>21</v>
       </c>
@@ -6772,7 +7140,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:8" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="31" t="s">
         <v>21</v>
       </c>
@@ -6798,7 +7166,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>11</v>
       </c>
@@ -6824,7 +7192,7 @@
         <v>345</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>11</v>
       </c>
@@ -6850,7 +7218,7 @@
         <v>345</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="31" t="s">
         <v>11</v>
       </c>
@@ -6876,7 +7244,7 @@
         <v>345</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>11</v>
       </c>
@@ -6899,7 +7267,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>11</v>
       </c>
@@ -6922,7 +7290,7 @@
         <v>283</v>
       </c>
     </row>
-    <row r="12" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="31" t="s">
         <v>11</v>
       </c>
@@ -6945,7 +7313,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>11</v>
       </c>
@@ -6968,7 +7336,7 @@
         <v>283</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>11</v>
       </c>
@@ -6991,7 +7359,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="15" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="31" t="s">
         <v>11</v>
       </c>
@@ -7014,30 +7382,30 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="8:8" x14ac:dyDescent="0.3">
+    <row r="21" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H21" t="s">
         <v>285</v>
       </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="A3:A32">
-    <cfRule type="cellIs" dxfId="7" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="29" priority="1" operator="equal">
       <formula>"Yes"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="6" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="28" priority="2" operator="equal">
       <formula>"No"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B3:D15">
-    <cfRule type="cellIs" dxfId="5" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="27" priority="3" operator="equal">
       <formula>"Initial"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B3:D17">
-    <cfRule type="cellIs" dxfId="4" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="26" priority="4" operator="equal">
       <formula>"Inital"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="3" priority="5" operator="equal">
+    <cfRule type="cellIs" dxfId="25" priority="5" operator="equal">
       <formula>"Final"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -7057,6 +7425,6 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Fluid substitution (fluid_substitution.py) using the new fluids_and_minerals.py has now passed a simple production test. well_new.py has been upgraded to have a better plotting functionality
</commit_message>
<xml_diff>
--- a/excels/project_table_new.xlsx
+++ b/excels/project_table_new.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="T:\Python\EMB\blixt_rp\excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93759F2E-467B-4E29-84F7-FECAE662F40D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B6006E1-5DAD-41D2-BF7E-CFB3416A2ED4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="685" firstSheet="5" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" tabRatio="685" firstSheet="5" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Well settings" sheetId="1" r:id="rId1"/>
@@ -64,7 +64,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1048" uniqueCount="397">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1055" uniqueCount="398">
   <si>
     <t>Select Yes or No</t>
   </si>
@@ -1110,9 +1110,6 @@
     <t>test</t>
   </si>
   <si>
-    <t>XX</t>
-  </si>
-  <si>
     <t>Seismic response</t>
   </si>
   <si>
@@ -1264,6 +1261,12 @@
   </si>
   <si>
     <t>TESTFLUID</t>
+  </si>
+  <si>
+    <t>The tag is used as indentifier of different fluid substitution scenarios, and are added to the name of the resulting well logs</t>
+  </si>
+  <si>
+    <t>MyTag</t>
   </si>
 </sst>
 </file>
@@ -1475,7 +1478,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1527,251 +1530,12 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="39">
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="19">
     <dxf>
       <font>
         <color rgb="FF9C5700"/>
@@ -1799,6 +1563,27 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2223,13 +2008,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:I13"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" customWidth="1"/>
-    <col min="2" max="2" width="12.42578125" customWidth="1"/>
+    <col min="1" max="1" width="5.6640625" customWidth="1"/>
+    <col min="2" max="2" width="12.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -2240,7 +2025,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:9" s="1" customFormat="1" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" s="1" customFormat="1" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
@@ -2269,7 +2054,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>21</v>
       </c>
@@ -2289,7 +2074,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>21</v>
       </c>
@@ -2303,7 +2088,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>21</v>
       </c>
@@ -2317,7 +2102,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>21</v>
       </c>
@@ -2331,7 +2116,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>21</v>
       </c>
@@ -2345,7 +2130,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>11</v>
       </c>
@@ -2365,7 +2150,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>21</v>
       </c>
@@ -2382,12 +2167,12 @@
         <v>34</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>21</v>
       </c>
       <c r="B10" s="13" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="C10" s="20" t="s">
         <v>23</v>
@@ -2396,7 +2181,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
       <c r="C11" s="21" t="s">
         <v>35</v>
       </c>
@@ -2404,7 +2189,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
       <c r="C12" s="22" t="s">
         <v>37</v>
       </c>
@@ -2412,7 +2197,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
       <c r="C13" s="23" t="s">
         <v>39</v>
       </c>
@@ -2422,10 +2207,10 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A3:A20">
-    <cfRule type="cellIs" dxfId="38" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="18" priority="1" operator="equal">
       <formula>"Yes"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="37" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="17" priority="2" operator="equal">
       <formula>"No"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -2436,21 +2221,21 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
   <dimension ref="A1:G33"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="17.42578125" customWidth="1"/>
+    <col min="1" max="1" width="17.44140625" customWidth="1"/>
     <col min="6" max="6" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" ht="26.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="F1" s="7" t="s">
         <v>286</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>395</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" s="8" customFormat="1" ht="30.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" s="8" customFormat="1" ht="30.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="33" t="s">
         <v>255</v>
       </c>
@@ -2473,7 +2258,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>289</v>
       </c>
@@ -2490,7 +2275,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>290</v>
       </c>
@@ -2510,10 +2295,10 @@
         <v>291</v>
       </c>
       <c r="G4" t="s">
-        <v>394</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>292</v>
       </c>
@@ -2530,7 +2315,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>293</v>
       </c>
@@ -2547,7 +2332,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>294</v>
       </c>
@@ -2564,7 +2349,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>295</v>
       </c>
@@ -2581,7 +2366,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>296</v>
       </c>
@@ -2598,7 +2383,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>297</v>
       </c>
@@ -2615,7 +2400,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>298</v>
       </c>
@@ -2632,7 +2417,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>299</v>
       </c>
@@ -2649,7 +2434,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>300</v>
       </c>
@@ -2666,7 +2451,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>301</v>
       </c>
@@ -2683,7 +2468,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>302</v>
       </c>
@@ -2700,7 +2485,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>303</v>
       </c>
@@ -2717,7 +2502,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>304</v>
       </c>
@@ -2734,7 +2519,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>305</v>
       </c>
@@ -2751,7 +2536,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>306</v>
       </c>
@@ -2768,7 +2553,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>307</v>
       </c>
@@ -2785,7 +2570,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>308</v>
       </c>
@@ -2802,7 +2587,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>309</v>
       </c>
@@ -2819,7 +2604,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>310</v>
       </c>
@@ -2836,7 +2621,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>311</v>
       </c>
@@ -2853,7 +2638,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>312</v>
       </c>
@@ -2870,7 +2655,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>313</v>
       </c>
@@ -2887,7 +2672,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>314</v>
       </c>
@@ -2904,7 +2689,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>315</v>
       </c>
@@ -2921,7 +2706,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>316</v>
       </c>
@@ -2938,7 +2723,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>317</v>
       </c>
@@ -2955,7 +2740,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>318</v>
       </c>
@@ -2972,7 +2757,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>319</v>
       </c>
@@ -2989,7 +2774,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>320</v>
       </c>
@@ -3015,23 +2800,23 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
   <dimension ref="A1:E8"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="3" width="10.28515625" customWidth="1"/>
-    <col min="4" max="4" width="17.42578125" customWidth="1"/>
+    <col min="2" max="3" width="10.33203125" customWidth="1"/>
+    <col min="4" max="4" width="17.44140625" customWidth="1"/>
     <col min="5" max="5" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="37" t="s">
+    <row r="1" spans="1:5" ht="26.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
       <c r="E1" s="5" t="s">
         <v>321</v>
       </c>
     </row>
-    <row r="2" spans="1:5" s="8" customFormat="1" ht="30.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="38" t="s">
+    <row r="2" spans="1:5" s="8" customFormat="1" ht="30.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="9" t="s">
         <v>2</v>
       </c>
       <c r="B2" s="9" t="s">
@@ -3047,8 +2832,8 @@
         <v>280</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="39" t="s">
+    <row r="3" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
         <v>11</v>
       </c>
       <c r="B3" t="s">
@@ -3064,151 +2849,111 @@
         <v>283</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="41" t="s">
+    <row r="4" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="31" t="s">
         <v>11</v>
       </c>
-      <c r="B4" s="41" t="s">
+      <c r="B4" s="31" t="s">
         <v>28</v>
       </c>
-      <c r="C4" s="41" t="s">
+      <c r="C4" s="31" t="s">
         <v>162</v>
       </c>
-      <c r="D4" s="41" t="s">
+      <c r="D4" s="31" t="s">
         <v>290</v>
       </c>
-      <c r="E4" s="41" t="s">
+      <c r="E4" s="31" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A5" s="39" t="s">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
         <v>11</v>
       </c>
-      <c r="B5" s="39" t="s">
+      <c r="B5" t="s">
         <v>28</v>
       </c>
-      <c r="C5" s="39" t="s">
+      <c r="C5" t="s">
         <v>161</v>
       </c>
-      <c r="D5" s="39" t="s">
+      <c r="D5" t="s">
         <v>289</v>
       </c>
-      <c r="E5" s="40" t="s">
+      <c r="E5" s="6" t="s">
         <v>283</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="41" t="s">
+    <row r="6" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="31" t="s">
         <v>11</v>
       </c>
-      <c r="B6" s="41" t="s">
+      <c r="B6" s="31" t="s">
         <v>28</v>
       </c>
-      <c r="C6" s="41" t="s">
+      <c r="C6" s="31" t="s">
         <v>161</v>
       </c>
-      <c r="D6" s="41" t="s">
+      <c r="D6" s="31" t="s">
         <v>290</v>
       </c>
-      <c r="E6" s="41" t="s">
+      <c r="E6" s="31" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A7" s="39" t="s">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
         <v>11</v>
       </c>
-      <c r="B7" s="39" t="s">
+      <c r="B7" t="s">
         <v>28</v>
       </c>
-      <c r="C7" s="39" t="s">
+      <c r="C7" t="s">
         <v>163</v>
       </c>
-      <c r="D7" s="39" t="s">
+      <c r="D7" t="s">
         <v>289</v>
       </c>
-      <c r="E7" s="40" t="s">
+      <c r="E7" s="6" t="s">
         <v>283</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="41" t="s">
+    <row r="8" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="31" t="s">
         <v>11</v>
       </c>
-      <c r="B8" s="41" t="s">
+      <c r="B8" s="31" t="s">
         <v>28</v>
       </c>
-      <c r="C8" s="41" t="s">
+      <c r="C8" s="31" t="s">
         <v>163</v>
       </c>
-      <c r="D8" s="41" t="s">
+      <c r="D8" s="31" t="s">
         <v>290</v>
       </c>
-      <c r="E8" s="41" t="s">
+      <c r="E8" s="31" t="s">
         <v>64</v>
       </c>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="A3:A8">
+    <cfRule type="cellIs" dxfId="4" priority="1" operator="equal">
+      <formula>"Yes"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="3" priority="2" operator="equal">
+      <formula>"No"</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="B3:D15 E5:E6">
-    <cfRule type="cellIs" dxfId="24" priority="13" operator="equal">
+    <cfRule type="cellIs" dxfId="2" priority="13" operator="equal">
       <formula>"Initial"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B3:D17 E5:E6">
-    <cfRule type="cellIs" dxfId="23" priority="14" operator="equal">
+    <cfRule type="cellIs" dxfId="1" priority="14" operator="equal">
       <formula>"Inital"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="22" priority="15" operator="equal">
+    <cfRule type="cellIs" dxfId="0" priority="15" operator="equal">
       <formula>"Final"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A3">
-    <cfRule type="cellIs" dxfId="17" priority="11" operator="equal">
-      <formula>"Yes"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="16" priority="12" operator="equal">
-      <formula>"No"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A4">
-    <cfRule type="cellIs" dxfId="13" priority="9" operator="equal">
-      <formula>"Yes"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="12" priority="10" operator="equal">
-      <formula>"No"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A5">
-    <cfRule type="cellIs" dxfId="9" priority="7" operator="equal">
-      <formula>"Yes"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="8" priority="8" operator="equal">
-      <formula>"No"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A6">
-    <cfRule type="cellIs" dxfId="7" priority="5" operator="equal">
-      <formula>"Yes"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="6" priority="6" operator="equal">
-      <formula>"No"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A7">
-    <cfRule type="cellIs" dxfId="5" priority="3" operator="equal">
-      <formula>"Yes"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="4" priority="4" operator="equal">
-      <formula>"No"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A8">
-    <cfRule type="cellIs" dxfId="1" priority="1" operator="equal">
-      <formula>"Yes"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="2" operator="equal">
-      <formula>"No"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
@@ -3228,9 +2973,9 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CCD9C215-DCD2-40A2-A7D5-172DC530BE0E}">
   <dimension ref="A1:Q2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.3">
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
       <c r="D1" s="2"/>
@@ -3244,49 +2989,49 @@
       <c r="J1" s="2"/>
       <c r="K1" s="2"/>
       <c r="L1" s="2" t="s">
+        <v>369</v>
+      </c>
+      <c r="M1" s="2" t="s">
+        <v>369</v>
+      </c>
+      <c r="O1" s="2"/>
+    </row>
+    <row r="2" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
         <v>370</v>
       </c>
-      <c r="M1" s="2" t="s">
-        <v>370</v>
-      </c>
-      <c r="O1" s="2"/>
-    </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
-        <v>371</v>
-      </c>
       <c r="B2" s="1" t="s">
+        <v>359</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>366</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>367</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>368</v>
+      </c>
+      <c r="F2" s="1" t="s">
         <v>360</v>
       </c>
-      <c r="C2" s="1" t="s">
-        <v>367</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>368</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>369</v>
-      </c>
-      <c r="F2" s="1" t="s">
+      <c r="G2" s="1" t="s">
         <v>361</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="H2" s="1" t="s">
         <v>362</v>
-      </c>
-      <c r="H2" s="1" t="s">
-        <v>363</v>
       </c>
       <c r="I2" s="1" t="s">
         <v>157</v>
       </c>
       <c r="J2" s="1" t="s">
+        <v>363</v>
+      </c>
+      <c r="K2" s="1" t="s">
         <v>364</v>
       </c>
-      <c r="K2" s="1" t="s">
+      <c r="L2" s="1" t="s">
         <v>365</v>
-      </c>
-      <c r="L2" s="1" t="s">
-        <v>366</v>
       </c>
       <c r="M2" s="1" t="s">
         <v>8</v>
@@ -3304,12 +3049,12 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3CCC2506-3BD3-4476-A9AA-1673C259914E}">
   <dimension ref="A1:M2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A1" s="2"/>
       <c r="B1" s="2" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="C1" s="2"/>
       <c r="D1" s="2"/>
@@ -3319,24 +3064,24 @@
       <c r="I1" s="2"/>
       <c r="K1" s="2"/>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>99</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="D2" s="1" t="s">
+        <v>372</v>
+      </c>
+      <c r="E2" s="1" t="s">
         <v>373</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="F2" s="1" t="s">
         <v>374</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>375</v>
       </c>
       <c r="G2" s="1"/>
       <c r="H2" s="1"/>
@@ -3365,19 +3110,19 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
   <dimension ref="A1:Q18"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="16.28515625" customWidth="1"/>
-    <col min="3" max="3" width="12.28515625" customWidth="1"/>
-    <col min="4" max="4" width="9.85546875" customWidth="1"/>
+    <col min="2" max="2" width="16.33203125" customWidth="1"/>
+    <col min="3" max="3" width="12.33203125" customWidth="1"/>
+    <col min="4" max="4" width="9.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.3">
       <c r="H1" s="2" t="s">
-        <v>359</v>
-      </c>
-    </row>
-    <row r="2" spans="1:17" s="6" customFormat="1" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="2" spans="1:17" s="6" customFormat="1" ht="42.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B2" s="6" t="s">
         <v>323</v>
       </c>
@@ -3400,7 +3145,7 @@
         <v>116</v>
       </c>
       <c r="I2" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="J2" s="6" t="s">
         <v>327</v>
@@ -3421,13 +3166,13 @@
         <v>102</v>
       </c>
       <c r="P2" t="s">
+        <v>345</v>
+      </c>
+      <c r="Q2" t="s">
         <v>346</v>
       </c>
-      <c r="Q2" t="s">
-        <v>347</v>
-      </c>
-    </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="3" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>11</v>
       </c>
@@ -3475,13 +3220,13 @@
         <v>106</v>
       </c>
       <c r="P3" t="s">
+        <v>347</v>
+      </c>
+      <c r="Q3" t="s">
         <v>348</v>
       </c>
-      <c r="Q3" t="s">
-        <v>349</v>
-      </c>
-    </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="4" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>21</v>
       </c>
@@ -3523,16 +3268,16 @@
         <v>105</v>
       </c>
       <c r="O4" t="s">
+        <v>349</v>
+      </c>
+      <c r="P4" t="s">
         <v>350</v>
       </c>
-      <c r="P4" t="s">
+      <c r="Q4" t="s">
         <v>351</v>
       </c>
-      <c r="Q4" t="s">
-        <v>352</v>
-      </c>
-    </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="5" spans="1:17" x14ac:dyDescent="0.3">
       <c r="E5" t="s">
         <v>337</v>
       </c>
@@ -3553,13 +3298,13 @@
         <v>105</v>
       </c>
       <c r="O5" t="s">
+        <v>352</v>
+      </c>
+      <c r="Q5" t="s">
         <v>353</v>
       </c>
-      <c r="Q5" t="s">
-        <v>354</v>
-      </c>
-    </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="6" spans="1:17" x14ac:dyDescent="0.3">
       <c r="E6" t="s">
         <v>274</v>
       </c>
@@ -3580,10 +3325,10 @@
         <v>338</v>
       </c>
       <c r="Q6" t="s">
-        <v>355</v>
-      </c>
-    </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="7" spans="1:17" x14ac:dyDescent="0.3">
       <c r="F7" t="s">
         <v>30</v>
       </c>
@@ -3595,13 +3340,13 @@
         <v>4</v>
       </c>
       <c r="O7" t="s">
+        <v>355</v>
+      </c>
+      <c r="Q7" t="s">
         <v>356</v>
       </c>
-      <c r="Q7" t="s">
-        <v>357</v>
-      </c>
-    </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="8" spans="1:17" x14ac:dyDescent="0.3">
       <c r="F8" t="s">
         <v>33</v>
       </c>
@@ -3613,7 +3358,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:17" x14ac:dyDescent="0.3">
       <c r="F9" t="s">
         <v>24</v>
       </c>
@@ -3625,7 +3370,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="10" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:17" x14ac:dyDescent="0.3">
       <c r="F10" t="s">
         <v>36</v>
       </c>
@@ -3637,7 +3382,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:17" x14ac:dyDescent="0.3">
       <c r="F11" t="s">
         <v>38</v>
       </c>
@@ -3649,7 +3394,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:17" x14ac:dyDescent="0.3">
       <c r="F12" t="s">
         <v>40</v>
       </c>
@@ -3661,7 +3406,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:17" x14ac:dyDescent="0.3">
       <c r="F13" t="s">
         <v>340</v>
       </c>
@@ -3673,7 +3418,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:17" x14ac:dyDescent="0.3">
       <c r="F14" t="s">
         <v>341</v>
       </c>
@@ -3685,7 +3430,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:17" x14ac:dyDescent="0.3">
       <c r="F15" t="s">
         <v>121</v>
       </c>
@@ -3697,7 +3442,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:17" x14ac:dyDescent="0.3">
       <c r="F16" t="s">
         <v>342</v>
       </c>
@@ -3709,7 +3454,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="8:9" x14ac:dyDescent="0.25">
+    <row r="17" spans="8:9" x14ac:dyDescent="0.3">
       <c r="H17" s="30" t="s">
         <v>173</v>
       </c>
@@ -3718,7 +3463,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="8:9" x14ac:dyDescent="0.25">
+    <row r="18" spans="8:9" x14ac:dyDescent="0.3">
       <c r="H18" s="30" t="s">
         <v>174</v>
       </c>
@@ -3736,19 +3481,19 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:R11"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="2" width="9.7109375" style="13" customWidth="1"/>
-    <col min="3" max="3" width="15.85546875" customWidth="1"/>
-    <col min="4" max="5" width="11.5703125" customWidth="1"/>
+    <col min="1" max="2" width="9.6640625" style="13" customWidth="1"/>
+    <col min="3" max="3" width="15.88671875" customWidth="1"/>
+    <col min="4" max="5" width="11.5546875" customWidth="1"/>
     <col min="6" max="7" width="10" customWidth="1"/>
-    <col min="11" max="11" width="16.140625" customWidth="1"/>
+    <col min="11" max="11" width="16.109375" customWidth="1"/>
     <col min="13" max="13" width="7" customWidth="1"/>
-    <col min="16" max="16" width="6.5703125" customWidth="1"/>
-    <col min="17" max="17" width="4.7109375" customWidth="1"/>
+    <col min="16" max="16" width="6.5546875" customWidth="1"/>
+    <col min="17" max="17" width="4.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A1" s="11" t="s">
         <v>41</v>
       </c>
@@ -3756,7 +3501,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="2" spans="1:18" s="1" customFormat="1" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:18" s="1" customFormat="1" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="12" t="s">
         <v>3</v>
       </c>
@@ -3812,7 +3557,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A3" s="13" t="s">
         <v>12</v>
       </c>
@@ -3841,7 +3586,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A4" s="13" t="s">
         <v>12</v>
       </c>
@@ -3858,7 +3603,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A5" s="13" t="s">
         <v>15</v>
       </c>
@@ -3884,7 +3629,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A6" s="13" t="s">
         <v>18</v>
       </c>
@@ -3910,7 +3655,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A7" s="13" t="s">
         <v>22</v>
       </c>
@@ -3939,7 +3684,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A8" s="13" t="s">
         <v>25</v>
       </c>
@@ -3956,7 +3701,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A9" s="13" t="s">
         <v>25</v>
       </c>
@@ -3979,7 +3724,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A10" s="13" t="s">
         <v>28</v>
       </c>
@@ -4011,7 +3756,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A11" s="13" t="s">
         <v>31</v>
       </c>
@@ -4045,10 +3790,10 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="B3:B16">
-    <cfRule type="cellIs" dxfId="36" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="16" priority="1" operator="equal">
       <formula>"Yes"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="35" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="15" priority="2" operator="equal">
       <formula>"No"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -4068,13 +3813,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{725EDE5F-2F74-4F10-B375-EE1EEF8AD52D}">
   <dimension ref="A1:M20"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="3" max="3" width="20.85546875" customWidth="1"/>
-    <col min="4" max="4" width="14.5703125" customWidth="1"/>
+    <col min="3" max="3" width="20.88671875" customWidth="1"/>
+    <col min="4" max="4" width="14.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A1" s="11" t="s">
         <v>41</v>
       </c>
@@ -4085,10 +3830,10 @@
         <v>98</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>379</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13" ht="30" x14ac:dyDescent="0.25">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A2" s="12" t="s">
         <v>3</v>
       </c>
@@ -4108,7 +3853,7 @@
         <v>245</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="H2" s="1" t="s">
         <v>241</v>
@@ -4125,7 +3870,7 @@
       <c r="L2" s="1"/>
       <c r="M2" s="1"/>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A3" s="13" t="s">
         <v>12</v>
       </c>
@@ -4142,16 +3887,16 @@
         <v>106</v>
       </c>
       <c r="F3" t="s">
+        <v>379</v>
+      </c>
+      <c r="G3" t="s">
         <v>380</v>
       </c>
-      <c r="G3" t="s">
+      <c r="H3" t="s">
         <v>381</v>
       </c>
-      <c r="H3" t="s">
-        <v>382</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A4" s="13" t="s">
         <v>12</v>
       </c>
@@ -4168,17 +3913,17 @@
         <v>106</v>
       </c>
       <c r="G4" t="s">
+        <v>382</v>
+      </c>
+      <c r="I4" t="s">
         <v>383</v>
       </c>
-      <c r="I4" t="s">
-        <v>384</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A5" s="13"/>
       <c r="C5" s="4"/>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A6" s="13" t="s">
         <v>15</v>
       </c>
@@ -4195,16 +3940,16 @@
         <v>106</v>
       </c>
       <c r="F6" t="s">
+        <v>379</v>
+      </c>
+      <c r="G6" t="s">
         <v>380</v>
       </c>
-      <c r="G6" t="s">
+      <c r="H6" t="s">
         <v>381</v>
       </c>
-      <c r="H6" t="s">
-        <v>382</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A7" s="13" t="s">
         <v>15</v>
       </c>
@@ -4221,17 +3966,17 @@
         <v>106</v>
       </c>
       <c r="G7" t="s">
+        <v>382</v>
+      </c>
+      <c r="I7" t="s">
         <v>383</v>
       </c>
-      <c r="I7" t="s">
-        <v>384</v>
-      </c>
-    </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A8" s="13"/>
       <c r="C8" s="4"/>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A9" s="13" t="s">
         <v>18</v>
       </c>
@@ -4248,16 +3993,16 @@
         <v>106</v>
       </c>
       <c r="F9" t="s">
+        <v>379</v>
+      </c>
+      <c r="G9" t="s">
         <v>380</v>
       </c>
-      <c r="G9" t="s">
+      <c r="H9" t="s">
         <v>381</v>
       </c>
-      <c r="H9" t="s">
-        <v>382</v>
-      </c>
-    </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A10" s="13" t="s">
         <v>18</v>
       </c>
@@ -4274,17 +4019,17 @@
         <v>106</v>
       </c>
       <c r="G10" t="s">
+        <v>382</v>
+      </c>
+      <c r="I10" t="s">
         <v>383</v>
       </c>
-      <c r="I10" t="s">
-        <v>384</v>
-      </c>
-    </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A11" s="13"/>
       <c r="C11" s="4"/>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A12" s="13" t="s">
         <v>22</v>
       </c>
@@ -4293,11 +4038,11 @@
       </c>
       <c r="C12" s="4"/>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A13" s="13"/>
       <c r="C13" s="4"/>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A14" s="13" t="s">
         <v>25</v>
       </c>
@@ -4306,7 +4051,7 @@
       </c>
       <c r="C14" s="4"/>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A15" s="13" t="s">
         <v>25</v>
       </c>
@@ -4315,11 +4060,11 @@
       </c>
       <c r="C15" s="4"/>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A16" s="13"/>
       <c r="C16" s="4"/>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A17" s="13" t="s">
         <v>28</v>
       </c>
@@ -4336,19 +4081,19 @@
         <v>106</v>
       </c>
       <c r="F17" t="s">
+        <v>379</v>
+      </c>
+      <c r="G17" t="s">
         <v>380</v>
       </c>
-      <c r="G17" t="s">
+      <c r="H17" t="s">
         <v>381</v>
       </c>
-      <c r="H17" t="s">
-        <v>382</v>
-      </c>
       <c r="K17" t="s">
-        <v>385</v>
-      </c>
-    </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
+        <v>384</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A18" s="13" t="s">
         <v>28</v>
       </c>
@@ -4365,17 +4110,17 @@
         <v>106</v>
       </c>
       <c r="G18" t="s">
+        <v>382</v>
+      </c>
+      <c r="I18" t="s">
         <v>383</v>
       </c>
-      <c r="I18" t="s">
-        <v>384</v>
-      </c>
-    </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A19" s="13"/>
       <c r="C19" s="4"/>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A20" s="13" t="s">
         <v>31</v>
       </c>
@@ -4387,10 +4132,10 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="B3:B20">
-    <cfRule type="cellIs" dxfId="34" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="14" priority="1" operator="equal">
       <formula>"Yes"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="33" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="13" priority="2" operator="equal">
       <formula>"No"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -4413,19 +4158,19 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:O31"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="11.42578125" customWidth="1"/>
-    <col min="2" max="2" width="14.140625" customWidth="1"/>
-    <col min="3" max="3" width="14.5703125" customWidth="1"/>
+    <col min="1" max="1" width="11.44140625" customWidth="1"/>
+    <col min="2" max="2" width="14.109375" customWidth="1"/>
+    <col min="3" max="3" width="14.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>175</v>
       </c>
     </row>
-    <row r="2" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>176</v>
       </c>
@@ -4466,13 +4211,13 @@
         <v>188</v>
       </c>
       <c r="N2" s="1" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="O2" s="1" t="s">
         <v>189</v>
       </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>190</v>
       </c>
@@ -4480,7 +4225,7 @@
         <v>55</v>
       </c>
       <c r="C3" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="D3" t="s">
         <v>191</v>
@@ -4507,7 +4252,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
       <c r="B4" t="s">
         <v>45</v>
       </c>
@@ -4539,7 +4284,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
       <c r="B5" t="s">
         <v>47</v>
       </c>
@@ -4571,7 +4316,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>197</v>
       </c>
@@ -4606,7 +4351,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>200</v>
       </c>
@@ -4614,7 +4359,7 @@
         <v>201</v>
       </c>
       <c r="C7" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="D7" t="s">
         <v>196</v>
@@ -4641,7 +4386,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>202</v>
       </c>
@@ -4676,7 +4421,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.3">
       <c r="B9" t="s">
         <v>206</v>
       </c>
@@ -4701,7 +4446,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.3">
       <c r="B10" t="s">
         <v>208</v>
       </c>
@@ -4726,7 +4471,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>209</v>
       </c>
@@ -4734,7 +4479,7 @@
         <v>52</v>
       </c>
       <c r="C11" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="D11" t="s">
         <v>196</v>
@@ -4761,7 +4506,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>210</v>
       </c>
@@ -4769,7 +4514,7 @@
         <v>53</v>
       </c>
       <c r="C12" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="D12" t="s">
         <v>196</v>
@@ -4796,7 +4541,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>213</v>
       </c>
@@ -4804,7 +4549,7 @@
         <v>54</v>
       </c>
       <c r="C13" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="D13" t="s">
         <v>196</v>
@@ -4831,7 +4576,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>77</v>
       </c>
@@ -4866,7 +4611,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>215</v>
       </c>
@@ -4901,7 +4646,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>218</v>
       </c>
@@ -4936,7 +4681,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>221</v>
       </c>
@@ -4971,7 +4716,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>224</v>
       </c>
@@ -4979,7 +4724,7 @@
         <v>46</v>
       </c>
       <c r="C18" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="D18" t="s">
         <v>196</v>
@@ -5006,7 +4751,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>225</v>
       </c>
@@ -5014,7 +4759,7 @@
         <v>226</v>
       </c>
       <c r="C19" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="D19" t="s">
         <v>196</v>
@@ -5041,7 +4786,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>227</v>
       </c>
@@ -5076,7 +4821,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>229</v>
       </c>
@@ -5114,7 +4859,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>234</v>
       </c>
@@ -5122,7 +4867,7 @@
         <v>235</v>
       </c>
       <c r="C22" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="D22" t="s">
         <v>196</v>
@@ -5143,7 +4888,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>236</v>
       </c>
@@ -5151,7 +4896,7 @@
         <v>237</v>
       </c>
       <c r="C23" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="D23" t="s">
         <v>231</v>
@@ -5178,7 +4923,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>240</v>
       </c>
@@ -5209,7 +4954,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>243</v>
       </c>
@@ -5244,7 +4989,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:13" x14ac:dyDescent="0.3">
       <c r="B26" t="s">
         <v>57</v>
       </c>
@@ -5264,9 +5009,9 @@
         <v>220</v>
       </c>
     </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:13" x14ac:dyDescent="0.3">
       <c r="B27" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="C27" t="s">
         <v>1</v>
@@ -5290,7 +5035,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:13" x14ac:dyDescent="0.3">
       <c r="B28" t="s">
         <v>245</v>
       </c>
@@ -5316,7 +5061,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>246</v>
       </c>
@@ -5345,7 +5090,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>248</v>
       </c>
@@ -5374,12 +5119,12 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:13" x14ac:dyDescent="0.3">
       <c r="B31" t="s">
         <v>250</v>
       </c>
       <c r="C31" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="D31" t="s">
         <v>196</v>
@@ -5414,13 +5159,13 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:M17"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
-    <col min="6" max="6" width="15.5703125" customWidth="1"/>
+    <col min="6" max="6" width="15.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A1" s="2"/>
       <c r="B1" s="2" t="s">
         <v>112</v>
@@ -5437,7 +5182,7 @@
       <c r="I1" s="2"/>
       <c r="K1" s="2"/>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>115</v>
       </c>
@@ -5478,7 +5223,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>125</v>
       </c>
@@ -5504,7 +5249,7 @@
         <v>-18877.708702820371</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>131</v>
       </c>
@@ -5530,7 +5275,7 @@
         <v>-19045.139985898601</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>133</v>
       </c>
@@ -5556,7 +5301,7 @@
         <v>-5.4445188599886638</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>135</v>
       </c>
@@ -5582,7 +5327,7 @@
         <v>2.671411511624413</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>137</v>
       </c>
@@ -5608,7 +5353,7 @@
         <v>9.5532474786010475</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>125</v>
       </c>
@@ -5634,7 +5379,7 @@
         <v>2866.0938229725748</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>131</v>
       </c>
@@ -5660,7 +5405,7 @@
         <v>1490.761502865475</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>133</v>
       </c>
@@ -5686,7 +5431,7 @@
         <v>2.217459469264154</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>135</v>
       </c>
@@ -5712,7 +5457,7 @@
         <v>0.2337935274525294</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>137</v>
       </c>
@@ -5738,7 +5483,7 @@
         <v>2.0873115011979051E-2</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>125</v>
       </c>
@@ -5764,7 +5509,7 @@
         <v>1351.711647219304</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>131</v>
       </c>
@@ -5790,7 +5535,7 @@
         <v>150.9391394665019</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>133</v>
       </c>
@@ -5816,7 +5561,7 @@
         <v>1.940117188288828</v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>135</v>
       </c>
@@ -5842,7 +5587,7 @@
         <v>-2.0146865510893688E-2</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>137</v>
       </c>
@@ -5876,22 +5621,22 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:G42"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="3" max="3" width="16.7109375" customWidth="1"/>
+    <col min="3" max="3" width="16.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>153</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="5" spans="1:7" s="1" customFormat="1" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" s="1" customFormat="1" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>2</v>
       </c>
@@ -5914,7 +5659,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B6" t="s">
         <v>12</v>
       </c>
@@ -5934,7 +5679,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="7" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="B7" t="s">
         <v>12</v>
       </c>
@@ -5951,7 +5696,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="8" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="B8" t="s">
         <v>12</v>
       </c>
@@ -5968,7 +5713,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="9" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="B9" t="s">
         <v>12</v>
       </c>
@@ -5985,7 +5730,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="10" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="B10" t="s">
         <v>12</v>
       </c>
@@ -6002,7 +5747,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="11" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="B11" t="s">
         <v>12</v>
       </c>
@@ -6019,7 +5764,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B12" t="s">
         <v>12</v>
       </c>
@@ -6036,7 +5781,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B13" t="s">
         <v>15</v>
       </c>
@@ -6053,7 +5798,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="14" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="B14" t="s">
         <v>15</v>
       </c>
@@ -6070,7 +5815,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="15" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="B15" t="s">
         <v>15</v>
       </c>
@@ -6087,7 +5832,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="16" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="B16" t="s">
         <v>15</v>
       </c>
@@ -6104,7 +5849,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="17" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B17" t="s">
         <v>15</v>
       </c>
@@ -6121,7 +5866,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="18" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B18" t="s">
         <v>15</v>
       </c>
@@ -6138,7 +5883,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="19" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B19" t="s">
         <v>15</v>
       </c>
@@ -6155,7 +5900,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="20" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B20" t="s">
         <v>18</v>
       </c>
@@ -6172,7 +5917,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="21" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B21" t="s">
         <v>18</v>
       </c>
@@ -6189,7 +5934,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="22" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B22" t="s">
         <v>18</v>
       </c>
@@ -6206,7 +5951,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="23" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B23" t="s">
         <v>18</v>
       </c>
@@ -6223,7 +5968,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="24" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B24" t="s">
         <v>18</v>
       </c>
@@ -6240,7 +5985,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="25" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B25" t="s">
         <v>18</v>
       </c>
@@ -6257,7 +6002,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="26" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B26" t="s">
         <v>18</v>
       </c>
@@ -6274,7 +6019,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="27" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B27" t="s">
         <v>28</v>
       </c>
@@ -6291,7 +6036,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="28" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B28" t="s">
         <v>28</v>
       </c>
@@ -6308,7 +6053,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="29" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B29" t="s">
         <v>28</v>
       </c>
@@ -6325,7 +6070,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="30" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B30" t="s">
         <v>28</v>
       </c>
@@ -6342,7 +6087,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="31" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B31" t="s">
         <v>28</v>
       </c>
@@ -6359,7 +6104,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="32" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B32" t="s">
         <v>28</v>
       </c>
@@ -6376,7 +6121,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="33" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B33" t="s">
         <v>28</v>
       </c>
@@ -6393,7 +6138,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="34" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B34" t="s">
         <v>31</v>
       </c>
@@ -6410,7 +6155,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="35" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B35" t="s">
         <v>31</v>
       </c>
@@ -6427,7 +6172,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="36" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B36" t="s">
         <v>31</v>
       </c>
@@ -6444,7 +6189,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="37" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B37" t="s">
         <v>31</v>
       </c>
@@ -6461,7 +6206,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="38" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B38" t="s">
         <v>31</v>
       </c>
@@ -6478,7 +6223,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="39" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B39" t="s">
         <v>31</v>
       </c>
@@ -6495,7 +6240,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="40" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B40" t="s">
         <v>31</v>
       </c>
@@ -6512,7 +6257,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="41" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="41" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B41" t="s">
         <v>31</v>
       </c>
@@ -6529,7 +6274,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="42" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="42" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B42" t="s">
         <v>31</v>
       </c>
@@ -6563,19 +6308,19 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9DE0C751-ACC1-462A-82AF-4CE9BB91C06B}">
   <dimension ref="A2:G21"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="C4" t="s">
-        <v>390</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>2</v>
       </c>
@@ -6583,10 +6328,10 @@
         <v>255</v>
       </c>
       <c r="C5" s="12" t="s">
+        <v>387</v>
+      </c>
+      <c r="D5" s="1" t="s">
         <v>388</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>389</v>
       </c>
       <c r="E5" s="1" t="s">
         <v>157</v>
@@ -6598,7 +6343,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>21</v>
       </c>
@@ -6612,7 +6357,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>11</v>
       </c>
@@ -6626,7 +6371,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>11</v>
       </c>
@@ -6640,7 +6385,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>11</v>
       </c>
@@ -6654,7 +6399,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>11</v>
       </c>
@@ -6668,7 +6413,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>11</v>
       </c>
@@ -6682,7 +6427,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>21</v>
       </c>
@@ -6696,7 +6441,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>11</v>
       </c>
@@ -6710,7 +6455,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>11</v>
       </c>
@@ -6724,7 +6469,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>11</v>
       </c>
@@ -6738,7 +6483,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>11</v>
       </c>
@@ -6752,7 +6497,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>11</v>
       </c>
@@ -6766,7 +6511,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>11</v>
       </c>
@@ -6780,7 +6525,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>11</v>
       </c>
@@ -6794,7 +6539,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>11</v>
       </c>
@@ -6808,7 +6553,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>11</v>
       </c>
@@ -6824,10 +6569,10 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A6:A22">
-    <cfRule type="cellIs" dxfId="32" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="12" priority="1" operator="equal">
       <formula>"Yes"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="31" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="11" priority="2" operator="equal">
       <formula>"No"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -6838,25 +6583,25 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:O8"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="8.5703125" customWidth="1"/>
+    <col min="1" max="1" width="8.5546875" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
-    <col min="3" max="3" width="12.85546875" customWidth="1"/>
+    <col min="3" max="3" width="12.88671875" customWidth="1"/>
     <col min="4" max="4" width="10" customWidth="1"/>
-    <col min="6" max="6" width="6.7109375" customWidth="1"/>
-    <col min="7" max="7" width="6.5703125" customWidth="1"/>
-    <col min="8" max="8" width="8.28515625" customWidth="1"/>
-    <col min="9" max="9" width="5.5703125" customWidth="1"/>
-    <col min="10" max="10" width="6.5703125" customWidth="1"/>
-    <col min="11" max="11" width="6.140625" customWidth="1"/>
-    <col min="12" max="12" width="5.140625" customWidth="1"/>
-    <col min="13" max="13" width="5.5703125" customWidth="1"/>
-    <col min="14" max="14" width="5.140625" customWidth="1"/>
-    <col min="15" max="15" width="4.42578125" customWidth="1"/>
+    <col min="6" max="6" width="6.6640625" customWidth="1"/>
+    <col min="7" max="7" width="6.5546875" customWidth="1"/>
+    <col min="8" max="8" width="8.33203125" customWidth="1"/>
+    <col min="9" max="9" width="5.5546875" customWidth="1"/>
+    <col min="10" max="10" width="6.5546875" customWidth="1"/>
+    <col min="11" max="11" width="6.109375" customWidth="1"/>
+    <col min="12" max="12" width="5.109375" customWidth="1"/>
+    <col min="13" max="13" width="5.5546875" customWidth="1"/>
+    <col min="14" max="14" width="5.109375" customWidth="1"/>
+    <col min="15" max="15" width="4.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>253</v>
       </c>
@@ -6864,7 +6609,7 @@
         <v>254</v>
       </c>
     </row>
-    <row r="2" spans="1:15" s="8" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:15" s="8" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="8" t="s">
         <v>255</v>
       </c>
@@ -6911,7 +6656,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>270</v>
       </c>
@@ -6951,7 +6696,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>273</v>
       </c>
@@ -6966,9 +6711,9 @@
         <v>274</v>
       </c>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="B5" s="3"/>
       <c r="C5" s="3"/>
@@ -7006,21 +6751,21 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
       <c r="B7" s="3"/>
       <c r="C7" s="3"/>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.3">
       <c r="B8" s="3"/>
       <c r="C8" s="3"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="A3:A28">
-    <cfRule type="duplicateValues" dxfId="30" priority="6"/>
+    <cfRule type="duplicateValues" dxfId="10" priority="6"/>
   </conditionalFormatting>
   <dataValidations count="1">
     <dataValidation showInputMessage="1" showErrorMessage="1" prompt="No duplicate names please" sqref="A3:A38" xr:uid="{00000000-0002-0000-0700-000000000000}"/>
@@ -7033,21 +6778,24 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
   <dimension ref="A1:H21"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="4" width="10.28515625" customWidth="1"/>
-    <col min="5" max="6" width="8.5703125" customWidth="1"/>
+    <col min="2" max="4" width="10.33203125" customWidth="1"/>
+    <col min="5" max="6" width="8.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
       <c r="G1" s="7" t="s">
         <v>275</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" s="8" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="H1" s="2" t="s">
+        <v>396</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" s="8" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
@@ -7073,7 +6821,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="31" t="s">
         <v>21</v>
       </c>
@@ -7087,8 +6835,9 @@
         <v>273</v>
       </c>
       <c r="G3" s="32"/>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="H3" s="32"/>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>21</v>
       </c>
@@ -7114,7 +6863,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>21</v>
       </c>
@@ -7140,7 +6889,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" s="31" t="s">
         <v>21</v>
       </c>
@@ -7162,11 +6911,11 @@
       <c r="G6" s="31">
         <v>1</v>
       </c>
-      <c r="H6" t="s">
+      <c r="H6" s="31" t="s">
         <v>344</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>11</v>
       </c>
@@ -7189,10 +6938,10 @@
         <v>283</v>
       </c>
       <c r="H7" t="s">
-        <v>345</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>11</v>
       </c>
@@ -7206,7 +6955,7 @@
         <v>162</v>
       </c>
       <c r="E8" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="F8" t="s">
         <v>273</v>
@@ -7215,10 +6964,10 @@
         <v>0.2</v>
       </c>
       <c r="H8" t="s">
-        <v>345</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A9" s="31" t="s">
         <v>11</v>
       </c>
@@ -7240,11 +6989,11 @@
       <c r="G9" s="31">
         <v>1</v>
       </c>
-      <c r="H9" t="s">
-        <v>345</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="H9" s="31" t="s">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>11</v>
       </c>
@@ -7258,7 +7007,7 @@
         <v>161</v>
       </c>
       <c r="E10" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="F10" t="s">
         <v>282</v>
@@ -7266,8 +7015,11 @@
       <c r="G10">
         <v>0.9</v>
       </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="H10" s="37" t="s">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>11</v>
       </c>
@@ -7289,8 +7041,11 @@
       <c r="G11" t="s">
         <v>283</v>
       </c>
-    </row>
-    <row r="12" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="H11" s="37" t="s">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A12" s="31" t="s">
         <v>11</v>
       </c>
@@ -7312,8 +7067,11 @@
       <c r="G12" s="31">
         <v>1</v>
       </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="H12" s="31" t="s">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>11</v>
       </c>
@@ -7335,8 +7093,11 @@
       <c r="G13" t="s">
         <v>283</v>
       </c>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="H13" s="37" t="s">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>11</v>
       </c>
@@ -7358,8 +7119,11 @@
       <c r="G14" t="s">
         <v>87</v>
       </c>
-    </row>
-    <row r="15" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="H14" s="37" t="s">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A15" s="31" t="s">
         <v>11</v>
       </c>
@@ -7381,31 +7145,34 @@
       <c r="G15" s="31">
         <v>1</v>
       </c>
-    </row>
-    <row r="21" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H15" s="31" t="s">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="21" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H21" t="s">
         <v>285</v>
       </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="A3:A32">
-    <cfRule type="cellIs" dxfId="29" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="9" priority="1" operator="equal">
       <formula>"Yes"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="28" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="8" priority="2" operator="equal">
       <formula>"No"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B3:D15">
-    <cfRule type="cellIs" dxfId="27" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="7" priority="3" operator="equal">
       <formula>"Initial"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B3:D17">
-    <cfRule type="cellIs" dxfId="26" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="6" priority="4" operator="equal">
       <formula>"Inital"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="25" priority="5" operator="equal">
+    <cfRule type="cellIs" dxfId="5" priority="5" operator="equal">
       <formula>"Final"</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
Added InterpolatedFluid() to fluids_and_minerals.py which takes a table of pressure, density and bulk modulus as input. It can then calculate the fluid properties at ~any pressure. This is useful for gas condensate which can't be modelled with accuracy using Batlze & Wang. Also updated the project_table_new.xlsx accordingly
</commit_message>
<xml_diff>
--- a/excels/project_table_new.xlsx
+++ b/excels/project_table_new.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="T:\Python\EMB\blixt_rp\excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B6006E1-5DAD-41D2-BF7E-CFB3416A2ED4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E934167C-C9C6-4E9B-BE94-D64AC4210161}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" tabRatio="685" firstSheet="5" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" tabRatio="685" firstSheet="5" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Well settings" sheetId="1" r:id="rId1"/>
@@ -31,8 +31,9 @@
   <definedNames>
     <definedName name="AvoClasses">Utils!$Q$3:$Q$7</definedName>
     <definedName name="CheckshotFormat">Utils!$M$3:$M$4</definedName>
+    <definedName name="FluidCalculations">Utils!$B$3:$B$5</definedName>
     <definedName name="FluidNames">Fluids!$A$3:$A$8</definedName>
-    <definedName name="FluidTypes">Utils!$E$3:$E$6</definedName>
+    <definedName name="FluidTypes">Utils!$E$3:$E$7</definedName>
     <definedName name="IntervalNames">Utils!$H$3:$H$18</definedName>
     <definedName name="LineStyles">Utils!$G$3:$G$6</definedName>
     <definedName name="LogTypes">Templates!$B$3:$B48</definedName>
@@ -64,7 +65,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1055" uniqueCount="398">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1082" uniqueCount="402">
   <si>
     <t>Select Yes or No</t>
   </si>
@@ -829,9 +830,6 @@
   </si>
   <si>
     <t>No duplicates please</t>
-  </si>
-  <si>
-    <t>Batzle and Wang' or 'User specified'</t>
   </si>
   <si>
     <t>Name</t>
@@ -1267,6 +1265,21 @@
   </si>
   <si>
     <t>MyTag</t>
+  </si>
+  <si>
+    <t>Gas condensate</t>
+  </si>
+  <si>
+    <t>Interpolation</t>
+  </si>
+  <si>
+    <t>Cond</t>
+  </si>
+  <si>
+    <t>FromTable</t>
+  </si>
+  <si>
+    <t>Batzle and Wang' or 'User specified' or "Interpolation"</t>
   </si>
 </sst>
 </file>
@@ -1478,7 +1491,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1530,7 +1543,6 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2172,7 +2184,7 @@
         <v>21</v>
       </c>
       <c r="B10" s="13" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="C10" s="20" t="s">
         <v>23</v>
@@ -2229,38 +2241,38 @@
   <sheetData>
     <row r="1" spans="1:7" ht="26.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="F1" s="7" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
     </row>
     <row r="2" spans="1:7" s="8" customFormat="1" ht="30.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="33" t="s">
+        <v>254</v>
+      </c>
+      <c r="B2" s="34" t="s">
         <v>255</v>
       </c>
-      <c r="B2" s="34" t="s">
+      <c r="C2" s="34" t="s">
         <v>256</v>
       </c>
-      <c r="C2" s="34" t="s">
+      <c r="D2" s="34" t="s">
         <v>257</v>
       </c>
-      <c r="D2" s="34" t="s">
+      <c r="E2" s="33" t="s">
+        <v>286</v>
+      </c>
+      <c r="F2" s="33" t="s">
         <v>258</v>
       </c>
-      <c r="E2" s="33" t="s">
+      <c r="G2" s="33" t="s">
         <v>287</v>
-      </c>
-      <c r="F2" s="33" t="s">
-        <v>259</v>
-      </c>
-      <c r="G2" s="33" t="s">
-        <v>288</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="B3">
         <v>36.6</v>
@@ -2277,7 +2289,7 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="B4">
         <v>11.4</v>
@@ -2292,15 +2304,15 @@
         <v>0</v>
       </c>
       <c r="F4" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="G4" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B5">
         <v>76.8</v>
@@ -2317,7 +2329,7 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="B6">
         <v>94.9</v>
@@ -2334,7 +2346,7 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="B7">
         <v>26</v>
@@ -2351,7 +2363,7 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="B8">
         <v>47</v>
@@ -2368,7 +2380,7 @@
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="B9">
         <v>114</v>
@@ -2385,7 +2397,7 @@
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="B10">
         <v>55</v>
@@ -2402,7 +2414,7 @@
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="B11">
         <v>48</v>
@@ -2419,7 +2431,7 @@
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="B12">
         <v>85</v>
@@ -2436,7 +2448,7 @@
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="B13">
         <v>52</v>
@@ -2453,7 +2465,7 @@
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="B14">
         <v>50</v>
@@ -2470,7 +2482,7 @@
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="B15">
         <v>25.2</v>
@@ -2487,7 +2499,7 @@
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="B16">
         <v>66.5</v>
@@ -2504,7 +2516,7 @@
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="B17">
         <v>58</v>
@@ -2521,7 +2533,7 @@
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="B18">
         <v>158</v>
@@ -2538,7 +2550,7 @@
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="B19">
         <v>27</v>
@@ -2555,7 +2567,7 @@
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="B20">
         <v>123.7</v>
@@ -2572,7 +2584,7 @@
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="B21">
         <v>15</v>
@@ -2589,7 +2601,7 @@
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="B22">
         <v>17.96</v>
@@ -2606,7 +2618,7 @@
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="B23">
         <v>55.8</v>
@@ -2623,7 +2635,7 @@
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="B24">
         <v>87</v>
@@ -2640,7 +2652,7 @@
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="B25">
         <v>103.67</v>
@@ -2657,7 +2669,7 @@
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="B26">
         <v>129.13999999999999</v>
@@ -2674,7 +2686,7 @@
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="B27">
         <v>4.5199999999999996</v>
@@ -2691,7 +2703,7 @@
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="B28">
         <v>160.29</v>
@@ -2708,7 +2720,7 @@
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="B29">
         <v>62.2</v>
@@ -2725,7 +2737,7 @@
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="B30">
         <v>146.25</v>
@@ -2742,7 +2754,7 @@
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="B31">
         <v>48.35</v>
@@ -2759,7 +2771,7 @@
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="B32">
         <v>2.9</v>
@@ -2776,7 +2788,7 @@
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="B33">
         <v>12.3</v>
@@ -2812,7 +2824,7 @@
         <v>0</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
     </row>
     <row r="2" spans="1:5" s="8" customFormat="1" ht="30.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -2820,16 +2832,16 @@
         <v>2</v>
       </c>
       <c r="B2" s="9" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="C2" s="9" t="s">
         <v>116</v>
       </c>
       <c r="D2" s="8" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="E2" s="10" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -2843,10 +2855,10 @@
         <v>162</v>
       </c>
       <c r="D3" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -2860,7 +2872,7 @@
         <v>162</v>
       </c>
       <c r="D4" s="31" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="E4" s="31" t="s">
         <v>64</v>
@@ -2877,10 +2889,10 @@
         <v>161</v>
       </c>
       <c r="D5" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -2894,7 +2906,7 @@
         <v>161</v>
       </c>
       <c r="D6" s="31" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="E6" s="31" t="s">
         <v>64</v>
@@ -2911,10 +2923,10 @@
         <v>163</v>
       </c>
       <c r="D7" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -2928,7 +2940,7 @@
         <v>163</v>
       </c>
       <c r="D8" s="31" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="E8" s="31" t="s">
         <v>64</v>
@@ -2989,49 +3001,49 @@
       <c r="J1" s="2"/>
       <c r="K1" s="2"/>
       <c r="L1" s="2" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="M1" s="2" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="O1" s="2"/>
     </row>
     <row r="2" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>358</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>365</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>366</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>367</v>
+      </c>
+      <c r="F2" s="1" t="s">
         <v>359</v>
       </c>
-      <c r="C2" s="1" t="s">
-        <v>366</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>367</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>368</v>
-      </c>
-      <c r="F2" s="1" t="s">
+      <c r="G2" s="1" t="s">
         <v>360</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="H2" s="1" t="s">
         <v>361</v>
-      </c>
-      <c r="H2" s="1" t="s">
-        <v>362</v>
       </c>
       <c r="I2" s="1" t="s">
         <v>157</v>
       </c>
       <c r="J2" s="1" t="s">
+        <v>362</v>
+      </c>
+      <c r="K2" s="1" t="s">
         <v>363</v>
       </c>
-      <c r="K2" s="1" t="s">
+      <c r="L2" s="1" t="s">
         <v>364</v>
-      </c>
-      <c r="L2" s="1" t="s">
-        <v>365</v>
       </c>
       <c r="M2" s="1" t="s">
         <v>8</v>
@@ -3054,7 +3066,7 @@
     <row r="1" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A1" s="2"/>
       <c r="B1" s="2" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="C1" s="2"/>
       <c r="D1" s="2"/>
@@ -3066,22 +3078,22 @@
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>99</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="D2" s="1" t="s">
+        <v>371</v>
+      </c>
+      <c r="E2" s="1" t="s">
         <v>372</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="F2" s="1" t="s">
         <v>373</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>374</v>
       </c>
       <c r="G2" s="1"/>
       <c r="H2" s="1"/>
@@ -3119,57 +3131,57 @@
   <sheetData>
     <row r="1" spans="1:17" x14ac:dyDescent="0.3">
       <c r="H1" s="2" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
     </row>
     <row r="2" spans="1:17" s="6" customFormat="1" ht="42.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B2" s="6" t="s">
+        <v>322</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>267</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>275</v>
+      </c>
+      <c r="E2" t="s">
         <v>323</v>
       </c>
-      <c r="C2" s="6" t="s">
-        <v>268</v>
-      </c>
-      <c r="D2" s="6" t="s">
-        <v>276</v>
-      </c>
-      <c r="E2" t="s">
+      <c r="F2" s="6" t="s">
         <v>324</v>
       </c>
-      <c r="F2" s="6" t="s">
+      <c r="G2" s="6" t="s">
         <v>325</v>
-      </c>
-      <c r="G2" s="6" t="s">
-        <v>326</v>
       </c>
       <c r="H2" s="1" t="s">
         <v>116</v>
       </c>
       <c r="I2" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="J2" s="6" t="s">
+        <v>326</v>
+      </c>
+      <c r="K2" t="s">
         <v>327</v>
       </c>
-      <c r="K2" t="s">
+      <c r="L2" t="s">
         <v>328</v>
       </c>
-      <c r="L2" t="s">
+      <c r="M2" t="s">
         <v>329</v>
       </c>
-      <c r="M2" t="s">
+      <c r="N2" t="s">
         <v>330</v>
-      </c>
-      <c r="N2" t="s">
-        <v>331</v>
       </c>
       <c r="O2" t="s">
         <v>102</v>
       </c>
       <c r="P2" t="s">
+        <v>344</v>
+      </c>
+      <c r="Q2" t="s">
         <v>345</v>
-      </c>
-      <c r="Q2" t="s">
-        <v>346</v>
       </c>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.3">
@@ -3177,16 +3189,16 @@
         <v>11</v>
       </c>
       <c r="B3" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="C3" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="D3" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="E3" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="F3" t="s">
         <v>14</v>
@@ -3202,16 +3214,16 @@
         <v>4</v>
       </c>
       <c r="J3" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="K3" t="s">
+        <v>332</v>
+      </c>
+      <c r="L3" t="s">
         <v>333</v>
       </c>
-      <c r="L3" t="s">
+      <c r="M3" t="s">
         <v>334</v>
-      </c>
-      <c r="M3" t="s">
-        <v>335</v>
       </c>
       <c r="N3" t="s">
         <v>128</v>
@@ -3220,10 +3232,10 @@
         <v>106</v>
       </c>
       <c r="P3" t="s">
+        <v>346</v>
+      </c>
+      <c r="Q3" t="s">
         <v>347</v>
-      </c>
-      <c r="Q3" t="s">
-        <v>348</v>
       </c>
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.3">
@@ -3231,16 +3243,16 @@
         <v>21</v>
       </c>
       <c r="B4" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="C4" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="D4" t="s">
+        <v>280</v>
+      </c>
+      <c r="E4" t="s">
         <v>281</v>
-      </c>
-      <c r="E4" t="s">
-        <v>282</v>
       </c>
       <c r="F4" t="s">
         <v>17</v>
@@ -3256,36 +3268,39 @@
         <v>4</v>
       </c>
       <c r="J4" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="K4" t="s">
         <v>103</v>
       </c>
       <c r="L4" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="M4" t="s">
         <v>105</v>
       </c>
       <c r="O4" t="s">
+        <v>348</v>
+      </c>
+      <c r="P4" t="s">
         <v>349</v>
       </c>
-      <c r="P4" t="s">
+      <c r="Q4" t="s">
         <v>350</v>
       </c>
-      <c r="Q4" t="s">
-        <v>351</v>
-      </c>
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="B5" t="s">
+        <v>398</v>
+      </c>
       <c r="E5" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="F5" t="s">
         <v>20</v>
       </c>
       <c r="G5" s="13" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="H5" t="s">
         <v>161</v>
@@ -3298,21 +3313,21 @@
         <v>105</v>
       </c>
       <c r="O5" t="s">
+        <v>351</v>
+      </c>
+      <c r="Q5" t="s">
         <v>352</v>
-      </c>
-      <c r="Q5" t="s">
-        <v>353</v>
       </c>
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.3">
       <c r="E6" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="F6" t="s">
         <v>27</v>
       </c>
       <c r="G6" s="13" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="H6" t="s">
         <v>162</v>
@@ -3322,13 +3337,16 @@
         <v>4</v>
       </c>
       <c r="O6" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="Q6" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
     </row>
     <row r="7" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="E7" t="s">
+        <v>397</v>
+      </c>
       <c r="F7" t="s">
         <v>30</v>
       </c>
@@ -3340,10 +3358,10 @@
         <v>4</v>
       </c>
       <c r="O7" t="s">
+        <v>354</v>
+      </c>
+      <c r="Q7" t="s">
         <v>355</v>
-      </c>
-      <c r="Q7" t="s">
-        <v>356</v>
       </c>
     </row>
     <row r="8" spans="1:17" x14ac:dyDescent="0.3">
@@ -3408,7 +3426,7 @@
     </row>
     <row r="13" spans="1:17" x14ac:dyDescent="0.3">
       <c r="F13" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="H13" s="30" t="s">
         <v>169</v>
@@ -3420,7 +3438,7 @@
     </row>
     <row r="14" spans="1:17" x14ac:dyDescent="0.3">
       <c r="F14" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="H14" s="30" t="s">
         <v>170</v>
@@ -3444,7 +3462,7 @@
     </row>
     <row r="16" spans="1:17" x14ac:dyDescent="0.3">
       <c r="F16" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="H16" s="30" t="s">
         <v>172</v>
@@ -3830,7 +3848,7 @@
         <v>98</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
     </row>
     <row r="2" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
@@ -3853,7 +3871,7 @@
         <v>245</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="H2" s="1" t="s">
         <v>241</v>
@@ -3887,13 +3905,13 @@
         <v>106</v>
       </c>
       <c r="F3" t="s">
+        <v>378</v>
+      </c>
+      <c r="G3" t="s">
         <v>379</v>
       </c>
-      <c r="G3" t="s">
+      <c r="H3" t="s">
         <v>380</v>
-      </c>
-      <c r="H3" t="s">
-        <v>381</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.3">
@@ -3913,10 +3931,10 @@
         <v>106</v>
       </c>
       <c r="G4" t="s">
+        <v>381</v>
+      </c>
+      <c r="I4" t="s">
         <v>382</v>
-      </c>
-      <c r="I4" t="s">
-        <v>383</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.3">
@@ -3940,13 +3958,13 @@
         <v>106</v>
       </c>
       <c r="F6" t="s">
+        <v>378</v>
+      </c>
+      <c r="G6" t="s">
         <v>379</v>
       </c>
-      <c r="G6" t="s">
+      <c r="H6" t="s">
         <v>380</v>
-      </c>
-      <c r="H6" t="s">
-        <v>381</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.3">
@@ -3966,10 +3984,10 @@
         <v>106</v>
       </c>
       <c r="G7" t="s">
+        <v>381</v>
+      </c>
+      <c r="I7" t="s">
         <v>382</v>
-      </c>
-      <c r="I7" t="s">
-        <v>383</v>
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.3">
@@ -3993,13 +4011,13 @@
         <v>106</v>
       </c>
       <c r="F9" t="s">
+        <v>378</v>
+      </c>
+      <c r="G9" t="s">
         <v>379</v>
       </c>
-      <c r="G9" t="s">
+      <c r="H9" t="s">
         <v>380</v>
-      </c>
-      <c r="H9" t="s">
-        <v>381</v>
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.3">
@@ -4019,10 +4037,10 @@
         <v>106</v>
       </c>
       <c r="G10" t="s">
+        <v>381</v>
+      </c>
+      <c r="I10" t="s">
         <v>382</v>
-      </c>
-      <c r="I10" t="s">
-        <v>383</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.3">
@@ -4081,16 +4099,16 @@
         <v>106</v>
       </c>
       <c r="F17" t="s">
+        <v>378</v>
+      </c>
+      <c r="G17" t="s">
         <v>379</v>
       </c>
-      <c r="G17" t="s">
+      <c r="H17" t="s">
         <v>380</v>
       </c>
-      <c r="H17" t="s">
-        <v>381</v>
-      </c>
       <c r="K17" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.3">
@@ -4110,10 +4128,10 @@
         <v>106</v>
       </c>
       <c r="G18" t="s">
+        <v>381</v>
+      </c>
+      <c r="I18" t="s">
         <v>382</v>
-      </c>
-      <c r="I18" t="s">
-        <v>383</v>
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.3">
@@ -4211,7 +4229,7 @@
         <v>188</v>
       </c>
       <c r="N2" s="1" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="O2" s="1" t="s">
         <v>189</v>
@@ -4225,7 +4243,7 @@
         <v>55</v>
       </c>
       <c r="C3" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="D3" t="s">
         <v>191</v>
@@ -4359,7 +4377,7 @@
         <v>201</v>
       </c>
       <c r="C7" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="D7" t="s">
         <v>196</v>
@@ -4479,7 +4497,7 @@
         <v>52</v>
       </c>
       <c r="C11" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="D11" t="s">
         <v>196</v>
@@ -4514,7 +4532,7 @@
         <v>53</v>
       </c>
       <c r="C12" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="D12" t="s">
         <v>196</v>
@@ -4549,7 +4567,7 @@
         <v>54</v>
       </c>
       <c r="C13" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="D13" t="s">
         <v>196</v>
@@ -4724,7 +4742,7 @@
         <v>46</v>
       </c>
       <c r="C18" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="D18" t="s">
         <v>196</v>
@@ -4759,7 +4777,7 @@
         <v>226</v>
       </c>
       <c r="C19" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="D19" t="s">
         <v>196</v>
@@ -4867,7 +4885,7 @@
         <v>235</v>
       </c>
       <c r="C22" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="D22" t="s">
         <v>196</v>
@@ -4896,7 +4914,7 @@
         <v>237</v>
       </c>
       <c r="C23" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="D23" t="s">
         <v>231</v>
@@ -5011,7 +5029,7 @@
     </row>
     <row r="27" spans="1:13" x14ac:dyDescent="0.3">
       <c r="B27" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="C27" t="s">
         <v>1</v>
@@ -5124,7 +5142,7 @@
         <v>250</v>
       </c>
       <c r="C31" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="D31" t="s">
         <v>196</v>
@@ -6317,7 +6335,7 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="C4" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
@@ -6325,13 +6343,13 @@
         <v>2</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="C5" s="12" t="s">
+        <v>386</v>
+      </c>
+      <c r="D5" s="1" t="s">
         <v>387</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>388</v>
       </c>
       <c r="E5" s="1" t="s">
         <v>157</v>
@@ -6606,64 +6624,64 @@
         <v>253</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>254</v>
+        <v>401</v>
       </c>
     </row>
     <row r="2" spans="1:15" s="8" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="8" t="s">
+        <v>254</v>
+      </c>
+      <c r="B2" s="9" t="s">
         <v>255</v>
       </c>
-      <c r="B2" s="9" t="s">
+      <c r="C2" s="9" t="s">
         <v>256</v>
       </c>
-      <c r="C2" s="9" t="s">
+      <c r="D2" s="9" t="s">
         <v>257</v>
       </c>
-      <c r="D2" s="9" t="s">
+      <c r="E2" s="8" t="s">
         <v>258</v>
       </c>
-      <c r="E2" s="8" t="s">
+      <c r="F2" s="8" t="s">
         <v>259</v>
       </c>
-      <c r="F2" s="8" t="s">
+      <c r="G2" s="8" t="s">
         <v>260</v>
       </c>
-      <c r="G2" s="8" t="s">
+      <c r="H2" s="8" t="s">
         <v>261</v>
       </c>
-      <c r="H2" s="8" t="s">
+      <c r="I2" s="8" t="s">
         <v>262</v>
       </c>
-      <c r="I2" s="8" t="s">
+      <c r="J2" s="8" t="s">
         <v>263</v>
       </c>
-      <c r="J2" s="8" t="s">
+      <c r="K2" s="8" t="s">
         <v>264</v>
       </c>
-      <c r="K2" s="8" t="s">
+      <c r="L2" s="8" t="s">
         <v>265</v>
       </c>
-      <c r="L2" s="8" t="s">
+      <c r="M2" s="8" t="s">
         <v>266</v>
       </c>
-      <c r="M2" s="8" t="s">
+      <c r="N2" s="8" t="s">
         <v>267</v>
       </c>
-      <c r="N2" s="8" t="s">
+      <c r="O2" s="8" t="s">
         <v>268</v>
-      </c>
-      <c r="O2" s="8" t="s">
-        <v>269</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="B3" s="3"/>
       <c r="C3" s="3"/>
       <c r="E3" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="F3">
         <v>0.03</v>
@@ -6690,7 +6708,7 @@
         <v>0.6</v>
       </c>
       <c r="N3" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="O3">
         <v>2</v>
@@ -6698,7 +6716,7 @@
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="B4" s="3">
         <v>2.68</v>
@@ -6708,17 +6726,17 @@
         <v>1.0229999999999999</v>
       </c>
       <c r="E4" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="B5" s="3"/>
       <c r="C5" s="3"/>
       <c r="E5" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="F5">
         <v>0.03</v>
@@ -6745,15 +6763,27 @@
         <v>0.6</v>
       </c>
       <c r="N5" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="O5">
         <v>2</v>
       </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>400</v>
+      </c>
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
+      <c r="E6" t="s">
+        <v>398</v>
+      </c>
+      <c r="H6">
+        <v>1.0699999999999999E-2</v>
+      </c>
+      <c r="I6">
+        <v>0</v>
+      </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.3">
       <c r="B7" s="3"/>
@@ -6767,8 +6797,11 @@
   <conditionalFormatting sqref="A3:A28">
     <cfRule type="duplicateValues" dxfId="10" priority="6"/>
   </conditionalFormatting>
-  <dataValidations count="1">
+  <dataValidations count="2">
     <dataValidation showInputMessage="1" showErrorMessage="1" prompt="No duplicate names please" sqref="A3:A38" xr:uid="{00000000-0002-0000-0700-000000000000}"/>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E3:E21" xr:uid="{4B1D0C30-264B-4F6B-B5AB-7C993CE4CEF2}">
+      <formula1>FluidCalculations</formula1>
+    </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -6789,10 +6822,10 @@
         <v>0</v>
       </c>
       <c r="G1" s="7" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
     </row>
     <row r="2" spans="1:8" s="8" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -6800,25 +6833,25 @@
         <v>2</v>
       </c>
       <c r="B2" s="9" t="s">
+        <v>275</v>
+      </c>
+      <c r="C2" s="9" t="s">
         <v>276</v>
-      </c>
-      <c r="C2" s="9" t="s">
-        <v>277</v>
       </c>
       <c r="D2" s="9" t="s">
         <v>116</v>
       </c>
       <c r="E2" s="9" t="s">
+        <v>277</v>
+      </c>
+      <c r="F2" s="8" t="s">
         <v>278</v>
       </c>
-      <c r="F2" s="8" t="s">
+      <c r="G2" s="9" t="s">
         <v>279</v>
       </c>
-      <c r="G2" s="9" t="s">
-        <v>280</v>
-      </c>
       <c r="H2" s="8" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -6829,10 +6862,10 @@
       <c r="C3" s="31"/>
       <c r="D3" s="31"/>
       <c r="E3" s="31" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="F3" s="31" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="G3" s="32"/>
       <c r="H3" s="32"/>
@@ -6842,7 +6875,7 @@
         <v>21</v>
       </c>
       <c r="B4" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="C4" t="s">
         <v>28</v>
@@ -6851,16 +6884,16 @@
         <v>162</v>
       </c>
       <c r="E4" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="F4" t="s">
+        <v>281</v>
+      </c>
+      <c r="G4" t="s">
         <v>282</v>
       </c>
-      <c r="G4" t="s">
-        <v>283</v>
-      </c>
       <c r="H4" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
@@ -6868,7 +6901,7 @@
         <v>21</v>
       </c>
       <c r="B5" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="C5" t="s">
         <v>28</v>
@@ -6877,16 +6910,16 @@
         <v>162</v>
       </c>
       <c r="E5" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="F5" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="G5" t="s">
         <v>87</v>
       </c>
       <c r="H5" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -6894,7 +6927,7 @@
         <v>21</v>
       </c>
       <c r="B6" s="31" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="C6" s="31" t="s">
         <v>28</v>
@@ -6903,16 +6936,16 @@
         <v>162</v>
       </c>
       <c r="E6" s="31" t="s">
+        <v>272</v>
+      </c>
+      <c r="F6" s="31" t="s">
         <v>273</v>
-      </c>
-      <c r="F6" s="31" t="s">
-        <v>274</v>
       </c>
       <c r="G6" s="31">
         <v>1</v>
       </c>
       <c r="H6" s="31" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.3">
@@ -6920,7 +6953,7 @@
         <v>11</v>
       </c>
       <c r="B7" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="C7" t="s">
         <v>28</v>
@@ -6929,16 +6962,16 @@
         <v>162</v>
       </c>
       <c r="E7" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="F7" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="G7" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="H7" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
@@ -6946,7 +6979,7 @@
         <v>11</v>
       </c>
       <c r="B8" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="C8" t="s">
         <v>28</v>
@@ -6955,16 +6988,16 @@
         <v>162</v>
       </c>
       <c r="E8" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="F8" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="G8">
         <v>0.2</v>
       </c>
       <c r="H8" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -6972,7 +7005,7 @@
         <v>11</v>
       </c>
       <c r="B9" s="31" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="C9" s="31" t="s">
         <v>28</v>
@@ -6981,16 +7014,16 @@
         <v>162</v>
       </c>
       <c r="E9" s="31" t="s">
+        <v>272</v>
+      </c>
+      <c r="F9" s="31" t="s">
         <v>273</v>
-      </c>
-      <c r="F9" s="31" t="s">
-        <v>274</v>
       </c>
       <c r="G9" s="31">
         <v>1</v>
       </c>
       <c r="H9" s="31" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.3">
@@ -6998,7 +7031,7 @@
         <v>11</v>
       </c>
       <c r="B10" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="C10" t="s">
         <v>28</v>
@@ -7007,16 +7040,16 @@
         <v>161</v>
       </c>
       <c r="E10" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="F10" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="G10">
         <v>0.9</v>
       </c>
-      <c r="H10" s="37" t="s">
-        <v>397</v>
+      <c r="H10" t="s">
+        <v>396</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.3">
@@ -7024,7 +7057,7 @@
         <v>11</v>
       </c>
       <c r="B11" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="C11" t="s">
         <v>28</v>
@@ -7033,16 +7066,16 @@
         <v>161</v>
       </c>
       <c r="E11" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="F11" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="G11" t="s">
-        <v>283</v>
-      </c>
-      <c r="H11" s="37" t="s">
-        <v>397</v>
+        <v>282</v>
+      </c>
+      <c r="H11" t="s">
+        <v>396</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -7050,7 +7083,7 @@
         <v>11</v>
       </c>
       <c r="B12" s="31" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="C12" s="31" t="s">
         <v>28</v>
@@ -7059,16 +7092,16 @@
         <v>161</v>
       </c>
       <c r="E12" s="31" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="F12" s="31" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="G12" s="31">
         <v>1</v>
       </c>
       <c r="H12" s="31" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.3">
@@ -7076,7 +7109,7 @@
         <v>11</v>
       </c>
       <c r="B13" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="C13" t="s">
         <v>28</v>
@@ -7085,16 +7118,16 @@
         <v>163</v>
       </c>
       <c r="E13" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="F13" t="s">
+        <v>281</v>
+      </c>
+      <c r="G13" t="s">
         <v>282</v>
       </c>
-      <c r="G13" t="s">
-        <v>283</v>
-      </c>
-      <c r="H13" s="37" t="s">
-        <v>397</v>
+      <c r="H13" t="s">
+        <v>396</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.3">
@@ -7102,7 +7135,7 @@
         <v>11</v>
       </c>
       <c r="B14" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="C14" t="s">
         <v>28</v>
@@ -7111,16 +7144,16 @@
         <v>163</v>
       </c>
       <c r="E14" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="F14" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="G14" t="s">
         <v>87</v>
       </c>
-      <c r="H14" s="37" t="s">
-        <v>397</v>
+      <c r="H14" t="s">
+        <v>396</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -7128,7 +7161,7 @@
         <v>11</v>
       </c>
       <c r="B15" s="31" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="C15" s="31" t="s">
         <v>28</v>
@@ -7137,42 +7170,118 @@
         <v>163</v>
       </c>
       <c r="E15" s="31" t="s">
+        <v>272</v>
+      </c>
+      <c r="F15" s="31" t="s">
         <v>273</v>
-      </c>
-      <c r="F15" s="31" t="s">
-        <v>274</v>
       </c>
       <c r="G15" s="31">
         <v>1</v>
       </c>
       <c r="H15" s="31" t="s">
+        <v>396</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>11</v>
+      </c>
+      <c r="B16" t="s">
+        <v>280</v>
+      </c>
+      <c r="C16" t="s">
+        <v>28</v>
+      </c>
+      <c r="D16" t="s">
+        <v>163</v>
+      </c>
+      <c r="E16" t="s">
+        <v>400</v>
+      </c>
+      <c r="F16" t="s">
         <v>397</v>
       </c>
-    </row>
-    <row r="21" spans="8:8" x14ac:dyDescent="0.3">
+      <c r="G16" t="s">
+        <v>282</v>
+      </c>
+      <c r="H16" t="s">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>11</v>
+      </c>
+      <c r="B17" t="s">
+        <v>280</v>
+      </c>
+      <c r="C17" t="s">
+        <v>28</v>
+      </c>
+      <c r="D17" t="s">
+        <v>163</v>
+      </c>
+      <c r="E17" t="s">
+        <v>269</v>
+      </c>
+      <c r="F17" t="s">
+        <v>272</v>
+      </c>
+      <c r="G17" t="s">
+        <v>87</v>
+      </c>
+      <c r="H17" t="s">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A18" s="31" t="s">
+        <v>11</v>
+      </c>
+      <c r="B18" s="31" t="s">
+        <v>283</v>
+      </c>
+      <c r="C18" s="31" t="s">
+        <v>28</v>
+      </c>
+      <c r="D18" s="31" t="s">
+        <v>163</v>
+      </c>
+      <c r="E18" s="31" t="s">
+        <v>272</v>
+      </c>
+      <c r="F18" s="31" t="s">
+        <v>273</v>
+      </c>
+      <c r="G18" s="31">
+        <v>1</v>
+      </c>
+      <c r="H18" s="31" t="s">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
       <c r="H21" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="A3:A32">
-    <cfRule type="cellIs" dxfId="9" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="9" priority="2" operator="equal">
       <formula>"Yes"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="8" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="8" priority="3" operator="equal">
       <formula>"No"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B3:D15">
-    <cfRule type="cellIs" dxfId="7" priority="3" operator="equal">
+  <conditionalFormatting sqref="B3:D18">
+    <cfRule type="cellIs" dxfId="7" priority="1" operator="equal">
       <formula>"Initial"</formula>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B3:D17">
-    <cfRule type="cellIs" dxfId="6" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="6" priority="5" operator="equal">
       <formula>"Inital"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="5" priority="5" operator="equal">
+    <cfRule type="cellIs" dxfId="5" priority="6" operator="equal">
       <formula>"Final"</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>